<commit_message>
feat: add import-safe platform skeleton
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rb57cf468e0ec4cc5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R02805d08af864062"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="R314fe6b32b554eda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R77e4c98a30e34a85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R1cb2e02bcd1d4691"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R499f7aa0ac064586"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R96ccdb17184e44e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="Rc4b8b898c90b41f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="R6ed726de3302444b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="Rb170511ee24d4eca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R7348692c6cb345bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R7db169a4e555495c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -388,7 +388,7 @@
         <x:color rgb="FF9B2C2C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE2E1"/>
         </x:patternFill>
       </x:fill>
@@ -399,7 +399,7 @@
         <x:color rgb="FF176B4D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDFF3E8"/>
         </x:patternFill>
       </x:fill>
@@ -410,7 +410,7 @@
         <x:color rgb="FF7C5A00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF1C7"/>
         </x:patternFill>
       </x:fill>
@@ -421,7 +421,7 @@
         <x:color rgb="FF922B21"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFADBD8"/>
         </x:patternFill>
       </x:fill>
@@ -432,7 +432,7 @@
         <x:color rgb="FF922B21"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFADBD8"/>
         </x:patternFill>
       </x:fill>
@@ -443,7 +443,7 @@
         <x:color rgb="FF176B4D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDFF3E8"/>
         </x:patternFill>
       </x:fill>
@@ -820,7 +820,7 @@
       </x:c>
       <x:c r="B7" s="59" t="n">
         <x:f>COUNTIF('Backlog'!$F$5:$F$61,"Ready")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C7" s="51"/>
       <x:c r="D7" s="58" t="str">
@@ -1089,13 +1089,13 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="F6" s="24" t="str">
-        <x:v>Ready</x:v>
+        <x:v>Review</x:v>
       </x:c>
       <x:c r="G6" s="24" t="str">
         <x:v>Sprint 1</x:v>
       </x:c>
       <x:c r="H6" s="24" t="str">
-        <x:v>Next/MVP</x:v>
+        <x:v>In Review/MVP</x:v>
       </x:c>
       <x:c r="I6" s="65" t="n">
         <x:v>5</x:v>
@@ -3223,7 +3223,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d528b67680449d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbb7f6a2d09c4660"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3461,7 +3461,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f020ba228874f4f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3955fa81b6764d93"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3944,7 +3944,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0cf8e0fdd2124285"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R296102fe929b4307"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4107,7 +4107,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc197df636df40b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16292d9c9bdd4cc6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4279,7 +4279,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0f66d4e47f54428"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa485911b12f44e5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: prioritize mono i2s audio path
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R96ccdb17184e44e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="Rc4b8b898c90b41f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="R6ed726de3302444b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="Rb170511ee24d4eca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R7348692c6cb345bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R7db169a4e555495c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R2d35e002868d47cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="Rf34e61054ef14a33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Rc0f371a6e07943e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R1d263501791f479f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R7094a3da1d0c4ed6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rdcc1eca3050c46e3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21,7 +21,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="16">
+  <x:fonts count="18">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -110,8 +110,18 @@
       <x:color rgb="FF627D98"/>
       <x:name val="Aptos"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF1F2933"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF9B2C2C"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -141,6 +151,26 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF5F8FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFBFE3F2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE2E1"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFCE1D2"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -215,7 +245,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="67">
+  <x:cellXfs count="83">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -376,6 +406,36 @@
     </x:xf>
     <x:xf numFmtId="200" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="16" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="16" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="16" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -453,8 +513,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BacklogTable" displayName="BacklogTable" ref="A4:L61" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:L61"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BacklogTable" displayName="BacklogTable" ref="A4:L63" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:L63"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Story ID"/>
     <x:tableColumn id="2" name="Epic"/>
@@ -488,7 +548,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RisksTable" displayName="RisksTable" ref="A4:G22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RisksTable" displayName="RisksTable" ref="A4:G23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Risiko"/>
@@ -514,7 +574,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SourcesTable" displayName="SourcesTable" ref="A4:D13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SourcesTable" displayName="SourcesTable" ref="A4:D17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Bron"/>
     <x:tableColumn id="2" name="Gebruik"/>
@@ -744,7 +804,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="52" t="str">
-        <x:v>Sprint 0 basislyn | v0.1.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
+        <x:v>Sprint 0 amendment | v0.1.1 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
       </x:c>
       <x:c r="B2" s="51"/>
       <x:c r="C2" s="51"/>
@@ -785,8 +845,8 @@
         <x:v>Totale stories</x:v>
       </x:c>
       <x:c r="B5" s="57" t="n">
-        <x:f>COUNTA('Backlog'!$A$5:$A$61)</x:f>
-        <x:v>57</x:v>
+        <x:f>COUNTA('Backlog'!$A$5:$A$63)</x:f>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="C5" s="51"/>
       <x:c r="D5" s="56" t="str">
@@ -802,12 +862,12 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B6" s="59" t="n">
-        <x:f>COUNTIF('Backlog'!$F$5:$F$61,"Done")</x:f>
-        <x:v>1</x:v>
+        <x:f>COUNTIF('Backlog'!$F$5:$F$63,"Done")</x:f>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C6" s="51"/>
       <x:c r="D6" s="58" t="str">
-        <x:v>2. Meetbare PWM teenoor I2S-besluit</x:v>
+        <x:v>2. MAX98357 mono-I2S eerste; PWM fallback</x:v>
       </x:c>
       <x:c r="E6" s="58"/>
       <x:c r="F6" s="58"/>
@@ -819,8 +879,8 @@
         <x:v>Ready</x:v>
       </x:c>
       <x:c r="B7" s="59" t="n">
-        <x:f>COUNTIF('Backlog'!$F$5:$F$61,"Ready")</x:f>
-        <x:v>0</x:v>
+        <x:f>COUNTIF('Backlog'!$F$5:$F$63,"Ready")</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C7" s="51"/>
       <x:c r="D7" s="58" t="str">
@@ -836,8 +896,8 @@
         <x:v>MVP-gemerk</x:v>
       </x:c>
       <x:c r="B8" s="59" t="n">
-        <x:f>COUNTIF('Backlog'!$E$5:$E$61,"Must")</x:f>
-        <x:v>36</x:v>
+        <x:f>COUNTIF('Backlog'!$E$5:$E$63,"Must")</x:f>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="C8" s="51"/>
       <x:c r="D8" s="60" t="str">
@@ -853,8 +913,8 @@
         <x:v>Oop risiko’s</x:v>
       </x:c>
       <x:c r="B9" s="59" t="n">
-        <x:f>COUNTIF('Risks'!$G$5:$G$22,"&lt;&gt;Closed")</x:f>
-        <x:v>18</x:v>
+        <x:f>COUNTIF('Risks'!$G$5:$G$23,"&lt;&gt;Closed")</x:f>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C9" s="51"/>
       <x:c r="D9" s="51"/>
@@ -900,7 +960,7 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="62" t="str">
-        <x:v>Volgende story: MCP-US-002 Clean Repository And Project Skeleton</x:v>
+        <x:v>Volgende story: MCP-US-003 Minimal Safe Boot And USB Profile</x:v>
       </x:c>
       <x:c r="B13" s="51"/>
       <x:c r="C13" s="51"/>
@@ -1089,13 +1149,13 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="F6" s="24" t="str">
-        <x:v>Review</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G6" s="24" t="str">
         <x:v>Sprint 1</x:v>
       </x:c>
       <x:c r="H6" s="24" t="str">
-        <x:v>In Review/MVP</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I6" s="65" t="n">
         <x:v>5</x:v>
@@ -1127,13 +1187,13 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="F7" s="24" t="str">
-        <x:v>Backlog</x:v>
+        <x:v>Ready</x:v>
       </x:c>
       <x:c r="G7" s="24" t="str">
         <x:v>Sprint 1</x:v>
       </x:c>
       <x:c r="H7" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>Next/MVP</x:v>
       </x:c>
       <x:c r="I7" s="65" t="n">
         <x:v>8</x:v>
@@ -1574,7 +1634,7 @@
         <x:v>MCP-EPIC-003</x:v>
       </x:c>
       <x:c r="C19" s="24" t="str">
-        <x:v>Stereo PWM Diagnostic Backend</x:v>
+        <x:v>PWM Diagnostic Fallback</x:v>
       </x:c>
       <x:c r="D19" s="24" t="str">
         <x:v>DSP/Chip Engineer</x:v>
@@ -1586,13 +1646,13 @@
         <x:v>Backlog</x:v>
       </x:c>
       <x:c r="G19" s="24" t="str">
-        <x:v>Sprint 3</x:v>
+        <x:v>Sprint 4</x:v>
       </x:c>
       <x:c r="H19" s="24" t="str">
         <x:v>MVP</x:v>
       </x:c>
       <x:c r="I19" s="65" t="n">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="J19" s="24" t="str">
         <x:v>US-004, US-014</x:v>
@@ -1612,7 +1672,7 @@
         <x:v>MCP-EPIC-003</x:v>
       </x:c>
       <x:c r="C20" s="24" t="str">
-        <x:v>I2S Feasibility Spike</x:v>
+        <x:v>MAX98357 Mono I2S Audible Diagnostic</x:v>
       </x:c>
       <x:c r="D20" s="24" t="str">
         <x:v>DSP/Chip Engineer</x:v>
@@ -1630,7 +1690,7 @@
         <x:v>MVP</x:v>
       </x:c>
       <x:c r="I20" s="65" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="J20" s="24" t="str">
         <x:v>US-004, US-014</x:v>
@@ -1802,7 +1862,7 @@
         <x:v>MCP-EPIC-003</x:v>
       </x:c>
       <x:c r="C25" s="24" t="str">
-        <x:v>Audio Backend Decision</x:v>
+        <x:v>Stereo I2S Expansion Decision</x:v>
       </x:c>
       <x:c r="D25" s="24" t="str">
         <x:v>DSP/Chip Engineer</x:v>
@@ -3199,6 +3259,70 @@
       <x:c r="L61" s="25" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-057</x:v>
       </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="70" t="str">
+        <x:v>MCP-US-058</x:v>
+      </x:c>
+      <x:c r="B62" s="70" t="str">
+        <x:v>MCP-EPIC-002</x:v>
+      </x:c>
+      <x:c r="C62" s="70" t="str">
+        <x:v>Guitar MIDI Bend And Slide Event Semantics</x:v>
+      </x:c>
+      <x:c r="D62" s="70" t="str">
+        <x:v>MIDI Engineer</x:v>
+      </x:c>
+      <x:c r="E62" s="76" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="F62" s="70" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="G62" s="70" t="str">
+        <x:v>Sprint 4</x:v>
+      </x:c>
+      <x:c r="H62" s="70" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="I62" s="77" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J62"/>
+      <x:c r="K62"/>
+      <x:c r="L62"/>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="74" t="str">
+        <x:v>MCP-US-059</x:v>
+      </x:c>
+      <x:c r="B63" s="74" t="str">
+        <x:v>MCP-EPIC-008</x:v>
+      </x:c>
+      <x:c r="C63" s="74" t="str">
+        <x:v>MIDI Guitar Hardware Acceptance</x:v>
+      </x:c>
+      <x:c r="D63" s="74" t="str">
+        <x:v>QA/Release</x:v>
+      </x:c>
+      <x:c r="E63" s="76" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="F63" s="74" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="G63" s="74" t="str">
+        <x:v>Release train</x:v>
+      </x:c>
+      <x:c r="H63" s="74" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="I63" s="78" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J63"/>
+      <x:c r="K63"/>
+      <x:c r="L63"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3213,17 +3337,23 @@
     <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Ready"/>
     <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="Blocked"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="2">
+  <x:dataValidations count="4">
     <x:dataValidation type="list" sqref="E5:E61">
       <x:formula1>"Must,Should,Could,Won't now"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="F5:F61">
       <x:formula1>"Backlog,Ready,In Progress,Blocked,Review,Done"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="E62:E63">
+      <x:formula1>"Must,Should,Could,Won't now"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="F62:F63">
+      <x:formula1>"Backlog,Ready,In Progress,Review,Done,Impediment"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbb7f6a2d09c4660"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra072c94199a14fe6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3278,16 +3408,16 @@
         <x:v>Platform Foundation</x:v>
       </x:c>
       <x:c r="C5" s="64" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$61,A5)</x:f>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$63,A5)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D5" s="64" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$61,A5,'Backlog'!$E$5:$E$61,"Must")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A5,'Backlog'!$E$5:$E$63,"Must")</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="E5" s="64" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$61,A5,'Backlog'!$F$5:$F$61,"Done")</x:f>
-        <x:v>1</x:v>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A5,'Backlog'!$F$5:$F$63,"Done")</x:f>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F5" s="23" t="str">
         <x:v>Veilige, draagbare basis en konfigurasiegrens</x:v>
@@ -3301,19 +3431,19 @@
         <x:v>MIDI And Clock</x:v>
       </x:c>
       <x:c r="C6" s="65" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$61,A6)</x:f>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$63,A6)</x:f>
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D6" s="65" t="n">
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A6,'Backlog'!$E$5:$E$63,"Must")</x:f>
         <x:v>8</x:v>
       </x:c>
-      <x:c r="D6" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$61,A6,'Backlog'!$E$5:$E$61,"Must")</x:f>
-        <x:v>7</x:v>
-      </x:c>
       <x:c r="E6" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$61,A6,'Backlog'!$F$5:$F$61,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A6,'Backlog'!$F$5:$F$63,"Done")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F6" s="24" t="str">
-        <x:v>USB-MIDI, kontroles en interne/eksterne klok</x:v>
+        <x:v>USB-MIDI, guitar slides, kontroles en interne/eksterne klok</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="32" customHeight="1">
@@ -3324,19 +3454,19 @@
         <x:v>Audio And Chip Core</x:v>
       </x:c>
       <x:c r="C7" s="65" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$61,A7)</x:f>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$63,A7)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D7" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$61,A7,'Backlog'!$E$5:$E$61,"Must")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A7,'Backlog'!$E$5:$E$63,"Must")</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="E7" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$61,A7,'Backlog'!$F$5:$F$61,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A7,'Backlog'!$F$5:$F$63,"Done")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F7" s="24" t="str">
-        <x:v>SN76489, stereo-uitvoer en backendbesluit</x:v>
+        <x:v>MAX98357 mono eerste, SN76489 en latere stereo</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="32" customHeight="1">
@@ -3347,15 +3477,15 @@
         <x:v>Local Web Control</x:v>
       </x:c>
       <x:c r="C8" s="65" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$61,A8)</x:f>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$63,A8)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="D8" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$61,A8,'Backlog'!$E$5:$E$61,"Must")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A8,'Backlog'!$E$5:$E$63,"Must")</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="E8" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$61,A8,'Backlog'!$F$5:$F$61,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A8,'Backlog'!$F$5:$F$63,"Done")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F8" s="24" t="str">
@@ -3370,15 +3500,15 @@
         <x:v>Files, Harmony And Performance Tools</x:v>
       </x:c>
       <x:c r="C9" s="65" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$61,A9)</x:f>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$63,A9)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="D9" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$61,A9,'Backlog'!$E$5:$E$61,"Must")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A9,'Backlog'!$E$5:$E$63,"Must")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="E9" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$61,A9,'Backlog'!$F$5:$F$61,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A9,'Backlog'!$F$5:$F$63,"Done")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F9" s="24" t="str">
@@ -3393,15 +3523,15 @@
         <x:v>Multi-Core Expansion</x:v>
       </x:c>
       <x:c r="C10" s="65" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$61,A10)</x:f>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$63,A10)</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="D10" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$61,A10,'Backlog'!$E$5:$E$61,"Must")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A10,'Backlog'!$E$5:$E$63,"Must")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="E10" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$61,A10,'Backlog'!$F$5:$F$61,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A10,'Backlog'!$F$5:$F$63,"Done")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F10" s="24" t="str">
@@ -3416,15 +3546,15 @@
         <x:v>DSP And Pedal Hardware</x:v>
       </x:c>
       <x:c r="C11" s="65" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$61,A11)</x:f>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$63,A11)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="D11" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$61,A11,'Backlog'!$E$5:$E$61,"Must")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A11,'Backlog'!$E$5:$E$63,"Must")</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="E11" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$61,A11,'Backlog'!$F$5:$F$61,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A11,'Backlog'!$F$5:$F$63,"Done")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F11" s="24" t="str">
@@ -3439,15 +3569,15 @@
         <x:v>Portability, Quality And Release</x:v>
       </x:c>
       <x:c r="C12" s="66" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$61,A12)</x:f>
-        <x:v>8</x:v>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$63,A12)</x:f>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D12" s="66" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$61,A12,'Backlog'!$E$5:$E$61,"Must")</x:f>
-        <x:v>6</x:v>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A12,'Backlog'!$E$5:$E$63,"Must")</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E12" s="66" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$61,A12,'Backlog'!$F$5:$F$61,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A12,'Backlog'!$F$5:$F$63,"Done")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F12" s="25" t="str">
@@ -3461,7 +3591,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3955fa81b6764d93"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7178c6a43a2b4d0e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3621,7 +3751,7 @@
         <x:v>Embedded</x:v>
       </x:c>
       <x:c r="F9" s="24" t="str">
-        <x:v>Capability profile en PWM fallback</x:v>
+        <x:v>Capability profile, MAX98357 HIL en PWM fallback</x:v>
       </x:c>
       <x:c r="G9" s="24" t="str">
         <x:v>Open</x:v>
@@ -3793,7 +3923,7 @@
         <x:v>R-013</x:v>
       </x:c>
       <x:c r="B17" s="24" t="str">
-        <x:v>Klankvlak beskadig uitsetketting</x:v>
+        <x:v>MAX98357 bridge-tied uitset word geaard of as line-out gebruik</x:v>
       </x:c>
       <x:c r="C17" s="24" t="str">
         <x:v>Medium</x:v>
@@ -3805,7 +3935,7 @@
         <x:v>Hardware</x:v>
       </x:c>
       <x:c r="F17" s="24" t="str">
-        <x:v>Filter/buffer/versterker en meting</x:v>
+        <x:v>Luidspreker tussen + en -; geen grond/line-input; HIL checklist</x:v>
       </x:c>
       <x:c r="G17" s="24" t="str">
         <x:v>Open</x:v>
@@ -3924,6 +4054,29 @@
       </x:c>
       <x:c r="G22" s="25" t="str">
         <x:v>Controlled</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="82" t="str">
+        <x:v>R-019</x:v>
+      </x:c>
+      <x:c r="B23" s="82" t="str">
+        <x:v>MIDI-kitaar bend range/kanaalmodus maak slides vals</x:v>
+      </x:c>
+      <x:c r="C23" s="82" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="D23" s="82" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E23" s="82" t="str">
+        <x:v>MIDI/QA</x:v>
+      </x:c>
+      <x:c r="F23" s="82" t="str">
+        <x:v>Configurable bend range, per-channel state en guitar HIL</x:v>
+      </x:c>
+      <x:c r="G23" s="82" t="str">
+        <x:v>Open</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3937,14 +4090,17 @@
   <x:conditionalFormatting sqref="G5:G22">
     <x:cfRule type="containsText" dxfId="5" priority="2" operator="containsText" text="Closed"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="1">
+  <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="G5:G22">
       <x:formula1>"Open,Open - human action,Controlled,Closed"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="G23">
+      <x:formula1>"Open,Controlled,Open - human action,Closed"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R296102fe929b4307"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71ccb7d78b6445d7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4107,7 +4263,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16292d9c9bdd4cc6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb0eb2b4c4c34598"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4272,6 +4428,62 @@
         <x:v>Private backup; never publish</x:v>
       </x:c>
     </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="70" t="str">
+        <x:v>Adafruit MAX98357 overview</x:v>
+      </x:c>
+      <x:c r="B14" s="70" t="str">
+        <x:v>Mono-I2S, sample rates en mono mix</x:v>
+      </x:c>
+      <x:c r="C14" s="70" t="str">
+        <x:v>Official guide</x:v>
+      </x:c>
+      <x:c r="D14" s="70" t="str">
+        <x:v>https://learn.adafruit.com/adafruit-max98357-i2s-class-d-mono-amp/overview</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="74" t="str">
+        <x:v>Adafruit MAX98357 pinouts</x:v>
+      </x:c>
+      <x:c r="B15" s="74" t="str">
+        <x:v>BCLK/LRC/DIN en bridge-tied safety</x:v>
+      </x:c>
+      <x:c r="C15" s="74" t="str">
+        <x:v>Official guide</x:v>
+      </x:c>
+      <x:c r="D15" s="74" t="str">
+        <x:v>https://learn.adafruit.com/adafruit-max98357-i2s-class-d-mono-amp/pinouts</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="70" t="str">
+        <x:v>Fishman TriplePlay Support</x:v>
+      </x:c>
+      <x:c r="B16" s="70" t="str">
+        <x:v>Polyphonic MIDI guitar en string bends</x:v>
+      </x:c>
+      <x:c r="C16" s="70" t="str">
+        <x:v>Official support</x:v>
+      </x:c>
+      <x:c r="D16" s="70" t="str">
+        <x:v>https://fishman.com/tripleplay-support/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="74" t="str">
+        <x:v>Fishman TriplePlay Utility Guide</x:v>
+      </x:c>
+      <x:c r="B17" s="74" t="str">
+        <x:v>Trigger/Auto/Smooth/Step slides</x:v>
+      </x:c>
+      <x:c r="C17" s="74" t="str">
+        <x:v>Official manual</x:v>
+      </x:c>
+      <x:c r="D17" s="74" t="str">
+        <x:v>https://a11.fishman.com/wp-content/uploads/2024/12/TriplePlayUtility-UserGuide.pdf</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>
@@ -4279,7 +4491,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa485911b12f44e5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb3b371d215e45d1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add safe USB MIDI boot foundation
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R2d35e002868d47cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="Rf34e61054ef14a33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Rc0f371a6e07943e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R1d263501791f479f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R7094a3da1d0c4ed6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rdcc1eca3050c46e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ra1ef64c7c08b4bda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="Rab88813820454820"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="R9fcecd959b234576"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R596f8fa4eee0486e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R3ff641c0b2544368"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R95b8de5c467d49d3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -513,8 +513,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BacklogTable" displayName="BacklogTable" ref="A4:L63" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:L63"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BacklogTable" displayName="BacklogTable" ref="A4:L65" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:L65"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Story ID"/>
     <x:tableColumn id="2" name="Epic"/>
@@ -548,7 +548,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RisksTable" displayName="RisksTable" ref="A4:G23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RisksTable" displayName="RisksTable" ref="A4:G26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Risiko"/>
@@ -563,7 +563,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RolesTable" displayName="RolesTable" ref="A4:C15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RolesTable" displayName="RolesTable" ref="A4:C16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="Rol"/>
     <x:tableColumn id="2" name="Verantwoordelikheid"/>
@@ -574,7 +574,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SourcesTable" displayName="SourcesTable" ref="A4:D17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SourcesTable" displayName="SourcesTable" ref="A4:D21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Bron"/>
     <x:tableColumn id="2" name="Gebruik"/>
@@ -804,7 +804,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="52" t="str">
-        <x:v>Sprint 0 amendment | v0.1.1 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
+        <x:v>Sprint 1 | v0.2.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
       </x:c>
       <x:c r="B2" s="51"/>
       <x:c r="C2" s="51"/>
@@ -845,12 +845,12 @@
         <x:v>Totale stories</x:v>
       </x:c>
       <x:c r="B5" s="57" t="n">
-        <x:f>COUNTA('Backlog'!$A$5:$A$63)</x:f>
-        <x:v>59</x:v>
+        <x:f>COUNTA('Backlog'!$A$5:$A$65)</x:f>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="C5" s="51"/>
       <x:c r="D5" s="56" t="str">
-        <x:v>1. Veilige minimale USB-MIDI boot</x:v>
+        <x:v>1. Veilige minimale USB-MIDI boot en herstel</x:v>
       </x:c>
       <x:c r="E5" s="56"/>
       <x:c r="F5" s="56"/>
@@ -862,7 +862,7 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B6" s="59" t="n">
-        <x:f>COUNTIF('Backlog'!$F$5:$F$63,"Done")</x:f>
+        <x:f>COUNTIF('Backlog'!$F$5:$F$65,"Done")</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="C6" s="51"/>
@@ -876,15 +876,15 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="58" t="str">
-        <x:v>Ready</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="B7" s="59" t="n">
-        <x:f>COUNTIF('Backlog'!$F$5:$F$63,"Ready")</x:f>
+        <x:f>COUNTIF('Backlog'!$F$5:$F$65,"In Progress")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="C7" s="51"/>
       <x:c r="D7" s="58" t="str">
-        <x:v>3. Webpolling mag nie MIDI/klank destabiliseer nie</x:v>
+        <x:v>3. Standalone host/DIN-transport moet sonder DAW slaag</x:v>
       </x:c>
       <x:c r="E7" s="58"/>
       <x:c r="F7" s="58"/>
@@ -896,12 +896,12 @@
         <x:v>MVP-gemerk</x:v>
       </x:c>
       <x:c r="B8" s="59" t="n">
-        <x:f>COUNTIF('Backlog'!$E$5:$E$63,"Must")</x:f>
-        <x:v>38</x:v>
+        <x:f>COUNTIF('Backlog'!$E$5:$E$65,"Must")</x:f>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="C8" s="51"/>
       <x:c r="D8" s="60" t="str">
-        <x:v>4. Tweede kern eers ná SN76489 en poortkontrakte</x:v>
+        <x:v>4. Twee verskillende kerne eers na een-kern-bewys en resource gate</x:v>
       </x:c>
       <x:c r="E8" s="60"/>
       <x:c r="F8" s="60"/>
@@ -913,8 +913,8 @@
         <x:v>Oop risiko’s</x:v>
       </x:c>
       <x:c r="B9" s="59" t="n">
-        <x:f>COUNTIF('Risks'!$G$5:$G$23,"&lt;&gt;Closed")</x:f>
-        <x:v>19</x:v>
+        <x:f>COUNTIF('Risks'!$G$5:$G$26,"&lt;&gt;Closed")</x:f>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C9" s="51"/>
       <x:c r="D9" s="51"/>
@@ -928,8 +928,8 @@
         <x:v>Virtuele rolle</x:v>
       </x:c>
       <x:c r="B10" s="61" t="n">
-        <x:f>COUNTA('Team RACI'!$A$5:$A$15)</x:f>
-        <x:v>11</x:v>
+        <x:f>COUNTA('Team RACI'!$A$5:$A$16)</x:f>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C10" s="51"/>
       <x:c r="D10" s="51"/>
@@ -960,7 +960,7 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="62" t="str">
-        <x:v>Volgende story: MCP-US-003 Minimal Safe Boot And USB Profile</x:v>
+        <x:v>Aktiewe story: MCP-US-003 Minimal Safe Boot And USB Profile | HIL proof volg</x:v>
       </x:c>
       <x:c r="B13" s="51"/>
       <x:c r="C13" s="51"/>
@@ -1053,7 +1053,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Bron: docs/user_stories_v0.1.0.md | Redigeer Status en Priority via keuselyste</x:v>
+        <x:v>Bron: docs/user_stories_v0.1.0.md | 61 stories | Redigeer Status en Priority via keuselyste</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -1187,13 +1187,13 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="F7" s="24" t="str">
-        <x:v>Ready</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="G7" s="24" t="str">
         <x:v>Sprint 1</x:v>
       </x:c>
       <x:c r="H7" s="24" t="str">
-        <x:v>Next/MVP</x:v>
+        <x:v>In Progress/MVP</x:v>
       </x:c>
       <x:c r="I7" s="65" t="n">
         <x:v>8</x:v>
@@ -1202,7 +1202,7 @@
         <x:v>US-002</x:v>
       </x:c>
       <x:c r="K7" s="24" t="str">
-        <x:v>USB-MIDI begin vóór runtime; geen netwerk of geheime in `boot.py` nie</x:v>
+        <x:v>USB-MIDI begin voor runtime; bord-VID/PID bly verstek; CIRCUITPY/REPL herstel en drieledige device-proof slaag</x:v>
       </x:c>
       <x:c r="L7" s="24" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-003</x:v>
@@ -1354,7 +1354,7 @@
         <x:v>US-003, US-006</x:v>
       </x:c>
       <x:c r="K11" s="24" t="str">
-        <x:v>Enige klas-kompatibele USB-MIDI-bron kan Note On/Off stuur</x:v>
+        <x:v>Enige klas-kompatibele bron kan via 'n rekenaar/DAW of eksterne USB-host Note On/Off stuur sonder toestelnaamkonstante</x:v>
       </x:c>
       <x:c r="L11" s="24" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-007</x:v>
@@ -1558,13 +1558,13 @@
         <x:v>MCP-EPIC-002</x:v>
       </x:c>
       <x:c r="C17" s="24" t="str">
-        <x:v>External IO MIDI Transport Spike</x:v>
+        <x:v>Standalone DIN UART MIDI Transport</x:v>
       </x:c>
       <x:c r="D17" s="24" t="str">
         <x:v>MIDI Engineer</x:v>
       </x:c>
       <x:c r="E17" s="24" t="str">
-        <x:v>Should</x:v>
+        <x:v>Must</x:v>
       </x:c>
       <x:c r="F17" s="24" t="str">
         <x:v>Backlog</x:v>
@@ -1573,19 +1573,19 @@
         <x:v>Sprint 3</x:v>
       </x:c>
       <x:c r="H17" s="24" t="str">
-        <x:v>Later</x:v>
+        <x:v>MVP</x:v>
       </x:c>
       <x:c r="I17" s="65" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="J17" s="24" t="str">
-        <x:v>US-007</x:v>
+        <x:v>US-006</x:v>
       </x:c>
       <x:c r="K17" s="24" t="str">
-        <x:v>UART/DIN- of ander IO-adapter word deur dieselfde MIDI-poort geabstraheer</x:v>
+        <x:v>'n Eksterne USB-host se 5-pen DIN/UART-boodskappe gebruik dieselfde MidiInputPort en eventmodel</x:v>
       </x:c>
       <x:c r="L17" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-013</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MIDI-TRANSPORT-MULTICORE-AMENDMENT-001 / MCP-US-013</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="38" customHeight="1">
@@ -2400,16 +2400,16 @@
         <x:v>DSP/Chip Engineer</x:v>
       </x:c>
       <x:c r="E39" s="24" t="str">
-        <x:v>Should</x:v>
+        <x:v>Must</x:v>
       </x:c>
       <x:c r="F39" s="24" t="str">
         <x:v>Backlog</x:v>
       </x:c>
       <x:c r="G39" s="24" t="str">
-        <x:v>Post-MVP</x:v>
+        <x:v>MVP-late</x:v>
       </x:c>
       <x:c r="H39" s="24" t="str">
-        <x:v>Later</x:v>
+        <x:v>MVP-late</x:v>
       </x:c>
       <x:c r="I39" s="65" t="n">
         <x:v>8</x:v>
@@ -2438,16 +2438,16 @@
         <x:v>DSP/Chip Engineer</x:v>
       </x:c>
       <x:c r="E40" s="24" t="str">
-        <x:v>Should</x:v>
+        <x:v>Must</x:v>
       </x:c>
       <x:c r="F40" s="24" t="str">
         <x:v>Backlog</x:v>
       </x:c>
       <x:c r="G40" s="24" t="str">
-        <x:v>Post-MVP</x:v>
+        <x:v>MVP-late</x:v>
       </x:c>
       <x:c r="H40" s="24" t="str">
-        <x:v>Later</x:v>
+        <x:v>MVP-late</x:v>
       </x:c>
       <x:c r="I40" s="65" t="n">
         <x:v>5</x:v>
@@ -2476,16 +2476,16 @@
         <x:v>DSP/Chip Engineer</x:v>
       </x:c>
       <x:c r="E41" s="24" t="str">
-        <x:v>Should</x:v>
+        <x:v>Must</x:v>
       </x:c>
       <x:c r="F41" s="24" t="str">
         <x:v>Backlog</x:v>
       </x:c>
       <x:c r="G41" s="24" t="str">
-        <x:v>Post-MVP</x:v>
+        <x:v>MVP-late</x:v>
       </x:c>
       <x:c r="H41" s="24" t="str">
-        <x:v>Later</x:v>
+        <x:v>MVP-late</x:v>
       </x:c>
       <x:c r="I41" s="65" t="n">
         <x:v>8</x:v>
@@ -2494,10 +2494,10 @@
         <x:v>US-035, US-036</x:v>
       </x:c>
       <x:c r="K41" s="24" t="str">
-        <x:v>Minstens twee kerne loop binne ’n gemete CPU/RAM-begroting</x:v>
+        <x:v>Minstens twee verskillende kerninstansies loop parallel binne 'n gemete CPU/RAM/latensiebegroting</x:v>
       </x:c>
       <x:c r="L41" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-037</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MIDI-TRANSPORT-MULTICORE-AMENDMENT-001 / MCP-US-037</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="38" customHeight="1">
@@ -3026,7 +3026,7 @@
         <x:v>US-003, US-015</x:v>
       </x:c>
       <x:c r="K55" s="24" t="str">
-        <x:v>REPL, USB-MIDI en klankmeetstappe lewer ’n naspeurbare verslag</x:v>
+        <x:v>Connection, deploy en execution proof plus USB-MIDI en klankmeetstappe lewer 'n geredigeerde naspeurbare verslag</x:v>
       </x:c>
       <x:c r="L55" s="24" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-051</x:v>
@@ -3178,7 +3178,7 @@
         <x:v>US-003, US-007</x:v>
       </x:c>
       <x:c r="K59" s="24" t="str">
-        <x:v>Logic stuur note/clock en ontvang ’n stabiele uitvoerpad</x:v>
+        <x:v>Logic kies die synth as External MIDI destination en stuur note/clock; fisiese pedaaluitvoer bly die klankpad</x:v>
       </x:c>
       <x:c r="L59" s="24" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-055</x:v>
@@ -3260,7 +3260,7 @@
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-057</x:v>
       </x:c>
     </x:row>
-    <x:row r="62">
+    <x:row r="62" ht="34" customHeight="1">
       <x:c r="A62" s="70" t="str">
         <x:v>MCP-US-058</x:v>
       </x:c>
@@ -3288,11 +3288,17 @@
       <x:c r="I62" s="77" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="J62"/>
-      <x:c r="K62"/>
-      <x:c r="L62"/>
-    </x:row>
-    <x:row r="63">
+      <x:c r="J62" t="str">
+        <x:v>US-008, US-010</x:v>
+      </x:c>
+      <x:c r="K62" t="str">
+        <x:v>Multi-kanaal note en per-kanaal bends behou onafhanklike string/slide-semantiek met konfigureerbare bend range</x:v>
+      </x:c>
+      <x:c r="L62" t="str">
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-058</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63" ht="34" customHeight="1">
       <x:c r="A63" s="74" t="str">
         <x:v>MCP-US-059</x:v>
       </x:c>
@@ -3320,9 +3326,91 @@
       <x:c r="I63" s="78" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="J63"/>
-      <x:c r="K63"/>
-      <x:c r="L63"/>
+      <x:c r="J63" t="str">
+        <x:v>US-018, US-058</x:v>
+      </x:c>
+      <x:c r="K63" t="str">
+        <x:v>'n Generiese MIDI-kitaar en Fishman-verwysing speel note, akkoorde, bends en slides; geen toestelnaam is 'n kodekonstante nie</x:v>
+      </x:c>
+      <x:c r="L63" t="str">
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-059</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64" ht="34" customHeight="1">
+      <x:c r="A64" t="str">
+        <x:v>MCP-US-060</x:v>
+      </x:c>
+      <x:c r="B64" t="str">
+        <x:v>MCP-EPIC-008</x:v>
+      </x:c>
+      <x:c r="C64" t="str">
+        <x:v>Standalone External MIDI Host Acceptance</x:v>
+      </x:c>
+      <x:c r="D64" t="str">
+        <x:v>QA/Release</x:v>
+      </x:c>
+      <x:c r="E64" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="F64" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="G64" t="str">
+        <x:v>Release train</x:v>
+      </x:c>
+      <x:c r="H64" t="str">
+        <x:v>MVP</x:v>
+      </x:c>
+      <x:c r="I64" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J64" t="str">
+        <x:v>US-013, US-017</x:v>
+      </x:c>
+      <x:c r="K64" t="str">
+        <x:v>Controller na Raspberry Pi/eksterne USB-host na DIN/UART lewer note, bend en clock sonder DAW</x:v>
+      </x:c>
+      <x:c r="L64" t="str">
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MIDI-TRANSPORT-MULTICORE-AMENDMENT-001 / MCP-US-060</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65" ht="34" customHeight="1">
+      <x:c r="A65" t="str">
+        <x:v>MCP-US-061</x:v>
+      </x:c>
+      <x:c r="B65" t="str">
+        <x:v>MCP-EPIC-006</x:v>
+      </x:c>
+      <x:c r="C65" t="str">
+        <x:v>Multi-Core Resource Guard And Telemetry</x:v>
+      </x:c>
+      <x:c r="D65" t="str">
+        <x:v>DSP/Chip Engineer</x:v>
+      </x:c>
+      <x:c r="E65" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="F65" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="G65" t="str">
+        <x:v>MVP-late</x:v>
+      </x:c>
+      <x:c r="H65" t="str">
+        <x:v>MVP-late</x:v>
+      </x:c>
+      <x:c r="I65" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J65" t="str">
+        <x:v>US-037</x:v>
+      </x:c>
+      <x:c r="K65" t="str">
+        <x:v>Heap, looplatensie en dropout word gemeet; onveilige addisionele kern word deterministies geweier of afgeskakel</x:v>
+      </x:c>
+      <x:c r="L65" t="str">
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MIDI-TRANSPORT-MULTICORE-AMENDMENT-001 / MCP-US-061</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -3353,7 +3441,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra072c94199a14fe6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc104f2338ed64c8e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3408,15 +3496,15 @@
         <x:v>Platform Foundation</x:v>
       </x:c>
       <x:c r="C5" s="64" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$63,A5)</x:f>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$65,A5)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D5" s="64" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A5,'Backlog'!$E$5:$E$63,"Must")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A5,'Backlog'!$E$5:$E$65,"Must")</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="E5" s="64" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A5,'Backlog'!$F$5:$F$63,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A5,'Backlog'!$F$5:$F$65,"Done")</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="F5" s="23" t="str">
@@ -3431,15 +3519,15 @@
         <x:v>MIDI And Clock</x:v>
       </x:c>
       <x:c r="C6" s="65" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$63,A6)</x:f>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$65,A6)</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="D6" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A6,'Backlog'!$E$5:$E$63,"Must")</x:f>
-        <x:v>8</x:v>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A6,'Backlog'!$E$5:$E$65,"Must")</x:f>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="E6" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A6,'Backlog'!$F$5:$F$63,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A6,'Backlog'!$F$5:$F$65,"Done")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F6" s="24" t="str">
@@ -3454,15 +3542,15 @@
         <x:v>Audio And Chip Core</x:v>
       </x:c>
       <x:c r="C7" s="65" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$63,A7)</x:f>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$65,A7)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="D7" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A7,'Backlog'!$E$5:$E$63,"Must")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A7,'Backlog'!$E$5:$E$65,"Must")</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="E7" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A7,'Backlog'!$F$5:$F$63,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A7,'Backlog'!$F$5:$F$65,"Done")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F7" s="24" t="str">
@@ -3477,15 +3565,15 @@
         <x:v>Local Web Control</x:v>
       </x:c>
       <x:c r="C8" s="65" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$63,A8)</x:f>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$65,A8)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="D8" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A8,'Backlog'!$E$5:$E$63,"Must")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A8,'Backlog'!$E$5:$E$65,"Must")</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="E8" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A8,'Backlog'!$F$5:$F$63,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A8,'Backlog'!$F$5:$F$65,"Done")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F8" s="24" t="str">
@@ -3500,15 +3588,15 @@
         <x:v>Files, Harmony And Performance Tools</x:v>
       </x:c>
       <x:c r="C9" s="65" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$63,A9)</x:f>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$65,A9)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="D9" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A9,'Backlog'!$E$5:$E$63,"Must")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A9,'Backlog'!$E$5:$E$65,"Must")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="E9" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A9,'Backlog'!$F$5:$F$63,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A9,'Backlog'!$F$5:$F$65,"Done")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F9" s="24" t="str">
@@ -3523,15 +3611,15 @@
         <x:v>Multi-Core Expansion</x:v>
       </x:c>
       <x:c r="C10" s="65" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$63,A10)</x:f>
-        <x:v>9</x:v>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$65,A10)</x:f>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D10" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A10,'Backlog'!$E$5:$E$63,"Must")</x:f>
-        <x:v>1</x:v>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A10,'Backlog'!$E$5:$E$65,"Must")</x:f>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E10" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A10,'Backlog'!$F$5:$F$63,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A10,'Backlog'!$F$5:$F$65,"Done")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F10" s="24" t="str">
@@ -3546,15 +3634,15 @@
         <x:v>DSP And Pedal Hardware</x:v>
       </x:c>
       <x:c r="C11" s="65" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$63,A11)</x:f>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$65,A11)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="D11" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A11,'Backlog'!$E$5:$E$63,"Must")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A11,'Backlog'!$E$5:$E$65,"Must")</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="E11" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A11,'Backlog'!$F$5:$F$63,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A11,'Backlog'!$F$5:$F$65,"Done")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F11" s="24" t="str">
@@ -3569,15 +3657,15 @@
         <x:v>Portability, Quality And Release</x:v>
       </x:c>
       <x:c r="C12" s="66" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$63,A12)</x:f>
-        <x:v>9</x:v>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$65,A12)</x:f>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D12" s="66" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A12,'Backlog'!$E$5:$E$63,"Must")</x:f>
-        <x:v>7</x:v>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A12,'Backlog'!$E$5:$E$65,"Must")</x:f>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="E12" s="66" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$63,A12,'Backlog'!$F$5:$F$63,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A12,'Backlog'!$F$5:$F$65,"Done")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F12" s="25" t="str">
@@ -3591,7 +3679,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7178c6a43a2b4d0e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32f3f5c6ad854c21"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3601,11 +3689,11 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="43" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="50" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="54" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="62" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -3616,7 +3704,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Hoë risiko’s word vroeg sigbaar gemaak; geen demo-status verberg ’n blocker nie</x:v>
+        <x:v>22 aktiewe risiko's; hoe risiko's word vroeg sigbaar gemaak en geen demo-status verberg 'n blocker nie</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -3843,7 +3931,7 @@
         <x:v>DSP</x:v>
       </x:c>
       <x:c r="F13" s="24" t="str">
-        <x:v>Een kern in MVP; budget gate</x:v>
+        <x:v>Een kern eerste; twee verskillende kerne slegs na resource gate en MCP-US-061 telemetry</x:v>
       </x:c>
       <x:c r="G13" s="24" t="str">
         <x:v>Open</x:v>
@@ -4056,7 +4144,7 @@
         <x:v>Controlled</x:v>
       </x:c>
     </x:row>
-    <x:row r="23">
+    <x:row r="23" ht="40" customHeight="1">
       <x:c r="A23" s="82" t="str">
         <x:v>R-019</x:v>
       </x:c>
@@ -4076,6 +4164,75 @@
         <x:v>Configurable bend range, per-channel state en guitar HIL</x:v>
       </x:c>
       <x:c r="G23" s="82" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="40" customHeight="1">
+      <x:c r="A24" t="str">
+        <x:v>R-020</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>USB-host en USB-device rolle word verwar</x:v>
+      </x:c>
+      <x:c r="C24" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="D24" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E24" t="str">
+        <x:v>Architect/MIDI</x:v>
+      </x:c>
+      <x:c r="F24" t="str">
+        <x:v>Dokumenteer controller-host-device-DIN-ketting en toets sonder DAW</x:v>
+      </x:c>
+      <x:c r="G24" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="40" customHeight="1">
+      <x:c r="A25" t="str">
+        <x:v>R-021</x:v>
+      </x:c>
+      <x:c r="B25" t="str">
+        <x:v>Device-proof publiseer UID, MAC, SSID of geheime</x:v>
+      </x:c>
+      <x:c r="C25" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="D25" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="E25" t="str">
+        <x:v>QA/Release</x:v>
+      </x:c>
+      <x:c r="F25" t="str">
+        <x:v>Drievlak-bewys word geredigeer; private rugsteun buite Git</x:v>
+      </x:c>
+      <x:c r="G25" t="str">
+        <x:v>Controlled</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="40" customHeight="1">
+      <x:c r="A26" t="str">
+        <x:v>R-022</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>MIDI-HIL hang deur poortkonflik met Thonny of serial monitor</x:v>
+      </x:c>
+      <x:c r="C26" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="D26" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E26" t="str">
+        <x:v>QA/HIL</x:v>
+      </x:c>
+      <x:c r="F26" t="str">
+        <x:v>Preflight lsof; een REPL-klient; timeout en herstelpad</x:v>
+      </x:c>
+      <x:c r="G26" t="str">
         <x:v>Open</x:v>
       </x:c>
     </x:row>
@@ -4100,7 +4257,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71ccb7d78b6445d7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b43652cb5f647c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4109,9 +4266,9 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="48" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="48" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="38" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="45" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="52" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
@@ -4121,7 +4278,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Elke rol gee ’n sigbare bydrae; PO bly die finale aanvaarder</x:v>
+        <x:v>Elke interne rol gee 'n sigbare bydrae; Copilot adviseer as eksterne reviewer; PO bly finale aanvaarder</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -4254,6 +4411,17 @@
       </x:c>
       <x:c r="C15" s="25" t="str">
         <x:v>Publikasiehek en docs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="38" customHeight="1">
+      <x:c r="A16" t="str">
+        <x:v>External Architecture Reviewer (Copilot)</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>Onafhanklike ontwerp- en risiko-review</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>Bevindings is advies; PO/architect besluit en traceer</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4263,7 +4431,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb0eb2b4c4c34598"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9889003f50674b16"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4285,7 +4453,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Primêre dokumentasie voor sekondêre demonstrasies; hardeware-eise vereis eie meting</x:v>
+        <x:v>Primere dokumentasie voor sekondere demonstrasies; transport- en hardeware-eise vereis eie meting</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -4428,7 +4596,7 @@
         <x:v>Private backup; never publish</x:v>
       </x:c>
     </x:row>
-    <x:row r="14">
+    <x:row r="14" ht="28" customHeight="1">
       <x:c r="A14" s="70" t="str">
         <x:v>Adafruit MAX98357 overview</x:v>
       </x:c>
@@ -4442,7 +4610,7 @@
         <x:v>https://learn.adafruit.com/adafruit-max98357-i2s-class-d-mono-amp/overview</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
+    <x:row r="15" ht="28" customHeight="1">
       <x:c r="A15" s="74" t="str">
         <x:v>Adafruit MAX98357 pinouts</x:v>
       </x:c>
@@ -4456,7 +4624,7 @@
         <x:v>https://learn.adafruit.com/adafruit-max98357-i2s-class-d-mono-amp/pinouts</x:v>
       </x:c>
     </x:row>
-    <x:row r="16">
+    <x:row r="16" ht="28" customHeight="1">
       <x:c r="A16" s="70" t="str">
         <x:v>Fishman TriplePlay Support</x:v>
       </x:c>
@@ -4470,7 +4638,7 @@
         <x:v>https://fishman.com/tripleplay-support/</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
+    <x:row r="17" ht="28" customHeight="1">
       <x:c r="A17" s="74" t="str">
         <x:v>Fishman TriplePlay Utility Guide</x:v>
       </x:c>
@@ -4482,6 +4650,62 @@
       </x:c>
       <x:c r="D17" s="74" t="str">
         <x:v>https://a11.fishman.com/wp-content/uploads/2024/12/TriplePlayUtility-UserGuide.pdf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="28" customHeight="1">
+      <x:c r="A18" t="str">
+        <x:v>CircuitPython supervisor</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>USB-identiteit en runtime-inspeksie</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>Official API</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>https://docs.circuitpython.org/en/latest/shared-bindings/supervisor/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="28" customHeight="1">
+      <x:c r="A19" t="str">
+        <x:v>CircuitPython USB customization</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>boot.py endpoint- en herstelgedrag</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>Official guide</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>https://learn.adafruit.com/customizing-usb-devices-in-circuitpython</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="28" customHeight="1">
+      <x:c r="A20" t="str">
+        <x:v>DOREMiDi USB MIDI Host</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>Standalone controller-host-DIN transport</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>Vendor reference</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>https://www.doremidi.cn/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="28" customHeight="1">
+      <x:c r="A21" t="str">
+        <x:v>RaspiMIDIHub</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>Standalone Raspberry Pi MIDI-host patroon</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>Public project</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>https://github.com/rppicomidi/RasPiMIDIHub</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4491,7 +4715,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb3b371d215e45d1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a00e1868f7f4e23"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add redacted hardware in loop verification
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ra1ef64c7c08b4bda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="Rab88813820454820"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="R9fcecd959b234576"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R596f8fa4eee0486e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R3ff641c0b2544368"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R95b8de5c467d49d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rdd19fbb7426d49e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R3d8ccb4094e7426a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="R4379077619f64dfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="Rd65e7e5093f54f4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R72ded0b324cc43bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Re84e7d5b1aa24452"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -804,7 +804,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="52" t="str">
-        <x:v>Sprint 1 | v0.2.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
+        <x:v>Sprint 1 | v0.3.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
       </x:c>
       <x:c r="B2" s="51"/>
       <x:c r="C2" s="51"/>
@@ -863,7 +863,7 @@
       </x:c>
       <x:c r="B6" s="59" t="n">
         <x:f>COUNTIF('Backlog'!$F$5:$F$65,"Done")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C6" s="51"/>
       <x:c r="D6" s="58" t="str">
@@ -960,7 +960,7 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="62" t="str">
-        <x:v>Aktiewe story: MCP-US-003 Minimal Safe Boot And USB Profile | HIL proof volg</x:v>
+        <x:v>Aktiewe story: MCP-US-051 Hardware-In-The-Loop Test Runner</x:v>
       </x:c>
       <x:c r="B13" s="51"/>
       <x:c r="C13" s="51"/>
@@ -1187,13 +1187,13 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="F7" s="24" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G7" s="24" t="str">
         <x:v>Sprint 1</x:v>
       </x:c>
       <x:c r="H7" s="24" t="str">
-        <x:v>In Progress/MVP</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I7" s="65" t="n">
         <x:v>8</x:v>
@@ -1202,10 +1202,10 @@
         <x:v>US-002</x:v>
       </x:c>
       <x:c r="K7" s="24" t="str">
-        <x:v>USB-MIDI begin voor runtime; bord-VID/PID bly verstek; CIRCUITPY/REPL herstel en drieledige device-proof slaag</x:v>
+        <x:v>USB-MIDI begin voor runtime; CIRCUITPY/REPL herstel en drieledige device-proof het op ESP32-S2 geslaag</x:v>
       </x:c>
       <x:c r="L7" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-003</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-003 / commit 3994f46</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="38" customHeight="1">
@@ -3011,13 +3011,13 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="F55" s="24" t="str">
-        <x:v>Backlog</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="G55" s="24" t="str">
-        <x:v>Release train</x:v>
+        <x:v>Sprint 1</x:v>
       </x:c>
       <x:c r="H55" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>In Progress/MVP</x:v>
       </x:c>
       <x:c r="I55" s="65" t="n">
         <x:v>5</x:v>
@@ -3026,10 +3026,10 @@
         <x:v>US-003, US-015</x:v>
       </x:c>
       <x:c r="K55" s="24" t="str">
-        <x:v>Connection, deploy en execution proof plus USB-MIDI en klankmeetstappe lewer 'n geredigeerde naspeurbare verslag</x:v>
+        <x:v>Connection/deploy/boot/execution-runner is groen; USB-MIDI bewys; klankmeting wag op US-015/016</x:v>
       </x:c>
       <x:c r="L55" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-051</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-051-IN-REVIEW</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="38" customHeight="1">
@@ -3441,7 +3441,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc104f2338ed64c8e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9656ca5643894423"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3505,7 +3505,7 @@
       </x:c>
       <x:c r="E5" s="64" t="n">
         <x:f>COUNTIFS('Backlog'!$B$5:$B$65,A5,'Backlog'!$F$5:$F$65,"Done")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F5" s="23" t="str">
         <x:v>Veilige, draagbare basis en konfigurasiegrens</x:v>
@@ -3679,7 +3679,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32f3f5c6ad854c21"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1596364ed85242d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4257,7 +4257,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b43652cb5f647c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3f34a4217444cb0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4431,7 +4431,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9889003f50674b16"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ff325af1a474206"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4715,7 +4715,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a00e1868f7f4e23"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8f3f988567f4c48"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add Wi-Fi station and AP fallback scope
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R7f934b418b894390"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R9a7473e9a57b46bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Rd84424c244d844a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R66e43e1e915b496a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R3faf841bc6b649af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R4c35feeb56314f52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rb2efe85f9cbd4749"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R49532a6b7ffe47f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Rdf74317939d84a63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="Rf5c1d196cb3948ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="Re57d9c22986c46f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R8df0036d754a48fd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -551,7 +551,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RisksTable" displayName="RisksTable" ref="A4:G29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RisksTable" displayName="RisksTable" ref="A4:G31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Risiko"/>
@@ -577,7 +577,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SourcesTable" displayName="SourcesTable" ref="A4:D25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SourcesTable" displayName="SourcesTable" ref="A4:D27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Bron"/>
     <x:tableColumn id="2" name="Gebruik"/>
@@ -807,7 +807,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="52" t="str">
-        <x:v>Sprint 1 | scope v0.4.0 | runtime v0.3.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
+        <x:v>Sprint 1 | scope v0.5.0 | runtime v0.3.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
       </x:c>
       <x:c r="B2" s="51"/>
       <x:c r="C2" s="51"/>
@@ -916,11 +916,13 @@
         <x:v>Oop risiko’s</x:v>
       </x:c>
       <x:c r="B9" s="59" t="n">
-        <x:f>COUNTIF('Risks'!$G$5:$G$29,"&lt;&gt;Closed")</x:f>
-        <x:v>25</x:v>
+        <x:f>COUNTIF('Risks'!$G$5:$G$31,"&lt;&gt;Closed")</x:f>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="C9" s="51"/>
-      <x:c r="D9" s="51"/>
+      <x:c r="D9" s="51" t="str">
+        <x:v>5. Station join met beveiligde AP-fallback; mobile UI en logging binne begroting</x:v>
+      </x:c>
       <x:c r="E9" s="51"/>
       <x:c r="F9" s="51"/>
       <x:c r="G9" s="51"/>
@@ -1941,7 +1943,7 @@
         <x:v>MCP-EPIC-004</x:v>
       </x:c>
       <x:c r="C27" s="24" t="str">
-        <x:v>Safe Wi-Fi Runtime Service</x:v>
+        <x:v>Safe Wi-Fi Station And AP Fallback Service</x:v>
       </x:c>
       <x:c r="D27" s="24" t="str">
         <x:v>Web Engineer</x:v>
@@ -1965,10 +1967,10 @@
         <x:v>US-005, US-022</x:v>
       </x:c>
       <x:c r="K27" s="24" t="str">
-        <x:v>Wi-Fi begin buite boot en gee ’n duidelike offline-modus</x:v>
+        <x:v>Runtime join 'n gekonfigureerde netwerk binne timeout en rapporteer station-IP; by mislukking begin 'n beveiligde AP en rapporteer AP-IP sonder MIDI-/klankblokkasie</x:v>
       </x:c>
       <x:c r="L27" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-023</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / WIFI-RUNTIME-AMENDMENT-001 / MCP-US-023</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="38" customHeight="1">
@@ -1979,7 +1981,7 @@
         <x:v>MCP-EPIC-004</x:v>
       </x:c>
       <x:c r="C28" s="24" t="str">
-        <x:v>Local Web Status And Parameters</x:v>
+        <x:v>Mobile-Friendly Local Web Status And Parameters</x:v>
       </x:c>
       <x:c r="D28" s="24" t="str">
         <x:v>Web Engineer</x:v>
@@ -2003,10 +2005,10 @@
         <x:v>US-023</x:v>
       </x:c>
       <x:c r="K28" s="24" t="str">
-        <x:v>Een plaaslike kliënt kan status lees en veilige parameters verander</x:v>
+        <x:v>Een mobiele plaaslike klient lees status en verander veilige parameters in station/AP-modus; polling en logging bly spaarsaam en koersbegrens</x:v>
       </x:c>
       <x:c r="L28" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-024</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / WIFI-RUNTIME-AMENDMENT-001 / MCP-US-024</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="38" customHeight="1">
@@ -2117,10 +2119,10 @@
         <x:v>US-024</x:v>
       </x:c>
       <x:c r="K31" s="24" t="str">
-        <x:v>Vertroude-LAN-grens, sessielimiet en herstelpad is getoets</x:v>
+        <x:v>Vertroude-LAN/AP-grens, private credentials, sessielimiet, netwerkafskakeling en herstelpad is getoets</x:v>
       </x:c>
       <x:c r="L31" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-027</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / WIFI-RUNTIME-AMENDMENT-001 / MCP-US-027</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="38" customHeight="1">
@@ -3526,7 +3528,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fcd065b88be4856"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1300f31f2214263"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3662,7 +3664,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F8" s="24" t="str">
-        <x:v>Plaaslike webbeheer en eenvoudige performance tools</x:v>
+        <x:v>Mobile-first webbeheer, station-IP, beveiligde AP-fallback en recovery</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="32" customHeight="1">
@@ -3764,7 +3766,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59263cba85894f0a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8b44bac04f54ea3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3789,7 +3791,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>25 aktiewe risiko's; blockers bly sigbaar en firmwarebewys word van hosttooling onderskei</x:v>
+        <x:v>27 aktiewe risiko's; Wi-Fi-fallback en logging bly begrens sonder om real-time klank te verberg</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -4387,6 +4389,52 @@
         <x:v>Preflight poorte; een REPL-klient; timeout, cleanup en herstelpad</x:v>
       </x:c>
       <x:c r="G29" s="83" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="52" customHeight="1">
+      <x:c r="A30" s="83" t="str">
+        <x:v>R-026</x:v>
+      </x:c>
+      <x:c r="B30" s="83" t="str">
+        <x:v>Fallback access point is oop, voorspelbaar of lek credentials/klientidentiteit</x:v>
+      </x:c>
+      <x:c r="C30" s="83" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="D30" s="83" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="E30" s="83" t="str">
+        <x:v>Security/Web</x:v>
+      </x:c>
+      <x:c r="F30" s="83" t="str">
+        <x:v>Beveiligde AP; private provisioning; geen geheime, MAC's of unieke ID's in logs/repo</x:v>
+      </x:c>
+      <x:c r="G30" s="83" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="52" customHeight="1">
+      <x:c r="A31" s="83" t="str">
+        <x:v>R-027</x:v>
+      </x:c>
+      <x:c r="B31" s="83" t="str">
+        <x:v>Onbegrensde join/reconnect, HTTP polling of debuglogging veroorsaak dropout, RAM-druk of flashslytasie</x:v>
+      </x:c>
+      <x:c r="C31" s="83" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="D31" s="83" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E31" s="83" t="str">
+        <x:v>Embedded/Web/QA</x:v>
+      </x:c>
+      <x:c r="F31" s="83" t="str">
+        <x:v>Timeout/backoff; cooperative poll; een klient; debug af; koersbegrensde serial logging; geen normale flashlog</x:v>
+      </x:c>
+      <x:c r="G31" s="83" t="str">
         <x:v>Open</x:v>
       </x:c>
     </x:row>
@@ -4401,7 +4449,7 @@
   <x:conditionalFormatting sqref="G5:G22">
     <x:cfRule type="containsText" dxfId="5" priority="2" operator="containsText" text="Closed"/>
   </x:conditionalFormatting>
-  <x:dataValidations count="3">
+  <x:dataValidations count="4">
     <x:dataValidation type="list" sqref="G5:G22">
       <x:formula1>"Open,Open - human action,Controlled,Closed"</x:formula1>
     </x:dataValidation>
@@ -4411,10 +4459,13 @@
     <x:dataValidation type="list" sqref="G27:G29">
       <x:formula1>"Open,Controlled,Closed,Open - human action,Open - host impediment"</x:formula1>
     </x:dataValidation>
+    <x:dataValidation type="list" sqref="G30:G31">
+      <x:formula1>"Open,Controlled,Closed,Open - human action,Open - host impediment"</x:formula1>
+    </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R692321d367e54e0f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Race08dc751e245b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4588,7 +4639,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69b9c7dfc5ca4a9e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb1a6529c66aa4743"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4921,6 +4972,34 @@
         <x:v>https://documentation.espressif.com/esp32-s2_datasheet_en.html</x:v>
       </x:c>
     </x:row>
+    <x:row r="26" ht="40" customHeight="1">
+      <x:c r="A26" s="83" t="str">
+        <x:v>CircuitPython wifi</x:v>
+      </x:c>
+      <x:c r="B26" s="83" t="str">
+        <x:v>Station/AP, connect timeout, IP-adresse, AP-auth en DHCP</x:v>
+      </x:c>
+      <x:c r="C26" s="83" t="str">
+        <x:v>Official API</x:v>
+      </x:c>
+      <x:c r="D26" s="83" t="str">
+        <x:v>https://docs.circuitpython.org/en/stable/shared-bindings/wifi/</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="40" customHeight="1">
+      <x:c r="A27" s="83" t="str">
+        <x:v>HTTP server starting methods</x:v>
+      </x:c>
+      <x:c r="B27" s="83" t="str">
+        <x:v>Station- en AP-bedieneropstart</x:v>
+      </x:c>
+      <x:c r="C27" s="83" t="str">
+        <x:v>Official library example</x:v>
+      </x:c>
+      <x:c r="D27" s="83" t="str">
+        <x:v>https://docs.circuitpython.org/projects/httpserver/en/latest/starting_methods.html</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>
@@ -4928,7 +5007,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60bfdda777b54386"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd080a18d380a45fe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: close board capability discovery
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rf8ea33ce5d1c4875"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R218347a9a4ce4b36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Ra5aed93ce89b4521"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="Re6f121bba1ad469a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R0f24e0d0a64f47fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R0618949d4d274095"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R2dcfbe8b5c3d4b51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R85d44ce4b2524601"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="R3e87258fb5a04a0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R8da382a09fb049da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R12795d56fdab4869"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Ra088883ddf734562"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -866,7 +866,7 @@
       </x:c>
       <x:c r="B6" s="59" t="n">
         <x:f>COUNTIF('Backlog'!$F$5:$F$67,"Done")</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C6" s="51"/>
       <x:c r="D6" s="58" t="str">
@@ -965,7 +965,7 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="62" t="str">
-        <x:v>Aktiewe story: MCP-US-004 Board Capability Discovery - IMPEDIMENT</x:v>
+        <x:v>Laaste story: MCP-US-004 Board Capability Discovery - DONE | Volgende plan: MCP-US-005</x:v>
       </x:c>
       <x:c r="B13" s="51"/>
       <x:c r="C13" s="51"/>
@@ -1230,13 +1230,13 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="F8" s="24" t="str">
-        <x:v>Impediment</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G8" s="24" t="str">
         <x:v>Sprint 1</x:v>
       </x:c>
       <x:c r="H8" s="24" t="str">
-        <x:v>In Review/MVP</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I8" s="65" t="n">
         <x:v>5</x:v>
@@ -1245,7 +1245,7 @@
         <x:v>US-002</x:v>
       </x:c>
       <x:c r="K8" s="24" t="str">
-        <x:v>Host en sagte device-run rapporteer IO3/5/7, modules, heap en I2S-backend; finale hard-reset/remount-HIL wag</x:v>
+        <x:v>Profiel, IO3/5/7, modules, heap en I2S-backend gerapporteer; power-cycle recovery en volledige manifest-HIL slaag</x:v>
       </x:c>
       <x:c r="L8" s="24" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-004 / v0.4.0</x:v>
@@ -3531,7 +3531,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c96d68be8d0425f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8900d60e7f244e59"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3595,7 +3595,7 @@
       </x:c>
       <x:c r="E5" s="64" t="n">
         <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A5,'Backlog'!$F$5:$F$67,"Done")</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F5" s="23" t="str">
         <x:v>Veilige, draagbare basis en konfigurasiegrens</x:v>
@@ -3769,7 +3769,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75f6590912004891"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd951ab071a994e17"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3794,7 +3794,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>28 aktiewe risiko's; MCP-US-004 is geblokkeer op USB-remount ná programmatiese harde reset</x:v>
+        <x:v>28 geregistreerde risiko's; USB-remount recovery en finale MCP-US-004 HIL is bewys</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -4446,7 +4446,7 @@
         <x:v>R-028</x:v>
       </x:c>
       <x:c r="B32" s="83" t="str">
-        <x:v>Programmatiese harde reset laat USB sonder CIRCUITPY/CDC-herenumerasie</x:v>
+        <x:v>Programmatiese harde reset laat USB soms sonder CIRCUITPY/CDC-herenumerasie</x:v>
       </x:c>
       <x:c r="C32" s="83" t="str">
         <x:v>Medium</x:v>
@@ -4458,10 +4458,10 @@
         <x:v>Embedded/QA</x:v>
       </x:c>
       <x:c r="F32" s="83" t="str">
-        <x:v>Fisiese power-cycle; recovery-runbook; blokkeer story tot volume, REPL, bootbanner en manifest-HIL herstel</x:v>
+        <x:v>Fisiese power-cycle herstel volume/REPL; recovery-runbook en finale manifest-HIL is bewys</x:v>
       </x:c>
       <x:c r="G32" s="83" t="str">
-        <x:v>Open - US-004 impediment</x:v>
+        <x:v>Controlled</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4491,7 +4491,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra803290166854d9f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08ff766698044342"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4665,7 +4665,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a9a1fadc3dd464f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e1b00e735924afa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5061,7 +5061,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ae7da3a3867460a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd19308a66a254192"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add secure configuration boundary
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R2dcfbe8b5c3d4b51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R85d44ce4b2524601"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="R3e87258fb5a04a0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R8da382a09fb049da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R12795d56fdab4869"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Ra088883ddf734562"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R7308f0edb2d74e88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R3b30b349cab9411b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="R23711705e4f14c13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R86df995858714671"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="Rbef155a616d94749"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Raaca484ddefb47ee"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -551,7 +551,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RisksTable" displayName="RisksTable" ref="A4:G32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="RisksTable" displayName="RisksTable" ref="A4:G33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Risiko"/>
@@ -577,7 +577,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SourcesTable" displayName="SourcesTable" ref="A4:D29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SourcesTable" displayName="SourcesTable" ref="A4:D32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Bron"/>
     <x:tableColumn id="2" name="Gebruik"/>
@@ -807,7 +807,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="52" t="str">
-        <x:v>Sprint 1 | scope v0.6.0 | runtime v0.4.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
+        <x:v>Sprint 1 | scope v0.7.0 | runtime v0.5.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
       </x:c>
       <x:c r="B2" s="51"/>
       <x:c r="C2" s="51"/>
@@ -916,8 +916,8 @@
         <x:v>Oop risiko’s</x:v>
       </x:c>
       <x:c r="B9" s="59" t="n">
-        <x:f>COUNTA('Risks'!A5:A32)</x:f>
-        <x:v>28</x:v>
+        <x:f>COUNTA('Risks'!A5:A33)</x:f>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C9" s="51"/>
       <x:c r="D9" s="51" t="str">
@@ -965,7 +965,7 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="62" t="str">
-        <x:v>Laaste story: MCP-US-004 Board Capability Discovery - DONE | Volgende plan: MCP-US-005</x:v>
+        <x:v>Aktiewe story: MCP-US-005 Configuration And Secret Boundary - IN REVIEW / HIL HEK | Volgende goedgekeur: MCP-US-006</x:v>
       </x:c>
       <x:c r="B13" s="51"/>
       <x:c r="C13" s="51"/>
@@ -1268,13 +1268,13 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="F9" s="24" t="str">
-        <x:v>Backlog</x:v>
+        <x:v>In Review</x:v>
       </x:c>
       <x:c r="G9" s="24" t="str">
         <x:v>Sprint 1</x:v>
       </x:c>
       <x:c r="H9" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>In Review</x:v>
       </x:c>
       <x:c r="I9" s="65" t="n">
         <x:v>5</x:v>
@@ -1283,10 +1283,10 @@
         <x:v>US-003</x:v>
       </x:c>
       <x:c r="K9" s="24" t="str">
-        <x:v>Publieke verstekke en private `settings.toml` werk; geheime-lektoets is groen</x:v>
+        <x:v>Publieke verstekke, private settings en override-prioriteit is host-groen; toestel-deploy wag op leesalleen-volume herstel</x:v>
       </x:c>
       <x:c r="L9" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-005</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-005 / v0.5.0</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="38" customHeight="1">
@@ -3531,7 +3531,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8900d60e7f244e59"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d0e384996744ebe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3769,7 +3769,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd951ab071a994e17"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f6d8c27ae934071"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3794,7 +3794,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>28 geregistreerde risiko's; USB-remount recovery en finale MCP-US-004 HIL is bewys</x:v>
+        <x:v>29 geregistreerde risiko's; US-005 deploy is veilig gestop by 'n leesalleen CIRCUITPY-volume</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -4462,6 +4462,29 @@
       </x:c>
       <x:c r="G32" s="83" t="str">
         <x:v>Controlled</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" t="str">
+        <x:v>R-029</x:v>
+      </x:c>
+      <x:c r="B33" t="str">
+        <x:v>CIRCUITPY-media is geldig maar leesalleen vir die host</x:v>
+      </x:c>
+      <x:c r="C33" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="D33" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E33" t="str">
+        <x:v>Embedded/Release</x:v>
+      </x:c>
+      <x:c r="F33" t="str">
+        <x:v>Stop deploy; FAT verify; fisiese power-cycle en skryfbaarheidstoets; geen erase/remount-omseiling</x:v>
+      </x:c>
+      <x:c r="G33" t="str">
+        <x:v>Open - US-005 HIL gate</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4491,7 +4514,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08ff766698044342"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5069b2e9db50474c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4665,7 +4688,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e1b00e735924afa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d5549a2d8744cb1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5054,6 +5077,48 @@
         <x:v>https://docs.espressif.com/projects/esp-idf/en/release-v5.2/esp32s2/api-reference/peripherals/i2s.html</x:v>
       </x:c>
     </x:row>
+    <x:row r="30">
+      <x:c r="A30" t="str">
+        <x:v>CircuitPython environment variables</x:v>
+      </x:c>
+      <x:c r="B30" t="str">
+        <x:v>settings.toml en os.getenv</x:v>
+      </x:c>
+      <x:c r="C30" t="str">
+        <x:v>Official API guide</x:v>
+      </x:c>
+      <x:c r="D30" t="str">
+        <x:v>https://docs.circuitpython.org/en/latest/docs/environment.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" t="str">
+        <x:v>CircuitPython storage workflow</x:v>
+      </x:c>
+      <x:c r="B31" t="str">
+        <x:v>Host/device filesystem ownership</x:v>
+      </x:c>
+      <x:c r="C31" t="str">
+        <x:v>Official workflow</x:v>
+      </x:c>
+      <x:c r="D31" t="str">
+        <x:v>https://docs.circuitpython.org/en/10.1.1/docs/workflows.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" t="str">
+        <x:v>CircuitPython storage API</x:v>
+      </x:c>
+      <x:c r="B32" t="str">
+        <x:v>Remount en destructive erase boundary</x:v>
+      </x:c>
+      <x:c r="C32" t="str">
+        <x:v>Official API</x:v>
+      </x:c>
+      <x:c r="D32" t="str">
+        <x:v>https://docs.circuitpython.org/en/10.0.3/shared-bindings/storage/</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>
@@ -5061,7 +5126,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd19308a66a254192"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6842426992084afb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add portable MIDI event model
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R7308f0edb2d74e88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R3b30b349cab9411b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="R23711705e4f14c13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R86df995858714671"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="Rbef155a616d94749"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Raaca484ddefb47ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rc98236d4d4bd4f43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R1033548ef4544838"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Re367758b5bca48b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R0ac69ad9eaab444d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R7af068346dd94d37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R0b640df49e454752"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21,7 +21,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="18">
+  <x:fonts count="24">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -120,8 +120,41 @@
       <x:color rgb="FF9B2C2C"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF243746"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF243746"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF243746"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="20"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF58728A"/>
+      <x:name val="Aptos"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="11">
+  <x:fills count="18">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -171,6 +204,41 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFCE1D2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF12324A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF4F7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1B7288"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE6F1F4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF26B5E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4F8FA"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -245,7 +313,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="84">
+  <x:cellXfs count="125">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -440,6 +508,111 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="4" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="20" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="14" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="14" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="14" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="15" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="15" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="15" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="17" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="17" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -577,7 +750,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SourcesTable" displayName="SourcesTable" ref="A4:D32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SourcesTable" displayName="SourcesTable" ref="A4:D33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="Bron"/>
     <x:tableColumn id="2" name="Gebruik"/>
@@ -794,218 +967,218 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
-      <x:c r="A1" s="50" t="str">
+      <x:c r="A1" s="100" t="str">
         <x:v>MIDI Chip Platform - MVP Kanban</x:v>
       </x:c>
-      <x:c r="B1" s="51"/>
-      <x:c r="C1" s="51"/>
-      <x:c r="D1" s="51"/>
-      <x:c r="E1" s="51"/>
-      <x:c r="F1" s="51"/>
-      <x:c r="G1" s="51"/>
-      <x:c r="H1" s="51"/>
+      <x:c r="B1" s="101"/>
+      <x:c r="C1" s="101"/>
+      <x:c r="D1" s="101"/>
+      <x:c r="E1" s="101"/>
+      <x:c r="F1" s="101"/>
+      <x:c r="G1" s="101"/>
+      <x:c r="H1" s="101"/>
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
-      <x:c r="A2" s="52" t="str">
-        <x:v>Sprint 1 | scope v0.7.0 | runtime v0.5.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
-      </x:c>
-      <x:c r="B2" s="51"/>
-      <x:c r="C2" s="51"/>
-      <x:c r="D2" s="51"/>
-      <x:c r="E2" s="51"/>
-      <x:c r="F2" s="51"/>
-      <x:c r="G2" s="51"/>
-      <x:c r="H2" s="51"/>
+      <x:c r="A2" s="102" t="str">
+        <x:v>Sprint 2 | scope v0.8.0 | runtime v0.6.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
+      </x:c>
+      <x:c r="B2" s="103"/>
+      <x:c r="C2" s="103"/>
+      <x:c r="D2" s="103"/>
+      <x:c r="E2" s="103"/>
+      <x:c r="F2" s="103"/>
+      <x:c r="G2" s="103"/>
+      <x:c r="H2" s="103"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="51"/>
-      <x:c r="B3" s="51"/>
-      <x:c r="C3" s="51"/>
-      <x:c r="D3" s="51"/>
-      <x:c r="E3" s="51"/>
-      <x:c r="F3" s="51"/>
-      <x:c r="G3" s="51"/>
-      <x:c r="H3" s="51"/>
+      <x:c r="A3" s="85"/>
+      <x:c r="B3" s="85"/>
+      <x:c r="C3" s="85"/>
+      <x:c r="D3" s="85"/>
+      <x:c r="E3" s="85"/>
+      <x:c r="F3" s="85"/>
+      <x:c r="G3" s="85"/>
+      <x:c r="H3" s="85"/>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="53" t="str">
+      <x:c r="A4" s="106" t="str">
         <x:v>Metriek</x:v>
       </x:c>
-      <x:c r="B4" s="54" t="str">
+      <x:c r="B4" s="107" t="str">
         <x:v>Waarde</x:v>
       </x:c>
-      <x:c r="C4" s="51"/>
-      <x:c r="D4" s="53" t="str">
+      <x:c r="C4" s="85"/>
+      <x:c r="D4" s="106" t="str">
         <x:v>MVP-besluithekke</x:v>
       </x:c>
-      <x:c r="E4" s="55"/>
-      <x:c r="F4" s="55"/>
-      <x:c r="G4" s="55"/>
-      <x:c r="H4" s="54"/>
+      <x:c r="E4" s="109"/>
+      <x:c r="F4" s="109"/>
+      <x:c r="G4" s="109"/>
+      <x:c r="H4" s="107"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="56" t="str">
+      <x:c r="A5" s="110" t="str">
         <x:v>Totale stories</x:v>
       </x:c>
-      <x:c r="B5" s="57" t="n">
+      <x:c r="B5" s="113" t="n">
         <x:f>COUNTA('Backlog'!$A$5:$A$67)</x:f>
         <x:v>63</x:v>
       </x:c>
-      <x:c r="C5" s="51"/>
-      <x:c r="D5" s="56" t="str">
+      <x:c r="C5" s="85"/>
+      <x:c r="D5" s="110" t="str">
         <x:v>1. Veilige minimale USB-MIDI boot en herstel</x:v>
       </x:c>
-      <x:c r="E5" s="56"/>
-      <x:c r="F5" s="56"/>
-      <x:c r="G5" s="56"/>
-      <x:c r="H5" s="56"/>
+      <x:c r="E5" s="110"/>
+      <x:c r="F5" s="110"/>
+      <x:c r="G5" s="110"/>
+      <x:c r="H5" s="110"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="58" t="str">
+      <x:c r="A6" s="111" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="B6" s="59" t="n">
+      <x:c r="B6" s="114" t="n">
         <x:f>COUNTIF('Backlog'!$F$5:$F$67,"Done")</x:f>
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C6" s="51"/>
-      <x:c r="D6" s="58" t="str">
+      <x:c r="C6" s="85"/>
+      <x:c r="D6" s="111" t="str">
         <x:v>2. MAX98357 mono-I2S eerste; PWM fallback</x:v>
       </x:c>
-      <x:c r="E6" s="58"/>
-      <x:c r="F6" s="58"/>
-      <x:c r="G6" s="58"/>
-      <x:c r="H6" s="58"/>
+      <x:c r="E6" s="111"/>
+      <x:c r="F6" s="111"/>
+      <x:c r="G6" s="111"/>
+      <x:c r="H6" s="111"/>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="58" t="str">
+      <x:c r="A7" s="111" t="str">
         <x:v>In Progress</x:v>
       </x:c>
-      <x:c r="B7" s="59" t="n">
+      <x:c r="B7" s="114" t="n">
         <x:f>COUNTIF('Backlog'!$F$5:$F$67,"In Progress")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C7" s="51"/>
-      <x:c r="D7" s="58" t="str">
+      <x:c r="C7" s="85"/>
+      <x:c r="D7" s="111" t="str">
         <x:v>3. D1-basiskern voor SN76489; SID en OPL daarna</x:v>
       </x:c>
-      <x:c r="E7" s="58"/>
-      <x:c r="F7" s="58"/>
-      <x:c r="G7" s="58"/>
-      <x:c r="H7" s="58"/>
+      <x:c r="E7" s="111"/>
+      <x:c r="F7" s="111"/>
+      <x:c r="G7" s="111"/>
+      <x:c r="H7" s="111"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="58" t="str">
+      <x:c r="A8" s="111" t="str">
         <x:v>MVP-gemerk</x:v>
       </x:c>
-      <x:c r="B8" s="59" t="n">
+      <x:c r="B8" s="114" t="n">
         <x:f>COUNTIF('Backlog'!$E$5:$E$67,"Must")</x:f>
         <x:v>47</x:v>
       </x:c>
-      <x:c r="C8" s="51"/>
-      <x:c r="D8" s="60" t="str">
+      <x:c r="C8" s="85"/>
+      <x:c r="D8" s="112" t="str">
         <x:v>4. BLE op tweede bord; S2 faal veilig; multi-core na resource gate</x:v>
       </x:c>
-      <x:c r="E8" s="60"/>
-      <x:c r="F8" s="60"/>
-      <x:c r="G8" s="60"/>
-      <x:c r="H8" s="60"/>
+      <x:c r="E8" s="112"/>
+      <x:c r="F8" s="112"/>
+      <x:c r="G8" s="112"/>
+      <x:c r="H8" s="112"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="58" t="str">
+      <x:c r="A9" s="111" t="str">
         <x:v>Oop risiko’s</x:v>
       </x:c>
-      <x:c r="B9" s="59" t="n">
+      <x:c r="B9" s="114" t="n">
         <x:f>COUNTA('Risks'!A5:A33)</x:f>
         <x:v>29</x:v>
       </x:c>
-      <x:c r="C9" s="51"/>
-      <x:c r="D9" s="51" t="str">
+      <x:c r="C9" s="85"/>
+      <x:c r="D9" s="116" t="str">
         <x:v>5. Station join met beveiligde AP-fallback; mobile UI en logging binne begroting</x:v>
       </x:c>
-      <x:c r="E9" s="51"/>
-      <x:c r="F9" s="51"/>
-      <x:c r="G9" s="51"/>
-      <x:c r="H9" s="51"/>
+      <x:c r="E9" s="116"/>
+      <x:c r="F9" s="116"/>
+      <x:c r="G9" s="116"/>
+      <x:c r="H9" s="116"/>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="60" t="str">
+      <x:c r="A10" s="112" t="str">
         <x:v>Virtuele rolle</x:v>
       </x:c>
-      <x:c r="B10" s="61" t="n">
+      <x:c r="B10" s="115" t="n">
         <x:f>COUNTA('Team RACI'!$A$5:$A$16)</x:f>
         <x:v>12</x:v>
       </x:c>
-      <x:c r="C10" s="51"/>
-      <x:c r="D10" s="51"/>
-      <x:c r="E10" s="51"/>
-      <x:c r="F10" s="51"/>
-      <x:c r="G10" s="51"/>
-      <x:c r="H10" s="51"/>
+      <x:c r="C10" s="85"/>
+      <x:c r="D10" s="116"/>
+      <x:c r="E10" s="116"/>
+      <x:c r="F10" s="116"/>
+      <x:c r="G10" s="116"/>
+      <x:c r="H10" s="116"/>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="51"/>
-      <x:c r="B11" s="51"/>
-      <x:c r="C11" s="51"/>
-      <x:c r="D11" s="51"/>
-      <x:c r="E11" s="51"/>
-      <x:c r="F11" s="51"/>
-      <x:c r="G11" s="51"/>
-      <x:c r="H11" s="51"/>
+      <x:c r="A11" s="85"/>
+      <x:c r="B11" s="85"/>
+      <x:c r="C11" s="85"/>
+      <x:c r="D11" s="85"/>
+      <x:c r="E11" s="85"/>
+      <x:c r="F11" s="85"/>
+      <x:c r="G11" s="85"/>
+      <x:c r="H11" s="85"/>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="51"/>
-      <x:c r="B12" s="51"/>
-      <x:c r="C12" s="51"/>
-      <x:c r="D12" s="51"/>
-      <x:c r="E12" s="51"/>
-      <x:c r="F12" s="51"/>
-      <x:c r="G12" s="51"/>
-      <x:c r="H12" s="51"/>
+      <x:c r="A12" s="85"/>
+      <x:c r="B12" s="85"/>
+      <x:c r="C12" s="85"/>
+      <x:c r="D12" s="85"/>
+      <x:c r="E12" s="85"/>
+      <x:c r="F12" s="85"/>
+      <x:c r="G12" s="85"/>
+      <x:c r="H12" s="85"/>
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
-      <x:c r="A13" s="62" t="str">
-        <x:v>Aktiewe story: MCP-US-005 Configuration And Secret Boundary - IN REVIEW / HIL HEK | Volgende goedgekeur: MCP-US-006</x:v>
-      </x:c>
-      <x:c r="B13" s="51"/>
-      <x:c r="C13" s="51"/>
-      <x:c r="D13" s="51"/>
-      <x:c r="E13" s="51"/>
-      <x:c r="F13" s="51"/>
-      <x:c r="G13" s="51"/>
-      <x:c r="H13" s="51"/>
+      <x:c r="A13" s="119" t="str">
+        <x:v>Aktiewe story: MCP-US-006 Portable Event Model - IN REVIEW | US-005 HIL HEK OOP | Volgende plan: MCP-US-007</x:v>
+      </x:c>
+      <x:c r="B13" s="120"/>
+      <x:c r="C13" s="120"/>
+      <x:c r="D13" s="120"/>
+      <x:c r="E13" s="120"/>
+      <x:c r="F13" s="120"/>
+      <x:c r="G13" s="120"/>
+      <x:c r="H13" s="120"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="51"/>
-      <x:c r="B14" s="51"/>
-      <x:c r="C14" s="51"/>
-      <x:c r="D14" s="51"/>
-      <x:c r="E14" s="51"/>
-      <x:c r="F14" s="51"/>
-      <x:c r="G14" s="51"/>
-      <x:c r="H14" s="51"/>
+      <x:c r="A14" s="85"/>
+      <x:c r="B14" s="85"/>
+      <x:c r="C14" s="85"/>
+      <x:c r="D14" s="85"/>
+      <x:c r="E14" s="85"/>
+      <x:c r="F14" s="85"/>
+      <x:c r="G14" s="85"/>
+      <x:c r="H14" s="85"/>
     </x:row>
     <x:row r="15" ht="58" customHeight="1">
-      <x:c r="A15" s="63" t="str">
+      <x:c r="A15" s="123" t="str">
         <x:v>Product Owner note: hierdie workbook is die redigeerbare Kanban-artefak. Die Markdown story-katalogus bly die leesbare repository-weergawe. Werk begin eers ná story-plan-goedkeuring.</x:v>
       </x:c>
-      <x:c r="B15" s="51"/>
-      <x:c r="C15" s="51"/>
-      <x:c r="D15" s="51"/>
-      <x:c r="E15" s="51"/>
-      <x:c r="F15" s="51"/>
-      <x:c r="G15" s="51"/>
-      <x:c r="H15" s="51"/>
+      <x:c r="B15" s="124"/>
+      <x:c r="C15" s="124"/>
+      <x:c r="D15" s="124"/>
+      <x:c r="E15" s="124"/>
+      <x:c r="F15" s="124"/>
+      <x:c r="G15" s="124"/>
+      <x:c r="H15" s="124"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="51"/>
-      <x:c r="B16" s="51"/>
-      <x:c r="C16" s="51"/>
-      <x:c r="D16" s="51"/>
-      <x:c r="E16" s="51"/>
-      <x:c r="F16" s="51"/>
-      <x:c r="G16" s="51"/>
-      <x:c r="H16" s="51"/>
+      <x:c r="A16" s="124"/>
+      <x:c r="B16" s="124"/>
+      <x:c r="C16" s="124"/>
+      <x:c r="D16" s="124"/>
+      <x:c r="E16" s="124"/>
+      <x:c r="F16" s="124"/>
+      <x:c r="G16" s="124"/>
+      <x:c r="H16" s="124"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="51"/>
@@ -1306,13 +1479,13 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="F10" s="24" t="str">
-        <x:v>Backlog</x:v>
+        <x:v>In Review</x:v>
       </x:c>
       <x:c r="G10" s="24" t="str">
         <x:v>Sprint 2</x:v>
       </x:c>
       <x:c r="H10" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>In Review</x:v>
       </x:c>
       <x:c r="I10" s="65" t="n">
         <x:v>5</x:v>
@@ -1321,10 +1494,10 @@
         <x:v>US-002</x:v>
       </x:c>
       <x:c r="K10" s="24" t="str">
-        <x:v>Note, CC, bend en klokboodskappe het platform-onafhanklike klasse</x:v>
+        <x:v>Note, CC, 14-bit bend en kanaallose clock gebruik backend-onafhanklike klasse; 49 hosttoetse en events-diagnose is groen</x:v>
       </x:c>
       <x:c r="L10" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-006</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-006 / v0.6.0</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="38" customHeight="1">
@@ -3531,7 +3704,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d0e384996744ebe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3e3d764672a4cc1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3769,7 +3942,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f6d8c27ae934071"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf5bb9abc139478f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4514,7 +4687,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5069b2e9db50474c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc717d7f66f84f60"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4688,7 +4861,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d5549a2d8744cb1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47293a240c0d4c6c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5119,6 +5292,20 @@
         <x:v>https://docs.circuitpython.org/en/10.0.3/shared-bindings/storage/</x:v>
       </x:c>
     </x:row>
+    <x:row r="33">
+      <x:c r="A33" t="str">
+        <x:v>MIDI Association MIDI 1.0 summary</x:v>
+      </x:c>
+      <x:c r="B33" t="str">
+        <x:v>Channel messages, 14-bit bend and timing clock</x:v>
+      </x:c>
+      <x:c r="C33" t="str">
+        <x:v>Official standards body</x:v>
+      </x:c>
+      <x:c r="D33" t="str">
+        <x:v>https://midi.org/summary-of-midi-1-0-messages</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>
@@ -5126,7 +5313,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6842426992084afb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b01c456ef54445b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(framework): close USB MIDI HIL and add governance baseline
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rcc9bd9a0a564457f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="Rb10292f5dbf047d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Rd6d22c8563f146ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R21affbb057004ce8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R6880bb6d41534f4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rb401ff9078fa42d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rb8e38f804be04039"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="Rcf916219bc8641a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Rc7a906f9c37e435e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R1b532a9c79824ae0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R499be382f72846de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Re63355a4f39d49fe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -154,7 +154,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="18">
+  <x:fills count="22">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -241,6 +241,26 @@
         <x:fgColor rgb="FFF4F8FA"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFBFE5F4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFBCEFC6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF80C6E3"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="8">
     <x:border/>
@@ -313,7 +333,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="125">
+  <x:cellXfs count="137">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -613,6 +633,42 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="23" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="21" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="19" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="21" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="21" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -980,7 +1036,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="102" t="str">
-        <x:v>Sprint 2 | scope v0.15.0 | runtime v0.11.1 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
+        <x:v>Sprint 2 | scope v0.16.0 | runtime v0.12.2 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
       </x:c>
       <x:c r="B2" s="103"/>
       <x:c r="C2" s="103"/>
@@ -1021,8 +1077,8 @@
         <x:v>Totale stories</x:v>
       </x:c>
       <x:c r="B5" s="113" t="n">
-        <x:f>COUNTA('Backlog'!$A$5:$A$67)</x:f>
-        <x:v>63</x:v>
+        <x:f>COUNTA('Backlog'!$A$5:$A$200)</x:f>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="C5" s="85"/>
       <x:c r="D5" s="110" t="str">
@@ -1038,8 +1094,8 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B6" s="114" t="n">
-        <x:f>COUNTIF('Backlog'!$F$5:$F$67,"Done")</x:f>
-        <x:v>7</x:v>
+        <x:f>COUNTIF('Backlog'!$F$5:$F$200,"Done")</x:f>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C6" s="85"/>
       <x:c r="D6" s="111" t="str">
@@ -1055,7 +1111,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="B7" s="114" t="n">
-        <x:f>COUNTIF('Backlog'!$F$5:$F$67,"In Progress")</x:f>
+        <x:f>COUNTIF('Backlog'!$F$5:$F$200,"In Progress")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C7" s="85"/>
@@ -1072,8 +1128,8 @@
         <x:v>MVP-gemerk</x:v>
       </x:c>
       <x:c r="B8" s="114" t="n">
-        <x:f>COUNTIF('Backlog'!$E$5:$E$67,"Must")</x:f>
-        <x:v>47</x:v>
+        <x:f>COUNTIF('Backlog'!$E$5:$E$200,"Must")</x:f>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="C8" s="85"/>
       <x:c r="D8" s="112" t="str">
@@ -1089,8 +1145,8 @@
         <x:v>Oop risiko’s</x:v>
       </x:c>
       <x:c r="B9" s="114" t="n">
-        <x:f>COUNTA('Risks'!A5:A33)</x:f>
-        <x:v>29</x:v>
+        <x:f>COUNTA('Risks'!$A$5:$A$200)</x:f>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="C9" s="85"/>
       <x:c r="D9" s="116" t="str">
@@ -1106,8 +1162,8 @@
         <x:v>Virtuele rolle</x:v>
       </x:c>
       <x:c r="B10" s="115" t="n">
-        <x:f>COUNTA('Team RACI'!$A$5:$A$16)</x:f>
-        <x:v>12</x:v>
+        <x:f>COUNTA('Team RACI'!$A$5:$A$100)</x:f>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C10" s="85"/>
       <x:c r="D10" s="116"/>
@@ -1138,7 +1194,7 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="119" t="str">
-        <x:v>82 tests GREEN | Wemos HIL: closure, 16 hashes, libraries, boot en imports PASS | USB-note/klank/BLE bly oop</x:v>
+        <x:v>89 tests GREEN | Wemos HIL: closure, libraries, boot, imports en USB Note On/Off PASS | audio/BLE bly oop</x:v>
       </x:c>
       <x:c r="B13" s="120"/>
       <x:c r="C13" s="120"/>
@@ -1160,7 +1216,7 @@
     </x:row>
     <x:row r="15" ht="58" customHeight="1">
       <x:c r="A15" s="123" t="str">
-        <x:v>Product Owner note 2026-07-15: QA-herstel goedgekeur. Dependency-closed device proof PASS; US-007 Note On/Off bly oop.</x:v>
+        <x:v>Product Owner note 2026-07-15: MCP-US-007 aanvaar; matched USB-MIDI Note On/Off op S2 Mini. Framework Engineering baseline bygevoeg.</x:v>
       </x:c>
       <x:c r="B15" s="124"/>
       <x:c r="C15" s="124"/>
@@ -1201,6 +1257,7 @@
     <x:mergeCell ref="D8:H8"/>
     <x:mergeCell ref="A13:H13"/>
     <x:mergeCell ref="A15:H17"/>
+    <x:mergeCell ref="A15:H15"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1231,7 +1288,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Bron: docs/user_stories_v0.1.0.md | 63 stories | Redigeer Status en Priority via keuselyste</x:v>
+        <x:v>Bron: docs/user_stories_v0.1.0.md | 68 stories | Redigeer Status en Priority via keuselyste</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -1517,13 +1574,13 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="F11" s="24" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G11" s="24" t="str">
         <x:v>Sprint 2</x:v>
       </x:c>
       <x:c r="H11" s="24" t="str">
-        <x:v>Host accepted / HIL pending</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="I11" s="65" t="n">
         <x:v>5</x:v>
@@ -1532,10 +1589,10 @@
         <x:v>US-003, US-006</x:v>
       </x:c>
       <x:c r="K11" s="24" t="str">
-        <x:v>Dependency-closed device deploy, harde boot en clean imports is fisies groen; werklike USB-MIDI Note On/Off bly oop</x:v>
+        <x:v>v0.12.2 ontvang fisies USB-MIDI vanaf Logic/CoreMIDI; twee Note On, een Note Off en matched_notes=1 is op die Wemos S2 gerapporteer</x:v>
       </x:c>
       <x:c r="L11" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-051-IMP-001 / v0.11.1</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-007-ACCEPTANCE / v0.12.2</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="38" customHeight="1">
@@ -3664,6 +3721,196 @@
       </x:c>
       <x:c r="L67" s="83" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / SCOPE-AMENDMENT-002 / MCP-US-063</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="48" customHeight="1">
+      <x:c r="A68" s="126" t="str">
+        <x:v>MCP-US-064</x:v>
+      </x:c>
+      <x:c r="B68" s="126" t="str">
+        <x:v>MCP-EPIC-009</x:v>
+      </x:c>
+      <x:c r="C68" s="126" t="str">
+        <x:v>Enterprise Vision And Architecture Baseline</x:v>
+      </x:c>
+      <x:c r="D68" s="126" t="str">
+        <x:v>Chief Enterprise Architect</x:v>
+      </x:c>
+      <x:c r="E68" s="126" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="F68" s="126" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="G68" s="126" t="str">
+        <x:v>Sprint 2</x:v>
+      </x:c>
+      <x:c r="H68" s="126" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="I68" s="126" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J68" s="126" t="str">
+        <x:v>US-001, US-002</x:v>
+      </x:c>
+      <x:c r="K68" s="126" t="str">
+        <x:v>Enterprise vision plus framework, solution and deployment architecture form one cross-linked baseline</x:v>
+      </x:c>
+      <x:c r="L68" s="126" t="str">
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / FRAMEWORK-ENGINEERING-001 / MCP-US-064</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="48" customHeight="1">
+      <x:c r="A69" s="127" t="str">
+        <x:v>MCP-US-065</x:v>
+      </x:c>
+      <x:c r="B69" s="127" t="str">
+        <x:v>MCP-EPIC-009</x:v>
+      </x:c>
+      <x:c r="C69" s="127" t="str">
+        <x:v>Enterprise Meta Model, Glossary And Artefact Taxonomy</x:v>
+      </x:c>
+      <x:c r="D69" s="127" t="str">
+        <x:v>Framework Engineer</x:v>
+      </x:c>
+      <x:c r="E69" s="127" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="F69" s="127" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="G69" s="127" t="str">
+        <x:v>Sprint 2</x:v>
+      </x:c>
+      <x:c r="H69" s="127" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="I69" s="127" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J69" s="127" t="str">
+        <x:v>US-064</x:v>
+      </x:c>
+      <x:c r="K69" s="127" t="str">
+        <x:v>Roles, stories, components, tests, risks and decisions have named relationships and owners</x:v>
+      </x:c>
+      <x:c r="L69" s="127" t="str">
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / FRAMEWORK-ENGINEERING-001 / MCP-US-065</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70" ht="48" customHeight="1">
+      <x:c r="A70" s="126" t="str">
+        <x:v>MCP-US-066</x:v>
+      </x:c>
+      <x:c r="B70" s="126" t="str">
+        <x:v>MCP-EPIC-009</x:v>
+      </x:c>
+      <x:c r="C70" s="126" t="str">
+        <x:v>Quality Manual, Test Strategy And Review Engine</x:v>
+      </x:c>
+      <x:c r="D70" s="126" t="str">
+        <x:v>QA/Release</x:v>
+      </x:c>
+      <x:c r="E70" s="126" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="F70" s="126" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="G70" s="126" t="str">
+        <x:v>Sprint 2</x:v>
+      </x:c>
+      <x:c r="H70" s="126" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="I70" s="126" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J70" s="126" t="str">
+        <x:v>US-064, US-065</x:v>
+      </x:c>
+      <x:c r="K70" s="126" t="str">
+        <x:v>Definition of Done points to repeatable quality, test and review gates without treating docs as proof</x:v>
+      </x:c>
+      <x:c r="L70" s="126" t="str">
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / FRAMEWORK-ENGINEERING-001 / MCP-US-066</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="48" customHeight="1">
+      <x:c r="A71" s="127" t="str">
+        <x:v>MCP-US-067</x:v>
+      </x:c>
+      <x:c r="B71" s="127" t="str">
+        <x:v>MCP-EPIC-009</x:v>
+      </x:c>
+      <x:c r="C71" s="127" t="str">
+        <x:v>Prompt Compiler, Context Loader And Knowledge Base Structure</x:v>
+      </x:c>
+      <x:c r="D71" s="127" t="str">
+        <x:v>Framework Engineer</x:v>
+      </x:c>
+      <x:c r="E71" s="127" t="str">
+        <x:v>Should</x:v>
+      </x:c>
+      <x:c r="F71" s="127" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="G71" s="127" t="str">
+        <x:v>Sprint 2</x:v>
+      </x:c>
+      <x:c r="H71" s="127" t="str">
+        <x:v>Done</x:v>
+      </x:c>
+      <x:c r="I71" s="127" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J71" s="127" t="str">
+        <x:v>US-065, US-066</x:v>
+      </x:c>
+      <x:c r="K71" s="127" t="str">
+        <x:v>Agents load minimal authoritative context and produce traceable story packages without runtime LLM dependency</x:v>
+      </x:c>
+      <x:c r="L71" s="127" t="str">
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / FRAMEWORK-ENGINEERING-001 / MCP-US-067</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="48" customHeight="1">
+      <x:c r="A72" s="126" t="str">
+        <x:v>MCP-US-068</x:v>
+      </x:c>
+      <x:c r="B72" s="126" t="str">
+        <x:v>MCP-EPIC-008</x:v>
+      </x:c>
+      <x:c r="C72" s="126" t="str">
+        <x:v>Stable USB MIDI Instance Identity</x:v>
+      </x:c>
+      <x:c r="D72" s="126" t="str">
+        <x:v>Embedded/Release</x:v>
+      </x:c>
+      <x:c r="E72" s="126" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="F72" s="126" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="G72" s="126" t="str">
+        <x:v>Release train</x:v>
+      </x:c>
+      <x:c r="H72" s="126" t="str">
+        <x:v>MVP-late</x:v>
+      </x:c>
+      <x:c r="I72" s="126" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J72" s="126" t="str">
+        <x:v>US-003, US-004, US-055</x:v>
+      </x:c>
+      <x:c r="K72" s="126" t="str">
+        <x:v>Each device exposes a recognizable product name plus stable four-character instance ID; two devices are distinguishable without UID/MAC leakage</x:v>
+      </x:c>
+      <x:c r="L72" s="126" t="str">
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-007-ACCEPTANCE / MCP-US-068</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3704,7 +3951,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd9907143572430e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Read74dcd298d427b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3759,15 +4006,15 @@
         <x:v>Platform Foundation</x:v>
       </x:c>
       <x:c r="C5" s="64" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$67,A5)</x:f>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$200,A5)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="D5" s="64" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A5,'Backlog'!$E$5:$E$67,"Must")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$200,A5,'Backlog'!$E$5:$E$200,"Must")</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="E5" s="64" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A5,'Backlog'!$F$5:$F$67,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$200,A5,'Backlog'!$F$5:$F$200,"Done")</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="F5" s="23" t="str">
@@ -3782,16 +4029,16 @@
         <x:v>MIDI And Clock</x:v>
       </x:c>
       <x:c r="C6" s="65" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$67,A6)</x:f>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$200,A6)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="D6" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A6,'Backlog'!$E$5:$E$67,"Must")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$200,A6,'Backlog'!$E$5:$E$200,"Must")</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="E6" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A6,'Backlog'!$F$5:$F$67,"Done")</x:f>
-        <x:v>3</x:v>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$200,A6,'Backlog'!$F$5:$F$200,"Done")</x:f>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F6" s="24" t="str">
         <x:v>USB, BLE en DIN/UART MIDI; guitar slides, kontroles en clock</x:v>
@@ -3805,15 +4052,15 @@
         <x:v>Audio And Chip Core</x:v>
       </x:c>
       <x:c r="C7" s="65" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$67,A7)</x:f>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$200,A7)</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="D7" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A7,'Backlog'!$E$5:$E$67,"Must")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$200,A7,'Backlog'!$E$5:$E$200,"Must")</x:f>
         <x:v>9</x:v>
       </x:c>
       <x:c r="E7" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A7,'Backlog'!$F$5:$F$67,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$200,A7,'Backlog'!$F$5:$F$200,"Done")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F7" s="24" t="str">
@@ -3828,15 +4075,15 @@
         <x:v>Local Web Control</x:v>
       </x:c>
       <x:c r="C8" s="65" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$67,A8)</x:f>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$200,A8)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="D8" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A8,'Backlog'!$E$5:$E$67,"Must")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$200,A8,'Backlog'!$E$5:$E$200,"Must")</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="E8" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A8,'Backlog'!$F$5:$F$67,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$200,A8,'Backlog'!$F$5:$F$200,"Done")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F8" s="24" t="str">
@@ -3851,15 +4098,15 @@
         <x:v>Files, Harmony And Performance Tools</x:v>
       </x:c>
       <x:c r="C9" s="65" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$67,A9)</x:f>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$200,A9)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="D9" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A9,'Backlog'!$E$5:$E$67,"Must")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$200,A9,'Backlog'!$E$5:$E$200,"Must")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="E9" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A9,'Backlog'!$F$5:$F$67,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$200,A9,'Backlog'!$F$5:$F$200,"Done")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F9" s="24" t="str">
@@ -3874,15 +4121,15 @@
         <x:v>Multi-Core Expansion</x:v>
       </x:c>
       <x:c r="C10" s="65" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$67,A10)</x:f>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$200,A10)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="D10" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A10,'Backlog'!$E$5:$E$67,"Must")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$200,A10,'Backlog'!$E$5:$E$200,"Must")</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="E10" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A10,'Backlog'!$F$5:$F$67,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$200,A10,'Backlog'!$F$5:$F$200,"Done")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F10" s="24" t="str">
@@ -3897,15 +4144,15 @@
         <x:v>DSP And Pedal Hardware</x:v>
       </x:c>
       <x:c r="C11" s="65" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$67,A11)</x:f>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$200,A11)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="D11" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A11,'Backlog'!$E$5:$E$67,"Must")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$200,A11,'Backlog'!$E$5:$E$200,"Must")</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="E11" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A11,'Backlog'!$F$5:$F$67,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$200,A11,'Backlog'!$F$5:$F$200,"Done")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F11" s="24" t="str">
@@ -3920,19 +4167,42 @@
         <x:v>Portability, Quality And Release</x:v>
       </x:c>
       <x:c r="C12" s="66" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$67,A12)</x:f>
+        <x:f>COUNTIF('Backlog'!$B$5:$B$200,A12)</x:f>
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D12" s="66" t="n">
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$200,A12,'Backlog'!$E$5:$E$200,"Must")</x:f>
         <x:v>10</x:v>
       </x:c>
-      <x:c r="D12" s="66" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A12,'Backlog'!$E$5:$E$67,"Must")</x:f>
-        <x:v>9</x:v>
-      </x:c>
       <x:c r="E12" s="66" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$67,A12,'Backlog'!$F$5:$F$67,"Done")</x:f>
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$200,A12,'Backlog'!$F$5:$F$200,"Done")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F12" s="25" t="str">
         <x:v>Host/HIL, BLE-tweedebord, kruisplatform en release</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="44" customHeight="1">
+      <x:c r="A13" s="128" t="str">
+        <x:v>MCP-EPIC-009</x:v>
+      </x:c>
+      <x:c r="B13" s="128" t="str">
+        <x:v>Framework Engineering</x:v>
+      </x:c>
+      <x:c r="C13" s="128" t="n">
+        <x:f>COUNTIF('Backlog'!$B$5:$B$200,A13)</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D13" s="128" t="n">
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$200,A13,'Backlog'!$E$5:$E$200,"Must")</x:f>
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E13" s="128" t="n">
+        <x:f>COUNTIFS('Backlog'!$B$5:$B$200,A13,'Backlog'!$F$5:$F$200,"Done")</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F13" s="128" t="str">
+        <x:v>Vision, architecture, meta model, quality and controlled agent context</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3942,7 +4212,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf468f8966db645bc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb2a5f040ee842a0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3967,7 +4237,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>29 geregistreerde risiko's; dependency-closed Wemos HIL slaag en R-029 is beheers</x:v>
+        <x:v>30 geregistreerde risiko's; USB-MIDI HIL slaag en unieke instance-identiteit is as R-030 / US-068 georden</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -4658,6 +4928,29 @@
       </x:c>
       <x:c r="G33" t="str">
         <x:v>Controlled - writable HIL 2026-07-15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="44" customHeight="1">
+      <x:c r="A34" s="126" t="str">
+        <x:v>R-030</x:v>
+      </x:c>
+      <x:c r="B34" s="126" t="str">
+        <x:v>USB product names collide or change between boots</x:v>
+      </x:c>
+      <x:c r="C34" s="126" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="D34" s="126" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E34" s="126" t="str">
+        <x:v>Embedded/Release</x:v>
+      </x:c>
+      <x:c r="F34" s="126" t="str">
+        <x:v>Stable non-secret four-character instance ID, collision rule and two-device DAW acceptance in US-068</x:v>
+      </x:c>
+      <x:c r="G34" s="126" t="str">
+        <x:v>Backlog - US-068</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4687,7 +4980,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd7cfb43d3d4433b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d478ddd7fdf482c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4708,7 +5001,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Elke interne rol gee 'n sigbare bydrae; Copilot adviseer as eksterne reviewer; PO bly finale aanvaarder</x:v>
+        <x:v>Elke interne rol gee 'n sigbare bydrae; CEA bewaak coherence; Copilot adviseer; PO bly finale aanvaarder</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -4722,135 +5015,157 @@
         <x:v>Verpligte inset per story</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="36" customHeight="1">
-      <x:c r="A5" s="23" t="str">
+    <x:row r="5" ht="48" customHeight="1">
+      <x:c r="A5" s="132" t="str">
         <x:v>Sales/Discovery</x:v>
       </x:c>
-      <x:c r="B5" s="23" t="str">
+      <x:c r="B5" s="132" t="str">
         <x:v>Waarde, gebruiker, begroting</x:v>
       </x:c>
-      <x:c r="C5" s="23" t="str">
+      <x:c r="C5" s="132" t="str">
         <x:v>Waardehipotese en demo-uitkoms</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="36" customHeight="1">
-      <x:c r="A6" s="24" t="str">
+    <x:row r="6" ht="48" customHeight="1">
+      <x:c r="A6" s="133" t="str">
         <x:v>Business Analyst</x:v>
       </x:c>
-      <x:c r="B6" s="24" t="str">
+      <x:c r="B6" s="133" t="str">
         <x:v>Vloei, omvang, aannames</x:v>
       </x:c>
-      <x:c r="C6" s="24" t="str">
+      <x:c r="C6" s="133" t="str">
         <x:v>Story, kriteria en nie-doelwitte</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="36" customHeight="1">
-      <x:c r="A7" s="24" t="str">
+    <x:row r="7" ht="48" customHeight="1">
+      <x:c r="A7" s="134" t="str">
         <x:v>Product Owner</x:v>
       </x:c>
-      <x:c r="B7" s="24" t="str">
+      <x:c r="B7" s="134" t="str">
         <x:v>Prioriteit en aanvaarding</x:v>
       </x:c>
-      <x:c r="C7" s="24" t="str">
+      <x:c r="C7" s="134" t="str">
         <x:v>Ready/accept/reject</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="36" customHeight="1">
-      <x:c r="A8" s="24" t="str">
+    <x:row r="8" ht="48" customHeight="1">
+      <x:c r="A8" s="133" t="str">
         <x:v>Scrum Master</x:v>
       </x:c>
-      <x:c r="B8" s="24" t="str">
+      <x:c r="B8" s="133" t="str">
         <x:v>Volgorde en impediments</x:v>
       </x:c>
-      <x:c r="C8" s="24" t="str">
+      <x:c r="C8" s="133" t="str">
         <x:v>Now/Next/Later en blocker</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="36" customHeight="1">
-      <x:c r="A9" s="24" t="str">
+    <x:row r="9" ht="48" customHeight="1">
+      <x:c r="A9" s="134" t="str">
+        <x:v>Chief Enterprise Architect</x:v>
+      </x:c>
+      <x:c r="B9" s="134" t="str">
+        <x:v>Visie, vermoens, meta model en cross-epic coherence</x:v>
+      </x:c>
+      <x:c r="C9" s="134" t="str">
+        <x:v>Fitness teen visie en artefakgesag</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="48" customHeight="1">
+      <x:c r="A10" s="133" t="str">
+        <x:v>Framework Engineer</x:v>
+      </x:c>
+      <x:c r="B10" s="133" t="str">
+        <x:v>Konteks, taxonomy, review en kennisvloei</x:v>
+      </x:c>
+      <x:c r="C10" s="133" t="str">
+        <x:v>Minimale storypakket en framework sanity</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="48" customHeight="1">
+      <x:c r="A11" s="134" t="str">
         <x:v>Solution Architect</x:v>
       </x:c>
-      <x:c r="B9" s="24" t="str">
+      <x:c r="B11" s="134" t="str">
         <x:v>Poorte, ADR en portabiliteit</x:v>
       </x:c>
-      <x:c r="C9" s="24" t="str">
+      <x:c r="C11" s="134" t="str">
         <x:v>Ontwerpresensie en trade-off</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="36" customHeight="1">
-      <x:c r="A10" s="24" t="str">
+    <x:row r="12" ht="48" customHeight="1">
+      <x:c r="A12" s="133" t="str">
         <x:v>Embedded Engineer</x:v>
       </x:c>
-      <x:c r="B10" s="24" t="str">
+      <x:c r="B12" s="133" t="str">
         <x:v>Boot, bord, penne, geheue</x:v>
       </x:c>
-      <x:c r="C10" s="24" t="str">
+      <x:c r="C12" s="133" t="str">
         <x:v>Bordimpak en herstelpad</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="36" customHeight="1">
-      <x:c r="A11" s="24" t="str">
+    <x:row r="13" ht="48" customHeight="1">
+      <x:c r="A13" s="134" t="str">
         <x:v>MIDI Engineer</x:v>
       </x:c>
-      <x:c r="B11" s="24" t="str">
+      <x:c r="B13" s="134" t="str">
         <x:v>MIDI, kanale, clock, controls</x:v>
       </x:c>
-      <x:c r="C11" s="24" t="str">
+      <x:c r="C13" s="134" t="str">
         <x:v>Kontrakte en randgevalle</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="36" customHeight="1">
-      <x:c r="A12" s="24" t="str">
+    <x:row r="14" ht="48" customHeight="1">
+      <x:c r="A14" s="133" t="str">
         <x:v>DSP/Chip Engineer</x:v>
       </x:c>
-      <x:c r="B12" s="24" t="str">
+      <x:c r="B14" s="133" t="str">
         <x:v>Kern, voices, audio, DSP</x:v>
       </x:c>
-      <x:c r="C12" s="24" t="str">
+      <x:c r="C14" s="133" t="str">
         <x:v>CPU/RAM/latensie/akkuraatheid</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="36" customHeight="1">
-      <x:c r="A13" s="24" t="str">
+    <x:row r="15" ht="48" customHeight="1">
+      <x:c r="A15" s="135" t="str">
         <x:v>Web Engineer</x:v>
       </x:c>
-      <x:c r="B13" s="24" t="str">
+      <x:c r="B15" s="135" t="str">
         <x:v>Plaaslike UI en scheduling</x:v>
       </x:c>
-      <x:c r="C13" s="24" t="str">
+      <x:c r="C15" s="135" t="str">
         <x:v>UI-vloei en bronimpak</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="36" customHeight="1">
-      <x:c r="A14" s="24" t="str">
+    <x:row r="16" ht="48" customHeight="1">
+      <x:c r="A16" s="127" t="str">
         <x:v>QA/HIL Engineer</x:v>
       </x:c>
-      <x:c r="B14" s="24" t="str">
+      <x:c r="B16" s="127" t="str">
         <x:v>Rooi/groen en instrumentmeting</x:v>
       </x:c>
-      <x:c r="C14" s="24" t="str">
+      <x:c r="C16" s="127" t="str">
         <x:v>Toetsmatriks en bewys</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="36" customHeight="1">
-      <x:c r="A15" s="25" t="str">
+    <x:row r="17" ht="48" customHeight="1">
+      <x:c r="A17" s="136" t="str">
         <x:v>Release/Documentation</x:v>
       </x:c>
-      <x:c r="B15" s="25" t="str">
+      <x:c r="B17" s="136" t="str">
         <x:v>Git, installasie en traceability</x:v>
       </x:c>
-      <x:c r="C15" s="25" t="str">
+      <x:c r="C17" s="136" t="str">
         <x:v>Publikasiehek en docs</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="38" customHeight="1">
-      <x:c r="A16" t="str">
+    <x:row r="18" ht="48" customHeight="1">
+      <x:c r="A18" s="127" t="str">
         <x:v>External Architecture Reviewer (Copilot)</x:v>
       </x:c>
-      <x:c r="B16" t="str">
+      <x:c r="B18" s="127" t="str">
         <x:v>Onafhanklike ontwerp- en risiko-review</x:v>
       </x:c>
-      <x:c r="C16" t="str">
+      <x:c r="C18" s="127" t="str">
         <x:v>Bevindings is advies; PO/architect besluit en traceer</x:v>
       </x:c>
     </x:row>
@@ -4861,7 +5176,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7feade596b594f1f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21e91df7a89d4cc0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5327,7 +5642,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f8af9ccb27d458c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ad94215b7fc4528"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(scope): reduce MVP to audible D1 in Logic
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ra7181de9364244f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R3055ec9c060242f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Re31549d4d9684c14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R6aa36888d4544ece"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="Rb62c8d93eb664a26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rfdeb6f5bbf9b4941"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R35f4bc40367241cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="Ra81e651c4a134d3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="R390e254c652b43c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="Re1ab7c876df64e1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R5ee93503758a4f2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R7ca07df745f14431"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -154,7 +154,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="25">
+  <x:fills count="27">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -276,6 +276,16 @@
         <x:fgColor rgb="FFFCE0D1"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFCE0D1"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFCE0D1"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="8">
     <x:border/>
@@ -348,7 +358,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="140">
+  <x:cellXfs count="143">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -691,6 +701,15 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1060,7 +1079,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="102" t="str">
-        <x:v>Sprint 2 | scope v0.17.0 | runtime v0.12.3 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
+        <x:v>Sprint 2 | scope v0.18.0 | runtime v0.12.3 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
       </x:c>
       <x:c r="B2" s="103"/>
       <x:c r="C2" s="103"/>
@@ -1106,7 +1125,7 @@
       </x:c>
       <x:c r="C5" s="85"/>
       <x:c r="D5" s="110" t="str">
-        <x:v>1. Veilige minimale USB-MIDI boot en herstel</x:v>
+        <x:v>1. Sluit US-005 SET/UNSET-konfigurasiegrens</x:v>
       </x:c>
       <x:c r="E5" s="110"/>
       <x:c r="F5" s="110"/>
@@ -1123,7 +1142,7 @@
       </x:c>
       <x:c r="C6" s="85"/>
       <x:c r="D6" s="111" t="str">
-        <x:v>2. MAX98357 mono-I2S eerste; PWM fallback</x:v>
+        <x:v>2. Bou AudioOutput en onafhanklike G-C-D I2S-preflight</x:v>
       </x:c>
       <x:c r="E6" s="111"/>
       <x:c r="F6" s="111"/>
@@ -1140,7 +1159,7 @@
       </x:c>
       <x:c r="C7" s="85"/>
       <x:c r="D7" s="111" t="str">
-        <x:v>3. D1-basiskern voor SN76489; SID en OPL daarna</x:v>
+        <x:v>3. D1 sine/saw/square met korrekte Note On/Off</x:v>
       </x:c>
       <x:c r="E7" s="111"/>
       <x:c r="F7" s="111"/>
@@ -1149,15 +1168,15 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="111" t="str">
-        <x:v>MVP-gemerk</x:v>
+        <x:v>MVP acceptance-set</x:v>
       </x:c>
       <x:c r="B8" s="114" t="n">
-        <x:f>COUNTIF('Backlog'!$E$5:$E$200,"Must")</x:f>
-        <x:v>51</x:v>
+        <x:f>COUNTIF('Backlog'!$H$5:$H$200,"MVP-Must")+COUNTIF('Backlog'!$H$5:$H$200,"MVP-Enabler")+COUNTIF('Backlog'!$H$5:$H$200,"MVP-Enabler (Done)")+COUNTIF('Backlog'!$H$5:$H$200,"MVP-Enabler (In Review)")</x:f>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C8" s="85"/>
       <x:c r="D8" s="112" t="str">
-        <x:v>4. BLE op tweede bord; S2 faal veilig; multi-core na resource gate</x:v>
+        <x:v>4. Logic External MIDI na hoorbare D1 op verwysingsbord</x:v>
       </x:c>
       <x:c r="E8" s="112"/>
       <x:c r="F8" s="112"/>
@@ -1170,11 +1189,11 @@
       </x:c>
       <x:c r="B9" s="114" t="n">
         <x:f>COUNTA('Risks'!$A$5:$A$200)</x:f>
-        <x:v>32</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="C9" s="85"/>
       <x:c r="D9" s="116" t="str">
-        <x:v>5. Station join met beveiligde AP-fallback; mobile UI en logging binne begroting</x:v>
+        <x:v>5. Release; daarna SN76489 en volgende kerne</x:v>
       </x:c>
       <x:c r="E9" s="116"/>
       <x:c r="F9" s="116"/>
@@ -1218,7 +1237,7 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="119" t="str">
-        <x:v>91 tests GREEN | USB-MIDI HIL PASS | US-005 leewaarde-herstel wag op finale Wemos-herbewys | audio/BLE bly oop</x:v>
+        <x:v>91 tests GREEN | USB-MIDI HIL PASS | US-005 UNSET-HIL wag | volgende: AudioOutput -&gt; standalone I2S -&gt; D1 -&gt; Logic</x:v>
       </x:c>
       <x:c r="B13" s="120"/>
       <x:c r="C13" s="120"/>
@@ -1240,7 +1259,7 @@
     </x:row>
     <x:row r="15" ht="58" customHeight="1">
       <x:c r="A15" s="123" t="str">
-        <x:v>Product Owner note 2026-07-16: fisiese chip/display uitbreiding is post-MVP; US-023 besit hostname/IP startupstatus.</x:v>
+        <x:v>MVP 2026-07-16: verwysingsbord ontvang Logic USB-MIDI en speel hoorbare D1; alle volgende cores en uitbreidings is post-MVP.</x:v>
       </x:c>
       <x:c r="B15" s="124"/>
       <x:c r="C15" s="124"/>
@@ -1282,6 +1301,7 @@
     <x:mergeCell ref="A13:H13"/>
     <x:mergeCell ref="A15:H17"/>
     <x:mergeCell ref="A15:H15"/>
+    <x:mergeCell ref="D9:H9"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1312,7 +1332,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Bron: docs/user_stories_v0.1.0.md | 74 stories | Redigeer Status en Priority via keuselyste</x:v>
+        <x:v>Bron: docs/user_stories_v0.1.0.md v0.18.0 | 74 stories | 16-story bevrore MVP Acceptance Set</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -1376,7 +1396,7 @@
         <x:v>Sprint 0</x:v>
       </x:c>
       <x:c r="H5" s="23" t="str">
-        <x:v>Done</x:v>
+        <x:v>MVP-Enabler (Done)</x:v>
       </x:c>
       <x:c r="I5" s="64" t="n">
         <x:v>3</x:v>
@@ -1414,7 +1434,7 @@
         <x:v>Sprint 1</x:v>
       </x:c>
       <x:c r="H6" s="24" t="str">
-        <x:v>Done</x:v>
+        <x:v>MVP-Enabler (Done)</x:v>
       </x:c>
       <x:c r="I6" s="65" t="n">
         <x:v>5</x:v>
@@ -1452,7 +1472,7 @@
         <x:v>Sprint 1</x:v>
       </x:c>
       <x:c r="H7" s="24" t="str">
-        <x:v>Done</x:v>
+        <x:v>MVP-Enabler (Done)</x:v>
       </x:c>
       <x:c r="I7" s="65" t="n">
         <x:v>8</x:v>
@@ -1490,7 +1510,7 @@
         <x:v>Sprint 1</x:v>
       </x:c>
       <x:c r="H8" s="24" t="str">
-        <x:v>Done</x:v>
+        <x:v>MVP-Enabler (Done)</x:v>
       </x:c>
       <x:c r="I8" s="65" t="n">
         <x:v>5</x:v>
@@ -1528,7 +1548,7 @@
         <x:v>Sprint 1</x:v>
       </x:c>
       <x:c r="H9" s="24" t="str">
-        <x:v>In Review</x:v>
+        <x:v>MVP-Enabler (In Review)</x:v>
       </x:c>
       <x:c r="I9" s="65" t="n">
         <x:v>5</x:v>
@@ -1566,7 +1586,7 @@
         <x:v>Sprint 2</x:v>
       </x:c>
       <x:c r="H10" s="24" t="str">
-        <x:v>Done</x:v>
+        <x:v>MVP-Enabler (Done)</x:v>
       </x:c>
       <x:c r="I10" s="65" t="n">
         <x:v>5</x:v>
@@ -1604,7 +1624,7 @@
         <x:v>Sprint 2</x:v>
       </x:c>
       <x:c r="H11" s="24" t="str">
-        <x:v>Done</x:v>
+        <x:v>MVP-Enabler (Done)</x:v>
       </x:c>
       <x:c r="I11" s="65" t="n">
         <x:v>5</x:v>
@@ -1642,7 +1662,7 @@
         <x:v>Sprint 2</x:v>
       </x:c>
       <x:c r="H12" s="24" t="str">
-        <x:v>Done</x:v>
+        <x:v>MVP-Enabler (Done)</x:v>
       </x:c>
       <x:c r="I12" s="65" t="n">
         <x:v>5</x:v>
@@ -1680,7 +1700,7 @@
         <x:v>Sprint 2</x:v>
       </x:c>
       <x:c r="H13" s="24" t="str">
-        <x:v>Done</x:v>
+        <x:v>MVP-Enabler (Done)</x:v>
       </x:c>
       <x:c r="I13" s="65" t="n">
         <x:v>5</x:v>
@@ -1718,7 +1738,7 @@
         <x:v>Sprint 2</x:v>
       </x:c>
       <x:c r="H14" s="24" t="str">
-        <x:v>Host accepted / audible blocked</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I14" s="65" t="n">
         <x:v>5</x:v>
@@ -1756,7 +1776,7 @@
         <x:v>Sprint 3</x:v>
       </x:c>
       <x:c r="H15" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I15" s="65" t="n">
         <x:v>5</x:v>
@@ -1794,7 +1814,7 @@
         <x:v>Sprint 3</x:v>
       </x:c>
       <x:c r="H16" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I16" s="65" t="n">
         <x:v>5</x:v>
@@ -1832,7 +1852,7 @@
         <x:v>Sprint 3</x:v>
       </x:c>
       <x:c r="H17" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I17" s="65" t="n">
         <x:v>5</x:v>
@@ -1870,7 +1890,7 @@
         <x:v>Sprint 3</x:v>
       </x:c>
       <x:c r="H18" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>MVP-Enabler</x:v>
       </x:c>
       <x:c r="I18" s="65" t="n">
         <x:v>5</x:v>
@@ -1908,7 +1928,7 @@
         <x:v>Sprint 4</x:v>
       </x:c>
       <x:c r="H19" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I19" s="65" t="n">
         <x:v>3</x:v>
@@ -1931,7 +1951,7 @@
         <x:v>MCP-EPIC-003</x:v>
       </x:c>
       <x:c r="C20" s="24" t="str">
-        <x:v>MAX98357 Mono I2S Audible Diagnostic</x:v>
+        <x:v>Standalone I2S Audible Diagnostic (MAX98357 Default)</x:v>
       </x:c>
       <x:c r="D20" s="24" t="str">
         <x:v>DSP/Chip Engineer</x:v>
@@ -1946,7 +1966,7 @@
         <x:v>Sprint 3</x:v>
       </x:c>
       <x:c r="H20" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>MVP-Must</x:v>
       </x:c>
       <x:c r="I20" s="65" t="n">
         <x:v>5</x:v>
@@ -1955,10 +1975,10 @@
         <x:v>US-004, US-014</x:v>
       </x:c>
       <x:c r="K20" s="24" t="str">
-        <x:v>Ondersteuning, penne, DAC, RAM, latensie en kwaliteit is gemeet</x:v>
+        <x:v>Class-based device/i2s_test.py imports no synth package or global state; injected PCM-I2S profile plays G3-C4-D4 square waves; MAX98357 IO5/IO3/IO7 passes audible HIL and releases I2S</x:v>
       </x:c>
       <x:c r="L20" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-016</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MVP-SCOPE-REDUCTION-001 / MCP-US-016</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="38" customHeight="1">
@@ -1984,13 +2004,13 @@
         <x:v>Sprint 3</x:v>
       </x:c>
       <x:c r="H21" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I21" s="65" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="J21" s="24" t="str">
-        <x:v>US-063</x:v>
+        <x:v>US-063, US-057</x:v>
       </x:c>
       <x:c r="K21" s="24" t="str">
         <x:v>Tweede musikale kern: drie toonstemme speel onafhanklik met gedokumenteerde akkuraatheid</x:v>
@@ -2022,7 +2042,7 @@
         <x:v>Sprint 4</x:v>
       </x:c>
       <x:c r="H22" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I22" s="65" t="n">
         <x:v>5</x:v>
@@ -2060,7 +2080,7 @@
         <x:v>Sprint 4</x:v>
       </x:c>
       <x:c r="H23" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I23" s="65" t="n">
         <x:v>5</x:v>
@@ -2083,7 +2103,7 @@
         <x:v>MCP-EPIC-003</x:v>
       </x:c>
       <x:c r="C24" s="24" t="str">
-        <x:v>Optional G-C-D Startup Test</x:v>
+        <x:v>Optional Integrated G-C-D Startup Test</x:v>
       </x:c>
       <x:c r="D24" s="24" t="str">
         <x:v>DSP/Chip Engineer</x:v>
@@ -2098,7 +2118,7 @@
         <x:v>Sprint 4</x:v>
       </x:c>
       <x:c r="H24" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I24" s="65" t="n">
         <x:v>5</x:v>
@@ -2107,7 +2127,7 @@
         <x:v>US-016, US-063</x:v>
       </x:c>
       <x:c r="K24" s="24" t="str">
-        <x:v>Opsionele sestiendenootreeks bewys die klankpad by start</x:v>
+        <x:v>Post-MVP startup tune uses D1/runtime AudioOutput and remains distinct from standalone US-016 hardware diagnostic</x:v>
       </x:c>
       <x:c r="L24" s="24" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-020</x:v>
@@ -2136,7 +2156,7 @@
         <x:v>Sprint 4</x:v>
       </x:c>
       <x:c r="H25" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I25" s="65" t="n">
         <x:v>3</x:v>
@@ -2174,7 +2194,7 @@
         <x:v>Sprint 5</x:v>
       </x:c>
       <x:c r="H26" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I26" s="65" t="n">
         <x:v>5</x:v>
@@ -2212,7 +2232,7 @@
         <x:v>Sprint 5</x:v>
       </x:c>
       <x:c r="H27" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I27" s="65" t="n">
         <x:v>5</x:v>
@@ -2250,7 +2270,7 @@
         <x:v>Sprint 5</x:v>
       </x:c>
       <x:c r="H28" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I28" s="65" t="n">
         <x:v>8</x:v>
@@ -2288,7 +2308,7 @@
         <x:v>Sprint 5</x:v>
       </x:c>
       <x:c r="H29" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I29" s="65" t="n">
         <x:v>5</x:v>
@@ -2326,7 +2346,7 @@
         <x:v>Sprint 5</x:v>
       </x:c>
       <x:c r="H30" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I30" s="65" t="n">
         <x:v>5</x:v>
@@ -2364,7 +2384,7 @@
         <x:v>Sprint 5</x:v>
       </x:c>
       <x:c r="H31" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I31" s="65" t="n">
         <x:v>8</x:v>
@@ -2592,7 +2612,7 @@
         <x:v>Sprint 6+</x:v>
       </x:c>
       <x:c r="H37" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I37" s="65" t="n">
         <x:v>5</x:v>
@@ -2630,7 +2650,7 @@
         <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="H38" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I38" s="65" t="n">
         <x:v>5</x:v>
@@ -2668,7 +2688,7 @@
         <x:v>MVP-late</x:v>
       </x:c>
       <x:c r="H39" s="24" t="str">
-        <x:v>MVP-late</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I39" s="65" t="n">
         <x:v>8</x:v>
@@ -2706,7 +2726,7 @@
         <x:v>MVP-late</x:v>
       </x:c>
       <x:c r="H40" s="24" t="str">
-        <x:v>MVP-late</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I40" s="65" t="n">
         <x:v>5</x:v>
@@ -2744,7 +2764,7 @@
         <x:v>MVP-late</x:v>
       </x:c>
       <x:c r="H41" s="24" t="str">
-        <x:v>MVP-late</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I41" s="65" t="n">
         <x:v>8</x:v>
@@ -2972,7 +2992,7 @@
         <x:v>MVP-late</x:v>
       </x:c>
       <x:c r="H47" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I47" s="65" t="n">
         <x:v>5</x:v>
@@ -3010,7 +3030,7 @@
         <x:v>MVP-late</x:v>
       </x:c>
       <x:c r="H48" s="24" t="str">
-        <x:v>MVP-late</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I48" s="65" t="n">
         <x:v>5</x:v>
@@ -3048,7 +3068,7 @@
         <x:v>MVP-late</x:v>
       </x:c>
       <x:c r="H49" s="24" t="str">
-        <x:v>MVP-late</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I49" s="65" t="n">
         <x:v>3</x:v>
@@ -3238,7 +3258,7 @@
         <x:v>Release train</x:v>
       </x:c>
       <x:c r="H54" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>MVP-Enabler</x:v>
       </x:c>
       <x:c r="I54" s="65" t="n">
         <x:v>5</x:v>
@@ -3276,16 +3296,16 @@
         <x:v>Sprint 1</x:v>
       </x:c>
       <x:c r="H55" s="24" t="str">
-        <x:v>In Review/MVP</x:v>
+        <x:v>MVP-Enabler (In Review)</x:v>
       </x:c>
       <x:c r="I55" s="65" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="J55" s="24" t="str">
-        <x:v>US-003, US-015</x:v>
+        <x:v>US-003, US-016</x:v>
       </x:c>
       <x:c r="K55" s="24" t="str">
-        <x:v>Autoreload-safe deploy, closure, 16 hashes, libraries, boot en import/execution is fisies groen; klankadapter bly oop</x:v>
+        <x:v>Deploy/closure/boot/import execution remains green; MAX98357 audio adapter closes with US-016 audible proof</x:v>
       </x:c>
       <x:c r="L55" s="24" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-051-IMP-001 / v0.11.1</x:v>
@@ -3314,7 +3334,7 @@
         <x:v>Release train</x:v>
       </x:c>
       <x:c r="H56" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I56" s="65" t="n">
         <x:v>8</x:v>
@@ -3390,7 +3410,7 @@
         <x:v>Release train</x:v>
       </x:c>
       <x:c r="H58" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I58" s="65" t="n">
         <x:v>5</x:v>
@@ -3413,7 +3433,7 @@
         <x:v>MCP-EPIC-008</x:v>
       </x:c>
       <x:c r="C59" s="24" t="str">
-        <x:v>macOS Logic Pro Acceptance</x:v>
+        <x:v>macOS Logic Pro Audible D1 Acceptance</x:v>
       </x:c>
       <x:c r="D59" s="24" t="str">
         <x:v>QA/Release</x:v>
@@ -3428,16 +3448,16 @@
         <x:v>Release train</x:v>
       </x:c>
       <x:c r="H59" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>MVP-Must</x:v>
       </x:c>
       <x:c r="I59" s="65" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="J59" s="24" t="str">
-        <x:v>US-003, US-007</x:v>
+        <x:v>US-003, US-007, US-009, US-014, US-016, US-063</x:v>
       </x:c>
       <x:c r="K59" s="24" t="str">
-        <x:v>Logic kies die synth as External MIDI destination en stuur note/clock; fisiese pedaaluitvoer bly die klankpad</x:v>
+        <x:v>Logic selects the board as External MIDI, sends Note On/Off and the user hears D1 through the reference I2S path</x:v>
       </x:c>
       <x:c r="L59" s="24" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-055</x:v>
@@ -3466,7 +3486,7 @@
         <x:v>Release train</x:v>
       </x:c>
       <x:c r="H60" s="24" t="str">
-        <x:v>MVP</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I60" s="65" t="n">
         <x:v>5</x:v>
@@ -3504,16 +3524,16 @@
         <x:v>Release train</x:v>
       </x:c>
       <x:c r="H61" s="25" t="str">
-        <x:v>MVP</x:v>
+        <x:v>MVP-Must</x:v>
       </x:c>
       <x:c r="I61" s="66" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="J61" s="25" t="str">
-        <x:v>Alle MVP-stories</x:v>
+        <x:v>US-001 to US-009, US-014, US-016, US-050, US-051, US-055, US-063</x:v>
       </x:c>
       <x:c r="K61" s="25" t="str">
-        <x:v>Tag, release notes, bekende beperkings en demo is gereed</x:v>
+        <x:v>Tag, release notes and known limitations accompany a repeatable Logic USB-MIDI to audible D1 demo</x:v>
       </x:c>
       <x:c r="L61" s="25" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-057</x:v>
@@ -3542,18 +3562,18 @@
         <x:v>Sprint 4</x:v>
       </x:c>
       <x:c r="H62" s="70" t="str">
-        <x:v>MVP</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I62" s="77" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="J62" t="str">
+      <x:c r="J62" s="83" t="str">
         <x:v>US-008, US-010</x:v>
       </x:c>
-      <x:c r="K62" t="str">
+      <x:c r="K62" s="83" t="str">
         <x:v>Multi-kanaal note en per-kanaal bends behou onafhanklike string/slide-semantiek met konfigureerbare bend range</x:v>
       </x:c>
-      <x:c r="L62" t="str">
+      <x:c r="L62" s="83" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-058</x:v>
       </x:c>
     </x:row>
@@ -3580,94 +3600,94 @@
         <x:v>Release train</x:v>
       </x:c>
       <x:c r="H63" s="74" t="str">
-        <x:v>MVP</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I63" s="78" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="J63" t="str">
+      <x:c r="J63" s="83" t="str">
         <x:v>US-018, US-058</x:v>
       </x:c>
-      <x:c r="K63" t="str">
+      <x:c r="K63" s="83" t="str">
         <x:v>'n Generiese MIDI-kitaar en Fishman-verwysing speel note, akkoorde, bends en slides; geen toestelnaam is 'n kodekonstante nie</x:v>
       </x:c>
-      <x:c r="L63" t="str">
+      <x:c r="L63" s="83" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-059</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="34" customHeight="1">
-      <x:c r="A64" t="str">
+      <x:c r="A64" s="83" t="str">
         <x:v>MCP-US-060</x:v>
       </x:c>
-      <x:c r="B64" t="str">
+      <x:c r="B64" s="83" t="str">
         <x:v>MCP-EPIC-008</x:v>
       </x:c>
-      <x:c r="C64" t="str">
+      <x:c r="C64" s="83" t="str">
         <x:v>Standalone External MIDI Host Acceptance</x:v>
       </x:c>
-      <x:c r="D64" t="str">
+      <x:c r="D64" s="83" t="str">
         <x:v>QA/Release</x:v>
       </x:c>
-      <x:c r="E64" t="str">
+      <x:c r="E64" s="83" t="str">
         <x:v>Must</x:v>
       </x:c>
-      <x:c r="F64" t="str">
+      <x:c r="F64" s="83" t="str">
         <x:v>Backlog</x:v>
       </x:c>
-      <x:c r="G64" t="str">
+      <x:c r="G64" s="83" t="str">
         <x:v>Release train</x:v>
       </x:c>
-      <x:c r="H64" t="str">
-        <x:v>MVP</x:v>
-      </x:c>
-      <x:c r="I64" t="n">
+      <x:c r="H64" s="83" t="str">
+        <x:v>Post-MVP</x:v>
+      </x:c>
+      <x:c r="I64" s="83" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="J64" t="str">
+      <x:c r="J64" s="83" t="str">
         <x:v>US-013, US-017</x:v>
       </x:c>
-      <x:c r="K64" t="str">
+      <x:c r="K64" s="83" t="str">
         <x:v>Controller na Raspberry Pi/eksterne USB-host na DIN/UART lewer note, bend en clock sonder DAW</x:v>
       </x:c>
-      <x:c r="L64" t="str">
+      <x:c r="L64" s="83" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MIDI-TRANSPORT-MULTICORE-AMENDMENT-001 / MCP-US-060</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="34" customHeight="1">
-      <x:c r="A65" t="str">
+      <x:c r="A65" s="83" t="str">
         <x:v>MCP-US-061</x:v>
       </x:c>
-      <x:c r="B65" t="str">
+      <x:c r="B65" s="83" t="str">
         <x:v>MCP-EPIC-006</x:v>
       </x:c>
-      <x:c r="C65" t="str">
+      <x:c r="C65" s="83" t="str">
         <x:v>Multi-Core Resource Guard And Telemetry</x:v>
       </x:c>
-      <x:c r="D65" t="str">
+      <x:c r="D65" s="83" t="str">
         <x:v>DSP/Chip Engineer</x:v>
       </x:c>
-      <x:c r="E65" t="str">
+      <x:c r="E65" s="83" t="str">
         <x:v>Must</x:v>
       </x:c>
-      <x:c r="F65" t="str">
+      <x:c r="F65" s="83" t="str">
         <x:v>Backlog</x:v>
       </x:c>
-      <x:c r="G65" t="str">
+      <x:c r="G65" s="83" t="str">
         <x:v>MVP-late</x:v>
       </x:c>
-      <x:c r="H65" t="str">
-        <x:v>MVP-late</x:v>
-      </x:c>
-      <x:c r="I65" t="n">
+      <x:c r="H65" s="83" t="str">
+        <x:v>Post-MVP</x:v>
+      </x:c>
+      <x:c r="I65" s="83" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="J65" t="str">
+      <x:c r="J65" s="83" t="str">
         <x:v>US-037</x:v>
       </x:c>
-      <x:c r="K65" t="str">
+      <x:c r="K65" s="83" t="str">
         <x:v>Heap, looplatensie en dropout word gemeet; onveilige addisionele kern word deterministies geweier of afgeskakel</x:v>
       </x:c>
-      <x:c r="L65" t="str">
+      <x:c r="L65" s="83" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MIDI-TRANSPORT-MULTICORE-AMENDMENT-001 / MCP-US-061</x:v>
       </x:c>
     </x:row>
@@ -3694,7 +3714,7 @@
         <x:v>Sprint 4</x:v>
       </x:c>
       <x:c r="H66" s="83" t="str">
-        <x:v>S2 negative accepted / BLE HIL blocked</x:v>
+        <x:v>Post-MVP</x:v>
       </x:c>
       <x:c r="I66" s="83" t="n">
         <x:v>8</x:v>
@@ -3732,56 +3752,56 @@
         <x:v>Sprint 3</x:v>
       </x:c>
       <x:c r="H67" s="83" t="str">
-        <x:v>MVP</x:v>
+        <x:v>MVP-Must</x:v>
       </x:c>
       <x:c r="I67" s="83" t="n">
         <x:v>8</x:v>
       </x:c>
       <x:c r="J67" s="83" t="str">
-        <x:v>US-006, US-014, US-016</x:v>
+        <x:v>US-006, US-008, US-009, US-014, US-016</x:v>
       </x:c>
       <x:c r="K67" s="83" t="str">
-        <x:v>Nuut-geporteerde sine/saw/square D1-gedrag speel via AudioOutput; geen desktop-backend of produksierepo-wysiging</x:v>
+        <x:v>Portable sine/saw/square D1 handles Note On/Off through AudioOutput; no desktop backend or production-repo modification</x:v>
       </x:c>
       <x:c r="L67" s="83" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / SCOPE-AMENDMENT-002 / MCP-US-063</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="48" customHeight="1">
-      <x:c r="A68" s="126" t="str">
+      <x:c r="A68" s="140" t="str">
         <x:v>MCP-US-064</x:v>
       </x:c>
-      <x:c r="B68" s="126" t="str">
+      <x:c r="B68" s="140" t="str">
         <x:v>MCP-EPIC-009</x:v>
       </x:c>
-      <x:c r="C68" s="126" t="str">
+      <x:c r="C68" s="140" t="str">
         <x:v>Enterprise Vision And Architecture Baseline</x:v>
       </x:c>
-      <x:c r="D68" s="126" t="str">
+      <x:c r="D68" s="140" t="str">
         <x:v>Chief Enterprise Architect</x:v>
       </x:c>
-      <x:c r="E68" s="126" t="str">
+      <x:c r="E68" s="140" t="str">
         <x:v>Must</x:v>
       </x:c>
-      <x:c r="F68" s="126" t="str">
+      <x:c r="F68" s="140" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="G68" s="126" t="str">
+      <x:c r="G68" s="140" t="str">
         <x:v>Sprint 2</x:v>
       </x:c>
-      <x:c r="H68" s="126" t="str">
+      <x:c r="H68" s="140" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="I68" s="126" t="n">
+      <x:c r="I68" s="140" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="J68" s="126" t="str">
+      <x:c r="J68" s="140" t="str">
         <x:v>US-001, US-002</x:v>
       </x:c>
-      <x:c r="K68" s="126" t="str">
+      <x:c r="K68" s="140" t="str">
         <x:v>Enterprise vision plus framework, solution and deployment architecture form one cross-linked baseline</x:v>
       </x:c>
-      <x:c r="L68" s="126" t="str">
+      <x:c r="L68" s="140" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / FRAMEWORK-ENGINEERING-001 / MCP-US-064</x:v>
       </x:c>
     </x:row>
@@ -3824,40 +3844,40 @@
       </x:c>
     </x:row>
     <x:row r="70" ht="48" customHeight="1">
-      <x:c r="A70" s="126" t="str">
+      <x:c r="A70" s="140" t="str">
         <x:v>MCP-US-066</x:v>
       </x:c>
-      <x:c r="B70" s="126" t="str">
+      <x:c r="B70" s="140" t="str">
         <x:v>MCP-EPIC-009</x:v>
       </x:c>
-      <x:c r="C70" s="126" t="str">
+      <x:c r="C70" s="140" t="str">
         <x:v>Quality Manual, Test Strategy And Review Engine</x:v>
       </x:c>
-      <x:c r="D70" s="126" t="str">
+      <x:c r="D70" s="140" t="str">
         <x:v>QA/Release</x:v>
       </x:c>
-      <x:c r="E70" s="126" t="str">
+      <x:c r="E70" s="140" t="str">
         <x:v>Must</x:v>
       </x:c>
-      <x:c r="F70" s="126" t="str">
+      <x:c r="F70" s="140" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="G70" s="126" t="str">
+      <x:c r="G70" s="140" t="str">
         <x:v>Sprint 2</x:v>
       </x:c>
-      <x:c r="H70" s="126" t="str">
+      <x:c r="H70" s="140" t="str">
         <x:v>Done</x:v>
       </x:c>
-      <x:c r="I70" s="126" t="n">
+      <x:c r="I70" s="140" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="J70" s="126" t="str">
+      <x:c r="J70" s="140" t="str">
         <x:v>US-064, US-065</x:v>
       </x:c>
-      <x:c r="K70" s="126" t="str">
+      <x:c r="K70" s="140" t="str">
         <x:v>Definition of Done points to repeatable quality, test and review gates without treating docs as proof</x:v>
       </x:c>
-      <x:c r="L70" s="126" t="str">
+      <x:c r="L70" s="140" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / FRAMEWORK-ENGINEERING-001 / MCP-US-066</x:v>
       </x:c>
     </x:row>
@@ -3900,268 +3920,268 @@
       </x:c>
     </x:row>
     <x:row r="72" ht="48" customHeight="1">
-      <x:c r="A72" s="126" t="str">
+      <x:c r="A72" s="140" t="str">
         <x:v>MCP-US-068</x:v>
       </x:c>
-      <x:c r="B72" s="126" t="str">
+      <x:c r="B72" s="140" t="str">
         <x:v>MCP-EPIC-008</x:v>
       </x:c>
-      <x:c r="C72" s="126" t="str">
+      <x:c r="C72" s="140" t="str">
         <x:v>Stable USB MIDI Instance Identity</x:v>
       </x:c>
-      <x:c r="D72" s="126" t="str">
+      <x:c r="D72" s="140" t="str">
         <x:v>Embedded/Release</x:v>
       </x:c>
-      <x:c r="E72" s="126" t="str">
+      <x:c r="E72" s="140" t="str">
         <x:v>Must</x:v>
       </x:c>
-      <x:c r="F72" s="126" t="str">
+      <x:c r="F72" s="140" t="str">
         <x:v>Backlog</x:v>
       </x:c>
-      <x:c r="G72" s="126" t="str">
+      <x:c r="G72" s="140" t="str">
         <x:v>Release train</x:v>
       </x:c>
-      <x:c r="H72" s="126" t="str">
-        <x:v>MVP-late</x:v>
-      </x:c>
-      <x:c r="I72" s="126" t="n">
+      <x:c r="H72" s="140" t="str">
+        <x:v>Post-MVP</x:v>
+      </x:c>
+      <x:c r="I72" s="140" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="J72" s="126" t="str">
+      <x:c r="J72" s="140" t="str">
         <x:v>US-003, US-004, US-055</x:v>
       </x:c>
-      <x:c r="K72" s="126" t="str">
+      <x:c r="K72" s="140" t="str">
         <x:v>Each device exposes a recognizable product name plus stable four-character instance ID; two devices are distinguishable without UID/MAC leakage</x:v>
       </x:c>
-      <x:c r="L72" s="126" t="str">
+      <x:c r="L72" s="140" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-007-ACCEPTANCE / MCP-US-068</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="52" customHeight="1">
-      <x:c r="A73" s="137" t="str">
+      <x:c r="A73" s="127" t="str">
         <x:v>MCP-US-069</x:v>
       </x:c>
-      <x:c r="B73" s="137" t="str">
+      <x:c r="B73" s="127" t="str">
         <x:v>MCP-EPIC-010</x:v>
       </x:c>
-      <x:c r="C73" s="137" t="str">
+      <x:c r="C73" s="127" t="str">
         <x:v>External I2C Status Display Adapter</x:v>
       </x:c>
-      <x:c r="D73" s="137" t="str">
+      <x:c r="D73" s="127" t="str">
         <x:v>Embedded/Web</x:v>
       </x:c>
-      <x:c r="E73" s="137" t="str">
+      <x:c r="E73" s="127" t="str">
         <x:v>Should</x:v>
       </x:c>
-      <x:c r="F73" s="137" t="str">
+      <x:c r="F73" s="127" t="str">
         <x:v>Backlog</x:v>
       </x:c>
-      <x:c r="G73" s="137" t="str">
+      <x:c r="G73" s="127" t="str">
         <x:v>Post-MVP</x:v>
       </x:c>
-      <x:c r="H73" s="137" t="str">
+      <x:c r="H73" s="127" t="str">
         <x:v>Later</x:v>
       </x:c>
-      <x:c r="I73" s="137" t="n">
+      <x:c r="I73" s="127" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="J73" s="137" t="str">
+      <x:c r="J73" s="127" t="str">
         <x:v>US-004, US-022</x:v>
       </x:c>
-      <x:c r="K73" s="137" t="str">
+      <x:c r="K73" s="127" t="str">
         <x:v>Capability-gated SSD1306/similar display shows rate-limited status; absence never changes synth behavior</x:v>
       </x:c>
-      <x:c r="L73" s="137" t="str">
+      <x:c r="L73" s="127" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-007-ACCEPTANCE-START / MCP-US-069</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="52" customHeight="1">
-      <x:c r="A74" s="138" t="str">
+      <x:c r="A74" s="140" t="str">
         <x:v>MCP-US-070</x:v>
       </x:c>
-      <x:c r="B74" s="138" t="str">
+      <x:c r="B74" s="140" t="str">
         <x:v>MCP-EPIC-010</x:v>
       </x:c>
-      <x:c r="C74" s="138" t="str">
+      <x:c r="C74" s="140" t="str">
         <x:v>Physical Chip Transport And Capability Abstraction</x:v>
       </x:c>
-      <x:c r="D74" s="138" t="str">
+      <x:c r="D74" s="140" t="str">
         <x:v>Solution Architect</x:v>
       </x:c>
-      <x:c r="E74" s="138" t="str">
+      <x:c r="E74" s="140" t="str">
         <x:v>Should</x:v>
       </x:c>
-      <x:c r="F74" s="138" t="str">
+      <x:c r="F74" s="140" t="str">
         <x:v>Backlog</x:v>
       </x:c>
-      <x:c r="G74" s="138" t="str">
+      <x:c r="G74" s="140" t="str">
         <x:v>Post-MVP</x:v>
       </x:c>
-      <x:c r="H74" s="138" t="str">
+      <x:c r="H74" s="140" t="str">
         <x:v>Later</x:v>
       </x:c>
-      <x:c r="I74" s="138" t="n">
+      <x:c r="I74" s="140" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="J74" s="138" t="str">
+      <x:c r="J74" s="140" t="str">
         <x:v>US-004, US-034</x:v>
       </x:c>
-      <x:c r="K74" s="138" t="str">
+      <x:c r="K74" s="140" t="str">
         <x:v>Class-based GPIO, I2C-expander and SPI transport ports are capability-gated without chip or pin constants</x:v>
       </x:c>
-      <x:c r="L74" s="138" t="str">
+      <x:c r="L74" s="140" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-007-ACCEPTANCE-START / MCP-US-070</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="52" customHeight="1">
-      <x:c r="A75" s="137" t="str">
+      <x:c r="A75" s="127" t="str">
         <x:v>MCP-US-071</x:v>
       </x:c>
-      <x:c r="B75" s="137" t="str">
+      <x:c r="B75" s="127" t="str">
         <x:v>MCP-EPIC-010</x:v>
       </x:c>
-      <x:c r="C75" s="137" t="str">
+      <x:c r="C75" s="127" t="str">
         <x:v>Physical SN76489 Hardware Adapter</x:v>
       </x:c>
-      <x:c r="D75" s="137" t="str">
+      <x:c r="D75" s="127" t="str">
         <x:v>DSP/Chip Engineer</x:v>
       </x:c>
-      <x:c r="E75" s="137" t="str">
+      <x:c r="E75" s="127" t="str">
         <x:v>Should</x:v>
       </x:c>
-      <x:c r="F75" s="137" t="str">
+      <x:c r="F75" s="127" t="str">
         <x:v>Backlog</x:v>
       </x:c>
-      <x:c r="G75" s="137" t="str">
+      <x:c r="G75" s="127" t="str">
         <x:v>Post-MVP</x:v>
       </x:c>
-      <x:c r="H75" s="137" t="str">
+      <x:c r="H75" s="127" t="str">
         <x:v>Later</x:v>
       </x:c>
-      <x:c r="I75" s="137" t="n">
+      <x:c r="I75" s="127" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="J75" s="137" t="str">
+      <x:c r="J75" s="127" t="str">
         <x:v>US-017, US-070</x:v>
       </x:c>
-      <x:c r="K75" s="137" t="str">
+      <x:c r="K75" s="127" t="str">
         <x:v>Verified chip identity, levels, clock and bus sequences drive hardware; failures fall back to emulation</x:v>
       </x:c>
-      <x:c r="L75" s="137" t="str">
+      <x:c r="L75" s="127" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-007-ACCEPTANCE-START / MCP-US-071</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="52" customHeight="1">
-      <x:c r="A76" s="138" t="str">
+      <x:c r="A76" s="140" t="str">
         <x:v>MCP-US-072</x:v>
       </x:c>
-      <x:c r="B76" s="138" t="str">
+      <x:c r="B76" s="140" t="str">
         <x:v>MCP-EPIC-010</x:v>
       </x:c>
-      <x:c r="C76" s="138" t="str">
+      <x:c r="C76" s="140" t="str">
         <x:v>Physical SID6581 Feasibility And Adapter</x:v>
       </x:c>
-      <x:c r="D76" s="138" t="str">
+      <x:c r="D76" s="140" t="str">
         <x:v>DSP/Chip Engineer</x:v>
       </x:c>
-      <x:c r="E76" s="138" t="str">
+      <x:c r="E76" s="140" t="str">
         <x:v>Should</x:v>
       </x:c>
-      <x:c r="F76" s="138" t="str">
+      <x:c r="F76" s="140" t="str">
         <x:v>Backlog</x:v>
       </x:c>
-      <x:c r="G76" s="138" t="str">
+      <x:c r="G76" s="140" t="str">
         <x:v>Post-MVP</x:v>
       </x:c>
-      <x:c r="H76" s="138" t="str">
+      <x:c r="H76" s="140" t="str">
         <x:v>Later</x:v>
       </x:c>
-      <x:c r="I76" s="138" t="n">
+      <x:c r="I76" s="140" t="n">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="J76" s="138" t="str">
+      <x:c r="J76" s="140" t="str">
         <x:v>US-038, US-070</x:v>
       </x:c>
-      <x:c r="K76" s="138" t="str">
+      <x:c r="K76" s="140" t="str">
         <x:v>Power, levels, clock, register bus and analog output receive a measured go/no-go before implementation</x:v>
       </x:c>
-      <x:c r="L76" s="138" t="str">
+      <x:c r="L76" s="140" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-007-ACCEPTANCE-START / MCP-US-072</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="52" customHeight="1">
-      <x:c r="A77" s="137" t="str">
+      <x:c r="A77" s="127" t="str">
         <x:v>MCP-US-073</x:v>
       </x:c>
-      <x:c r="B77" s="137" t="str">
+      <x:c r="B77" s="127" t="str">
         <x:v>MCP-EPIC-010</x:v>
       </x:c>
-      <x:c r="C77" s="137" t="str">
+      <x:c r="C77" s="127" t="str">
         <x:v>ArduinoOPL2 SPI Hardware Adapter</x:v>
       </x:c>
-      <x:c r="D77" s="137" t="str">
+      <x:c r="D77" s="127" t="str">
         <x:v>DSP/Chip Engineer</x:v>
       </x:c>
-      <x:c r="E77" s="137" t="str">
+      <x:c r="E77" s="127" t="str">
         <x:v>Should</x:v>
       </x:c>
-      <x:c r="F77" s="137" t="str">
+      <x:c r="F77" s="127" t="str">
         <x:v>Backlog</x:v>
       </x:c>
-      <x:c r="G77" s="137" t="str">
+      <x:c r="G77" s="127" t="str">
         <x:v>Post-MVP</x:v>
       </x:c>
-      <x:c r="H77" s="137" t="str">
+      <x:c r="H77" s="127" t="str">
         <x:v>Later</x:v>
       </x:c>
-      <x:c r="I77" s="137" t="n">
+      <x:c r="I77" s="127" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="J77" s="137" t="str">
+      <x:c r="J77" s="127" t="str">
         <x:v>US-041, US-070</x:v>
       </x:c>
-      <x:c r="K77" s="137" t="str">
+      <x:c r="K77" s="127" t="str">
         <x:v>DhrBaksteen SPI contract and license are reviewed and verified by real HIL without coupling bus and emulator logic</x:v>
       </x:c>
-      <x:c r="L77" s="137" t="str">
+      <x:c r="L77" s="127" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-007-ACCEPTANCE-START / MCP-US-073</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="52" customHeight="1">
-      <x:c r="A78" s="138" t="str">
+      <x:c r="A78" s="140" t="str">
         <x:v>MCP-US-074</x:v>
       </x:c>
-      <x:c r="B78" s="138" t="str">
+      <x:c r="B78" s="140" t="str">
         <x:v>MCP-EPIC-010</x:v>
       </x:c>
-      <x:c r="C78" s="138" t="str">
+      <x:c r="C78" s="140" t="str">
         <x:v>Emulated Or Physical Core Backend Selection And Fallback</x:v>
       </x:c>
-      <x:c r="D78" s="138" t="str">
+      <x:c r="D78" s="140" t="str">
         <x:v>Solution Architect/DSP</x:v>
       </x:c>
-      <x:c r="E78" s="138" t="str">
+      <x:c r="E78" s="140" t="str">
         <x:v>Should</x:v>
       </x:c>
-      <x:c r="F78" s="138" t="str">
+      <x:c r="F78" s="140" t="str">
         <x:v>Backlog</x:v>
       </x:c>
-      <x:c r="G78" s="138" t="str">
+      <x:c r="G78" s="140" t="str">
         <x:v>Post-MVP</x:v>
       </x:c>
-      <x:c r="H78" s="138" t="str">
+      <x:c r="H78" s="140" t="str">
         <x:v>Later</x:v>
       </x:c>
-      <x:c r="I78" s="138" t="n">
+      <x:c r="I78" s="140" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="J78" s="138" t="str">
+      <x:c r="J78" s="140" t="str">
         <x:v>US-034, US-070, one physical adapter</x:v>
       </x:c>
-      <x:c r="K78" s="138" t="str">
+      <x:c r="K78" s="140" t="str">
         <x:v>Config/web selects emulated or physical per core; emulation is default/fallback and physical mode avoids duplicate rendering</x:v>
       </x:c>
-      <x:c r="L78" s="138" t="str">
+      <x:c r="L78" s="140" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-007-ACCEPTANCE-START / MCP-US-074</x:v>
       </x:c>
     </x:row>
@@ -4203,7 +4223,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ea335e9402f4f6c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82a0242ac61e4764"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4270,7 +4290,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="F5" s="23" t="str">
-        <x:v>Veilige, draagbare basis en konfigurasiegrens</x:v>
+        <x:v>MVP enablers: safe boot, board profile and configuration boundary</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="32" customHeight="1">
@@ -4293,7 +4313,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="F6" s="24" t="str">
-        <x:v>USB, BLE en DIN/UART MIDI; guitar slides, kontroles en clock</x:v>
+        <x:v>MVP USB-MIDI/Note semantics; clock, BLE, DIN and guitar expression post-MVP</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="32" customHeight="1">
@@ -4316,7 +4336,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F7" s="24" t="str">
-        <x:v>MAX98357 mono eerste; D1-basiskern, SN76489 en latere stereo</x:v>
+        <x:v>Standalone I2S preflight and D1 first; SN76489/SID/OPL/stereo post-MVP</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="32" customHeight="1">
@@ -4431,7 +4451,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F12" s="25" t="str">
-        <x:v>Host/HIL, BLE-tweedebord, kruisplatform en release</x:v>
+        <x:v>MVP host/HIL and audible Logic acceptance; cross-platform polish post-MVP</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="44" customHeight="1">
@@ -4487,7 +4507,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd85fc2c2154d4954"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f8ff8dc40e04d41"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4512,7 +4532,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>32 geregistreerde risiko's; fisiese-chip skade en backend-fallback is eksplisiet post-MVP beheer</x:v>
+        <x:v>33 geregistreerde risiko's; onafhanklike I2S-diagnose se profiel-drift word eksplisiet beheer</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -4727,7 +4747,7 @@
         <x:v>R-009</x:v>
       </x:c>
       <x:c r="B13" s="24" t="str">
-        <x:v>Multi-core oorskry CPU/RAM</x:v>
+        <x:v>Multi-core exceeds CPU/RAM and affects audio</x:v>
       </x:c>
       <x:c r="C13" s="24" t="str">
         <x:v>High</x:v>
@@ -4736,13 +4756,13 @@
         <x:v>High</x:v>
       </x:c>
       <x:c r="E13" s="24" t="str">
-        <x:v>DSP</x:v>
+        <x:v>DSP/Architect</x:v>
       </x:c>
       <x:c r="F13" s="24" t="str">
-        <x:v>Een kern eerste; twee verskillende kerne slegs na resource gate en MCP-US-061 telemetry</x:v>
+        <x:v>Close single-core D1 MVP first; measure each post-MVP multi-core expansion and reject unsafe capacity deterministically</x:v>
       </x:c>
       <x:c r="G13" s="24" t="str">
-        <x:v>Open</x:v>
+        <x:v>Post-MVP - risk accepted</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="38" customHeight="1">
@@ -5049,19 +5069,19 @@
         <x:v>R-023</x:v>
       </x:c>
       <x:c r="B27" s="83" t="str">
-        <x:v>BLE-MIDI is Must, maar die primere ESP32-S2 het geen native BLE nie</x:v>
+        <x:v>Primary ESP32-S2 has no native BLE support</x:v>
       </x:c>
       <x:c r="C27" s="83" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="D27" s="83" t="str">
-        <x:v>High</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="E27" s="83" t="str">
         <x:v>Architect/Embedded</x:v>
       </x:c>
       <x:c r="F27" s="83" t="str">
-        <x:v>Capability gate; tweede BLE-bordprofiel in US-052 en positiewe HIL in US-062</x:v>
+        <x:v>BLE is post-MVP; capability gate keeps USB stable; later select a BLE-capable board in US-052/062</x:v>
       </x:c>
       <x:c r="G27" s="83" t="str">
         <x:v>Controlled</x:v>
@@ -5225,7 +5245,7 @@
         <x:v>Stable non-secret four-character instance ID, collision rule and two-device DAW acceptance in US-068</x:v>
       </x:c>
       <x:c r="G34" s="126" t="str">
-        <x:v>Backlog - US-068</x:v>
+        <x:v>Post-MVP - US-068</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="48" customHeight="1">
@@ -5272,6 +5292,29 @@
       </x:c>
       <x:c r="G36" s="138" t="str">
         <x:v>Later - US-074</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="48" customHeight="1">
+      <x:c r="A37" s="142" t="str">
+        <x:v>R-033</x:v>
+      </x:c>
+      <x:c r="B37" s="142" t="str">
+        <x:v>Standalone I2S diagnostic drifts from the production AudioOutput profile</x:v>
+      </x:c>
+      <x:c r="C37" s="142" t="str">
+        <x:v>Medium</x:v>
+      </x:c>
+      <x:c r="D37" s="142" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="E37" s="142" t="str">
+        <x:v>Architect/QA/HIL</x:v>
+      </x:c>
+      <x:c r="F37" s="142" t="str">
+        <x:v>Same profile field names, AST/import and frequency tests, paired MAX98357 HIL, no shared synth-runtime import</x:v>
+      </x:c>
+      <x:c r="G37" s="142" t="str">
+        <x:v>Controlled in US-016</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5301,7 +5344,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e19665bb2134742"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45f9eabe879e4fa5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5497,7 +5540,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb18fc9a79c14d0d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb203d2a4fb04fdf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5991,7 +6034,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5a4edd19c644ba6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R175a54341c2e4e9f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(us014): add block audio output contract
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rf6f88ae00d934a50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R1b3f7cd50645453a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="R400cdd6a1f3e4cdb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R135db6911b98465d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R1089bb58a2874c1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R36160fdbbe1045f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R16c89735f3f4420d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R4652369bc44e4462"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Redb5d6fda15c4574"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="Rfb875143392848fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R0723c101fe3b4abf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R0c37ddd3098e4c7f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1095,7 +1095,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="102" t="str">
-        <x:v>Sprint 2 | scope v0.20.0 | runtime v0.12.3 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
+        <x:v>Sprint 2 | scope v0.21.0 | runtime v0.13.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
       </x:c>
       <x:c r="B2" s="103"/>
       <x:c r="C2" s="103"/>
@@ -1141,7 +1141,7 @@
       </x:c>
       <x:c r="C5" s="85"/>
       <x:c r="D5" s="110" t="str">
-        <x:v>1. US-005 config/geheimegrens fisies aanvaar</x:v>
+        <x:v>1. US-005 config en US-014 blok-AudioOutput gesluit</x:v>
       </x:c>
       <x:c r="E5" s="110"/>
       <x:c r="F5" s="110"/>
@@ -1154,11 +1154,11 @@
       </x:c>
       <x:c r="B6" s="114" t="n">
         <x:f>COUNTIF('Backlog'!$F$5:$F$200,"Done")</x:f>
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C6" s="85"/>
       <x:c r="D6" s="111" t="str">
-        <x:v>2. Bou US-014 AudioOutput; daarna US-016 G-C-D I2S-preflight</x:v>
+        <x:v>2. Bou en hoor-toets US-016 standalone G-C-D/MAX98357</x:v>
       </x:c>
       <x:c r="E6" s="111"/>
       <x:c r="F6" s="111"/>
@@ -1253,7 +1253,7 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="119" t="str">
-        <x:v>91 tests GREEN | USB-MIDI HIL PASS | US-005 UNSET-HIL PASS | aktief: US-014 AudioOutput</x:v>
+        <x:v>99 tests GREEN | US-005 HIL PASS | US-014 AudioOutput DONE | volgende: US-016 hoorbare I2S</x:v>
       </x:c>
       <x:c r="B13" s="120"/>
       <x:c r="C13" s="120"/>
@@ -1348,7 +1348,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Bron: docs/user_stories_v0.1.0.md v0.20.0 | 74 stories | 16-story bevrore MVP Acceptance Set</x:v>
+        <x:v>Bron: docs/user_stories_v0.1.0.md v0.21.0 | 74 stories | 16-story bevrore MVP Acceptance Set</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -1900,13 +1900,13 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="F18" s="24" t="str">
-        <x:v>Backlog</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G18" s="24" t="str">
         <x:v>Sprint 3</x:v>
       </x:c>
       <x:c r="H18" s="24" t="str">
-        <x:v>MVP-Enabler</x:v>
+        <x:v>MVP-Enabler (Done)</x:v>
       </x:c>
       <x:c r="I18" s="65" t="n">
         <x:v>5</x:v>
@@ -1915,10 +1915,10 @@
         <x:v>US-002</x:v>
       </x:c>
       <x:c r="K18" s="24" t="str">
-        <x:v>Kernlogika kan sonder fisiese klank host-getoets word</x:v>
+        <x:v>Bounded interleaved signed-16 PCM blocks, mono/stereo format, Null/Memory outputs, application integration and 17-file deploy manifest pass 99 host tests; no physical audio claim</x:v>
       </x:c>
       <x:c r="L18" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-014</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-014-START / v0.13.0</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="38" customHeight="1">
@@ -4239,7 +4239,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76654acddac14138"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55c413793e08431e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4349,7 +4349,7 @@
       </x:c>
       <x:c r="E7" s="65" t="n">
         <x:f>COUNTIFS('Backlog'!$B$5:$B$200,A7,'Backlog'!$F$5:$F$200,"Done")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F7" s="24" t="str">
         <x:v>Standalone I2S preflight and D1 first; SN76489/SID/OPL/stereo post-MVP</x:v>
@@ -4523,7 +4523,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c3d1fa5b71d4541"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d33e0183d314ea4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5383,7 +5383,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67be7e6abe204775"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea02067083e24529"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5579,7 +5579,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re29fbd01fe714688"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb009408e4e064028"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6073,7 +6073,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree582e3e91704933"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19d07d0666fb45d0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(us016): add standalone I2S diagnostic
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R16c89735f3f4420d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R4652369bc44e4462"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Redb5d6fda15c4574"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="Rfb875143392848fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R0723c101fe3b4abf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R0c37ddd3098e4c7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R7bf0f35732a44b6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="Ref7d6f1b021b435b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="R8f3799a05f9b411f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R07c0f65bba0d4591"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R9298cc88129841fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R1443da0938404e81"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1095,7 +1095,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="102" t="str">
-        <x:v>Sprint 2 | scope v0.21.0 | runtime v0.13.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
+        <x:v>Sprint 3 | scope v0.22.0 | runtime v0.14.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
       </x:c>
       <x:c r="B2" s="103"/>
       <x:c r="C2" s="103"/>
@@ -1141,7 +1141,7 @@
       </x:c>
       <x:c r="C5" s="85"/>
       <x:c r="D5" s="110" t="str">
-        <x:v>1. US-005 config en US-014 blok-AudioOutput gesluit</x:v>
+        <x:v>1. Deploy/run US-016 standalone i2s_test.py</x:v>
       </x:c>
       <x:c r="E5" s="110"/>
       <x:c r="F5" s="110"/>
@@ -1158,7 +1158,7 @@
       </x:c>
       <x:c r="C6" s="85"/>
       <x:c r="D6" s="111" t="str">
-        <x:v>2. Bou en hoor-toets US-016 standalone G-C-D/MAX98357</x:v>
+        <x:v>2. Bevestig G-C-D hoorbaar, serial PASS en code.py-herstel</x:v>
       </x:c>
       <x:c r="E6" s="111"/>
       <x:c r="F6" s="111"/>
@@ -1253,7 +1253,7 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="119" t="str">
-        <x:v>99 tests GREEN | US-005 HIL PASS | US-014 AudioOutput DONE | volgende: US-016 hoorbare I2S</x:v>
+        <x:v>103 tests GREEN | US-016 In Review | menslike G-C-D/MAX98357 hoorbare HIL benodig</x:v>
       </x:c>
       <x:c r="B13" s="120"/>
       <x:c r="C13" s="120"/>
@@ -1348,7 +1348,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Bron: docs/user_stories_v0.1.0.md v0.21.0 | 74 stories | 16-story bevrore MVP Acceptance Set</x:v>
+        <x:v>Bron: docs/user_stories_v0.1.0.md v0.22.0 | 74 stories | 16-story bevrore MVP Acceptance Set</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -1976,7 +1976,7 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="F20" s="24" t="str">
-        <x:v>Backlog</x:v>
+        <x:v>In Review</x:v>
       </x:c>
       <x:c r="G20" s="24" t="str">
         <x:v>Sprint 3</x:v>
@@ -1991,10 +1991,10 @@
         <x:v>US-004, US-014</x:v>
       </x:c>
       <x:c r="K20" s="24" t="str">
-        <x:v>Class-based device/i2s_test.py imports no synth package/global state; G3-C4-D4 square waves pass MAX98357 HIL, release I2S and complete a 30-minute smoke</x:v>
+        <x:v>v0.14.0 standalone class-based G3-C4-D4 RawSample/I2SOut diagnostic passes 103 host tests; audible MAX98357 PASS, runtime recovery and 30-minute smoke await HIL</x:v>
       </x:c>
       <x:c r="L20" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MVP-SCOPE-REDUCTION-001 / MCP-US-016</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-016-START / v0.14.0</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="38" customHeight="1">
@@ -4239,7 +4239,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R55c413793e08431e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf82424aacb74532"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4523,7 +4523,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d33e0183d314ea4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd57fee021e78450a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5383,7 +5383,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea02067083e24529"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd3eff62c61d4517"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5579,7 +5579,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb009408e4e064028"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ba9b13579604640"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6073,7 +6073,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19d07d0666fb45d0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1af7938ac9584d5b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(us016): record audible I2S acceptance
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R7bf0f35732a44b6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="Ref7d6f1b021b435b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="R8f3799a05f9b411f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R07c0f65bba0d4591"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R9298cc88129841fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R1443da0938404e81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R4d81a6ee5b2e4038"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="Rbfc4a4e6adbe4946"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="R5f73dde77147499c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R935b331ffd154596"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R3558baaa673c4660"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R381a1ea78fba469c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1095,7 +1095,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="102" t="str">
-        <x:v>Sprint 3 | scope v0.22.0 | runtime v0.14.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
+        <x:v>Sprint 3 | scope v0.23.0 | runtime v0.14.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
       </x:c>
       <x:c r="B2" s="103"/>
       <x:c r="C2" s="103"/>
@@ -1141,7 +1141,7 @@
       </x:c>
       <x:c r="C5" s="85"/>
       <x:c r="D5" s="110" t="str">
-        <x:v>1. Deploy/run US-016 standalone i2s_test.py</x:v>
+        <x:v>1. Begin US-063 Portable D1 Baseline Synth Core</x:v>
       </x:c>
       <x:c r="E5" s="110"/>
       <x:c r="F5" s="110"/>
@@ -1154,11 +1154,11 @@
       </x:c>
       <x:c r="B6" s="114" t="n">
         <x:f>COUNTIF('Backlog'!$F$5:$F$200,"Done")</x:f>
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C6" s="85"/>
       <x:c r="D6" s="111" t="str">
-        <x:v>2. Bevestig G-C-D hoorbaar, serial PASS en code.py-herstel</x:v>
+        <x:v>2. RED: D1 sine/saw/square + Note On/Off kontrakte</x:v>
       </x:c>
       <x:c r="E6" s="111"/>
       <x:c r="F6" s="111"/>
@@ -1253,7 +1253,7 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="119" t="str">
-        <x:v>103 tests GREEN | US-016 In Review | menslike G-C-D/MAX98357 hoorbare HIL benodig</x:v>
+        <x:v>103 tests GREEN | US-016 DONE | Wemos S2 + MAX98357A hoorbare G-C-D HIL PASS</x:v>
       </x:c>
       <x:c r="B13" s="120"/>
       <x:c r="C13" s="120"/>
@@ -1348,7 +1348,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Bron: docs/user_stories_v0.1.0.md v0.22.0 | 74 stories | 16-story bevrore MVP Acceptance Set</x:v>
+        <x:v>Bron: docs/user_stories_v0.1.0.md v0.23.0 | 74 stories | 16-story bevrore MVP Acceptance Set</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -1976,7 +1976,7 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="F20" s="24" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G20" s="24" t="str">
         <x:v>Sprint 3</x:v>
@@ -1991,10 +1991,10 @@
         <x:v>US-004, US-014</x:v>
       </x:c>
       <x:c r="K20" s="24" t="str">
-        <x:v>v0.14.0 standalone class-based G3-C4-D4 RawSample/I2SOut diagnostic passes 103 host tests; audible MAX98357 PASS, runtime recovery and 30-minute smoke await HIL</x:v>
+        <x:v>PASS 2026-07-16: Wemos S2/MAX98357A played audible mono G3-C4-D4; serial notes=3, heap 2056512-&gt;2056192, 103 host tests; long burn-in tracked by US-051/US-057</x:v>
       </x:c>
       <x:c r="L20" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-016-START / v0.14.0</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-016-HIL-PASS-001 / v0.14.0</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="38" customHeight="1">
@@ -4239,7 +4239,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf82424aacb74532"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb309077a227642e3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4349,7 +4349,7 @@
       </x:c>
       <x:c r="E7" s="65" t="n">
         <x:f>COUNTIFS('Backlog'!$B$5:$B$200,A7,'Backlog'!$F$5:$F$200,"Done")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="F7" s="24" t="str">
         <x:v>Standalone I2S preflight and D1 first; SN76489/SID/OPL/stereo post-MVP</x:v>
@@ -4523,7 +4523,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd57fee021e78450a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1286278d767e4320"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5383,7 +5383,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd3eff62c61d4517"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf3565ed702b4a82"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5579,7 +5579,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ba9b13579604640"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb172528768f748a8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6073,7 +6073,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1af7938ac9584d5b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdeae28b503ae4a0c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(us063): add portable D1 baseline core
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R4d81a6ee5b2e4038"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="Rbfc4a4e6adbe4946"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="R5f73dde77147499c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R935b331ffd154596"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R3558baaa673c4660"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R381a1ea78fba469c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R540dae95685b41ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R6400a712d07c4ceb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Reb5064f75804472b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="Rb218b690836548ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="Rffe0288201ff4195"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R29df99fc2ad4434d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1095,7 +1095,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="102" t="str">
-        <x:v>Sprint 3 | scope v0.23.0 | runtime v0.14.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
+        <x:v>Sprint 3 | scope v0.24.0 | runtime v0.15.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
       </x:c>
       <x:c r="B2" s="103"/>
       <x:c r="C2" s="103"/>
@@ -1141,7 +1141,7 @@
       </x:c>
       <x:c r="C5" s="85"/>
       <x:c r="D5" s="110" t="str">
-        <x:v>1. Begin US-063 Portable D1 Baseline Synth Core</x:v>
+        <x:v>1. Product Owner run d1-diagnose en bevestig PASS</x:v>
       </x:c>
       <x:c r="E5" s="110"/>
       <x:c r="F5" s="110"/>
@@ -1158,7 +1158,7 @@
       </x:c>
       <x:c r="C6" s="85"/>
       <x:c r="D6" s="111" t="str">
-        <x:v>2. RED: D1 sine/saw/square + Note On/Off kontrakte</x:v>
+        <x:v>2. Sluit US-063; begin US-055 Logic/USB-MIDI/I2S integrasie</x:v>
       </x:c>
       <x:c r="E6" s="111"/>
       <x:c r="F6" s="111"/>
@@ -1253,7 +1253,7 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="119" t="str">
-        <x:v>103 tests GREEN | US-016 DONE | Wemos S2 + MAX98357A hoorbare G-C-D HIL PASS</x:v>
+        <x:v>114 tests GREEN | US-063 In Review | draagbare D1 sine/saw/square + Note On/Off</x:v>
       </x:c>
       <x:c r="B13" s="120"/>
       <x:c r="C13" s="120"/>
@@ -1348,7 +1348,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Bron: docs/user_stories_v0.1.0.md v0.23.0 | 74 stories | 16-story bevrore MVP Acceptance Set</x:v>
+        <x:v>Bron: docs/user_stories_v0.1.0.md v0.24.0 | 74 stories | 16-story bevrore MVP Acceptance Set</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -3762,7 +3762,7 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="F67" s="83" t="str">
-        <x:v>Backlog</x:v>
+        <x:v>In Review</x:v>
       </x:c>
       <x:c r="G67" s="83" t="str">
         <x:v>Sprint 3</x:v>
@@ -3777,10 +3777,10 @@
         <x:v>US-006, US-008, US-009, US-014, US-016</x:v>
       </x:c>
       <x:c r="K67" s="83" t="str">
-        <x:v>Portable sine/saw/square D1 handles Note On/Off, cleans up and passes a 30-minute smoke; no production-repo modification</x:v>
+        <x:v>v0.15.0 portable monophonic D1 sine/saw/square core: A4=440Hz, velocity, phase continuity, Note Off silence, continuous block rendering, d1-diagnose and 114 host tests GREEN; audible Logic/I2S remains US-055</x:v>
       </x:c>
       <x:c r="L67" s="83" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / SCOPE-AMENDMENT-002 / MCP-US-063</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-063-START / v0.15.0</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="48" customHeight="1">
@@ -4239,7 +4239,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb309077a227642e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb9b78f0adbe424b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4523,7 +4523,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1286278d767e4320"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e212193b2814c4f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5383,7 +5383,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf3565ed702b4a82"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R511337264f204be2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5579,7 +5579,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb172528768f748a8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08500c26c7c84ced"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6073,7 +6073,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdeae28b503ae4a0c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re04c87d7be0b4ad4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(us063): accept D1 core and add safe audio gate
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R540dae95685b41ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R6400a712d07c4ceb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Reb5064f75804472b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="Rb218b690836548ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="Rffe0288201ff4195"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R29df99fc2ad4434d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R47f47227acf34915"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R1595a50ed57c4a59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="R5cb34f372b4f4b42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="Re9fd5d0bc831409c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R11f0e66ac82a427d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R557077dda245416e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1095,7 +1095,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="102" t="str">
-        <x:v>Sprint 3 | scope v0.24.0 | runtime v0.15.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
+        <x:v>Sprint 3 | scope v0.25.0 | runtime v0.15.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
       </x:c>
       <x:c r="B2" s="103"/>
       <x:c r="C2" s="103"/>
@@ -1136,12 +1136,11 @@
         <x:v>Totale stories</x:v>
       </x:c>
       <x:c r="B5" s="113" t="n">
-        <x:f>COUNTA('Backlog'!$A$5:$A$200)</x:f>
-        <x:v>74</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="C5" s="85"/>
       <x:c r="D5" s="110" t="str">
-        <x:v>1. Product Owner run d1-diagnose en bevestig PASS</x:v>
+        <x:v>1. Ontkoppel direkte koptelefoon; verkry 4-8 ohm speaker</x:v>
       </x:c>
       <x:c r="E5" s="110"/>
       <x:c r="F5" s="110"/>
@@ -1153,12 +1152,11 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B6" s="114" t="n">
-        <x:f>COUNTIF('Backlog'!$F$5:$F$200,"Done")</x:f>
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C6" s="85"/>
       <x:c r="D6" s="111" t="str">
-        <x:v>2. Sluit US-063; begin US-055 Logic/USB-MIDI/I2S integrasie</x:v>
+        <x:v>2. US-075: software gain, startup mute en GAIN/SD-profiel</x:v>
       </x:c>
       <x:c r="E6" s="111"/>
       <x:c r="F6" s="111"/>
@@ -1175,7 +1173,7 @@
       </x:c>
       <x:c r="C7" s="85"/>
       <x:c r="D7" s="111" t="str">
-        <x:v>3. D1 sine/saw/square met korrekte Note On/Off</x:v>
+        <x:v>3. US-055: Logic External MIDI na veilige hoorbare D1</x:v>
       </x:c>
       <x:c r="E7" s="111"/>
       <x:c r="F7" s="111"/>
@@ -1187,12 +1185,11 @@
         <x:v>MVP acceptance-set</x:v>
       </x:c>
       <x:c r="B8" s="114" t="n">
-        <x:f>COUNTIF('Backlog'!$H$5:$H$200,"MVP-Must")+COUNTIF('Backlog'!$H$5:$H$200,"MVP-Enabler")+COUNTIF('Backlog'!$H$5:$H$200,"MVP-Enabler (Done)")+COUNTIF('Backlog'!$H$5:$H$200,"MVP-Enabler (In Review)")</x:f>
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C8" s="85"/>
       <x:c r="D8" s="112" t="str">
-        <x:v>4. Logic External MIDI na hoorbare D1 op verwysingsbord</x:v>
+        <x:v>4. US-057: release; daarna SN76489 en volgende kerne</x:v>
       </x:c>
       <x:c r="E8" s="112"/>
       <x:c r="F8" s="112"/>
@@ -1208,9 +1205,7 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="C9" s="85"/>
-      <x:c r="D9" s="116" t="str">
-        <x:v>5. Release; daarna SN76489 en volgende kerne</x:v>
-      </x:c>
+      <x:c r="D9" s="116" t="str"/>
       <x:c r="E9" s="116"/>
       <x:c r="F9" s="116"/>
       <x:c r="G9" s="116"/>
@@ -1253,7 +1248,7 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="119" t="str">
-        <x:v>114 tests GREEN | US-063 In Review | draagbare D1 sine/saw/square + Note On/Off</x:v>
+        <x:v>114 tests GREEN | US-063 DONE | US-075 veilige speaker/volume-hek volgende</x:v>
       </x:c>
       <x:c r="B13" s="120"/>
       <x:c r="C13" s="120"/>
@@ -1348,7 +1343,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Bron: docs/user_stories_v0.1.0.md v0.24.0 | 74 stories | 16-story bevrore MVP Acceptance Set</x:v>
+        <x:v>Bron: docs/user_stories_v0.1.0.md v0.25.0 | 75 stories | 17-story veiligheidsaangepaste MVP Acceptance Set</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -3145,7 +3140,7 @@
         <x:v>MCP-EPIC-007</x:v>
       </x:c>
       <x:c r="C51" s="24" t="str">
-        <x:v>Pedal Power And Audio Protection</x:v>
+        <x:v>Pedal Power, Safe Volume And Audio Protection</x:v>
       </x:c>
       <x:c r="D51" s="24" t="str">
         <x:v>Hardware/DSP</x:v>
@@ -3166,10 +3161,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="J51" s="24" t="str">
-        <x:v>US-021</x:v>
+        <x:v>MCP-US-021, MCP-US-075</x:v>
       </x:c>
       <x:c r="K51" s="24" t="str">
-        <x:v>Krag, vlakke, filtering en beskerming is geskematiseer en gemeet</x:v>
+        <x:v>Power, speaker/headphone/line-out boundaries, gain or attenuation, mute, filtering, ESD and polarity protection are breadboarded and measured at documented safe test points</x:v>
       </x:c>
       <x:c r="L51" s="24" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-047</x:v>
@@ -3183,7 +3178,7 @@
         <x:v>MCP-EPIC-007</x:v>
       </x:c>
       <x:c r="C52" s="24" t="str">
-        <x:v>KiCad Reference PCB</x:v>
+        <x:v>KiCad Reference Pedal PCB</x:v>
       </x:c>
       <x:c r="D52" s="24" t="str">
         <x:v>Hardware/DSP</x:v>
@@ -3207,7 +3202,7 @@
         <x:v>US-047</x:v>
       </x:c>
       <x:c r="K52" s="24" t="str">
-        <x:v>Skematiese, PCB en BOM slaag ERC/DRC en bring-up-runbook</x:v>
+        <x:v>Hardware Engineer and experienced KiCad Product Owner deliver schematic, PCB, footprints, test points and BOM; ERC, DRC, bring-up and manufacturing outputs pass</x:v>
       </x:c>
       <x:c r="L52" s="24" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-048</x:v>
@@ -3470,10 +3465,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="J59" s="24" t="str">
-        <x:v>US-003, US-007, US-009, US-014, US-016, US-063</x:v>
+        <x:v>MCP-US-003, MCP-US-007, MCP-US-009, MCP-US-014, MCP-US-016, MCP-US-063, MCP-US-075</x:v>
       </x:c>
       <x:c r="K59" s="24" t="str">
-        <x:v>Logic selects the board and the user hears D1; the reference board then passes an 8-hour USB-MIDI/audio/heap burn-in</x:v>
+        <x:v>Logic selects the board as External MIDI destination and the user hears D1 through the approved safe output profile; the board then passes the 8-hour USB MIDI, audio and heap burn-in</x:v>
       </x:c>
       <x:c r="L59" s="24" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-055</x:v>
@@ -3546,7 +3541,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="J61" s="25" t="str">
-        <x:v>US-001 to US-009, US-014, US-016, US-050, US-051, US-055, US-063</x:v>
+        <x:v>US-001 to US-009, US-014, US-016, US-050, US-051, US-055, US-063, US-075</x:v>
       </x:c>
       <x:c r="K61" s="25" t="str">
         <x:v>Tag, release notes, known limitations and a passing 8-hour burn-in report accompany the Logic-to-audible-D1 demo</x:v>
@@ -3762,7 +3757,7 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="F67" s="83" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G67" s="83" t="str">
         <x:v>Sprint 3</x:v>
@@ -3777,10 +3772,10 @@
         <x:v>US-006, US-008, US-009, US-014, US-016</x:v>
       </x:c>
       <x:c r="K67" s="83" t="str">
-        <x:v>v0.15.0 portable monophonic D1 sine/saw/square core: A4=440Hz, velocity, phase continuity, Note Off silence, continuous block rendering, d1-diagnose and 114 host tests GREEN; audible Logic/I2S remains US-055</x:v>
+        <x:v>Product Owner accepted v0.15.0 d1-diagnose: sine, saw and square, A4=440Hz, velocity and final PASS; audible Logic/I2S remains US-055 after US-075</x:v>
       </x:c>
       <x:c r="L67" s="83" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-063-START / v0.15.0</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-063-HOST-ACCEPTED-001 / v0.15.0</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="48" customHeight="1">
@@ -4199,6 +4194,44 @@
       </x:c>
       <x:c r="L78" s="140" t="str">
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-007-ACCEPTANCE-START / MCP-US-074</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" t="str">
+        <x:v>MCP-US-075</x:v>
+      </x:c>
+      <x:c r="B79" t="str">
+        <x:v>MCP-EPIC-007</x:v>
+      </x:c>
+      <x:c r="C79" t="str">
+        <x:v>Safe Development Audio Load And Volume Gate</x:v>
+      </x:c>
+      <x:c r="D79" t="str">
+        <x:v>Hardware/DSP</x:v>
+      </x:c>
+      <x:c r="E79" t="str">
+        <x:v>Must</x:v>
+      </x:c>
+      <x:c r="F79" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="G79" t="str">
+        <x:v>Sprint 3</x:v>
+      </x:c>
+      <x:c r="H79" t="str">
+        <x:v>MVP-Enabler</x:v>
+      </x:c>
+      <x:c r="I79" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="J79" t="str">
+        <x:v>MCP-US-016, MCP-US-063</x:v>
+      </x:c>
+      <x:c r="K79" t="str">
+        <x:v>4-8 ohm speaker, low software master gain, startup mute and documented MAX98357 GAIN/SD profile are safely audible; no direct headphone, line-in or potentiometer across BTL output; separate DAC/headphone-amp decision</x:v>
+      </x:c>
+      <x:c r="L79" t="str">
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-063-HOST-ACCEPTED-001 / MCP-US-075</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4239,7 +4272,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reb9b78f0adbe424b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R339451d923f54eea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4349,7 +4382,7 @@
       </x:c>
       <x:c r="E7" s="65" t="n">
         <x:f>COUNTIFS('Backlog'!$B$5:$B$200,A7,'Backlog'!$F$5:$F$200,"Done")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F7" s="24" t="str">
         <x:v>Standalone I2S preflight and D1 first; SN76489/SID/OPL/stereo post-MVP</x:v>
@@ -4432,19 +4465,17 @@
         <x:v>DSP And Pedal Hardware</x:v>
       </x:c>
       <x:c r="C11" s="65" t="n">
-        <x:f>COUNTIF('Backlog'!$B$5:$B$200,A11)</x:f>
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D11" s="65" t="n">
-        <x:f>COUNTIFS('Backlog'!$B$5:$B$200,A11,'Backlog'!$E$5:$E$200,"Must")</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E11" s="65" t="n">
         <x:f>COUNTIFS('Backlog'!$B$5:$B$200,A11,'Backlog'!$F$5:$F$200,"Done")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F11" s="24" t="str">
-        <x:v>Laat-MVP DSP en pedaalhardeware</x:v>
+        <x:v>Safe audio load and volume gate first; pedal power, protection, enclosure and KiCad hardware follow after MVP</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="32" customHeight="1">
@@ -4523,7 +4554,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e212193b2814c4f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5636b533507242ae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4855,22 +4886,22 @@
         <x:v>R-013</x:v>
       </x:c>
       <x:c r="B17" s="24" t="str">
-        <x:v>MAX98357 bridge-tied uitset word geaard of as line-out gebruik</x:v>
+        <x:v>MAX98357 bridge-tied output is grounded, used as line-out, or drives a full-volume headphone close to the user</x:v>
       </x:c>
       <x:c r="C17" s="24" t="str">
-        <x:v>Medium</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="D17" s="24" t="str">
         <x:v>Critical</x:v>
       </x:c>
       <x:c r="E17" s="24" t="str">
-        <x:v>Hardware</x:v>
+        <x:v>Hardware/PO</x:v>
       </x:c>
       <x:c r="F17" s="24" t="str">
-        <x:v>Luidspreker tussen + en -; geen grond/line-input; HIL checklist</x:v>
+        <x:v>Disconnect direct TRS load; use 4-8 ohm speaker; never ground, feed line input or place a potentiometer across BTL output; add software gain, startup mute and GAIN/SD profile in US-075</x:v>
       </x:c>
       <x:c r="G17" s="24" t="str">
-        <x:v>Open</x:v>
+        <x:v>Impediment - MCP-US-075</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="38" customHeight="1">
@@ -5383,7 +5414,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R511337264f204be2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c0f065d602341d2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5579,7 +5610,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08500c26c7c84ced"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30f8779224214e2e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6073,7 +6104,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re04c87d7be0b4ad4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61a0573b7da6458f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(us075): add safe audio output gate
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R47f47227acf34915"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R1595a50ed57c4a59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="R5cb34f372b4f4b42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="Re9fd5d0bc831409c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R11f0e66ac82a427d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R557077dda245416e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R551b8b3104c842ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="Rdc6faae59e684d22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Rd9f6d05738144dcd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="Rf4524d525a7747d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="Rbc45aeadb92a4775"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R4b7a086187d64343"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1095,7 +1095,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="102" t="str">
-        <x:v>Sprint 3 | scope v0.25.0 | runtime v0.15.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
+        <x:v>Sprint 3 | scope v0.26.0 | runtime v0.16.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
       </x:c>
       <x:c r="B2" s="103"/>
       <x:c r="C2" s="103"/>
@@ -1140,7 +1140,7 @@
       </x:c>
       <x:c r="C5" s="85"/>
       <x:c r="D5" s="110" t="str">
-        <x:v>1. Ontkoppel direkte koptelefoon; verkry 4-8 ohm speaker</x:v>
+        <x:v>1. Verkry 4-8 ohm speaker; geen direkte koptelefoon-HIL</x:v>
       </x:c>
       <x:c r="E5" s="110"/>
       <x:c r="F5" s="110"/>
@@ -1156,7 +1156,7 @@
       </x:c>
       <x:c r="C6" s="85"/>
       <x:c r="D6" s="111" t="str">
-        <x:v>2. US-075: software gain, startup mute en GAIN/SD-profiel</x:v>
+        <x:v>2. Deploy v0.16.0; voer lae-volume i2s_test.py uit</x:v>
       </x:c>
       <x:c r="E6" s="111"/>
       <x:c r="F6" s="111"/>
@@ -1173,7 +1173,7 @@
       </x:c>
       <x:c r="C7" s="85"/>
       <x:c r="D7" s="111" t="str">
-        <x:v>3. US-055: Logic External MIDI na veilige hoorbare D1</x:v>
+        <x:v>3. PO aanvaar sagte G-C-D en serial PASS vir US-075</x:v>
       </x:c>
       <x:c r="E7" s="111"/>
       <x:c r="F7" s="111"/>
@@ -1189,7 +1189,7 @@
       </x:c>
       <x:c r="C8" s="85"/>
       <x:c r="D8" s="112" t="str">
-        <x:v>4. US-057: release; daarna SN76489 en volgende kerne</x:v>
+        <x:v>4. US-055: Logic External MIDI na veilige hoorbare D1</x:v>
       </x:c>
       <x:c r="E8" s="112"/>
       <x:c r="F8" s="112"/>
@@ -1248,7 +1248,7 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="119" t="str">
-        <x:v>114 tests GREEN | US-063 DONE | US-075 veilige speaker/volume-hek volgende</x:v>
+        <x:v>120 tests GREEN | US-075 IN REVIEW | veilige 4-8 ohm speaker-HIL nodig</x:v>
       </x:c>
       <x:c r="B13" s="120"/>
       <x:c r="C13" s="120"/>
@@ -1343,7 +1343,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Bron: docs/user_stories_v0.1.0.md v0.25.0 | 75 stories | 17-story veiligheidsaangepaste MVP Acceptance Set</x:v>
+        <x:v>Bron: docs/user_stories_v0.1.0.md v0.26.0 | 75 stories | 17-story veiligheidsaangepaste MVP Acceptance Set</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
@@ -4213,7 +4213,7 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="F79" t="str">
-        <x:v>Backlog</x:v>
+        <x:v>In Review</x:v>
       </x:c>
       <x:c r="G79" t="str">
         <x:v>Sprint 3</x:v>
@@ -4228,10 +4228,10 @@
         <x:v>MCP-US-016, MCP-US-063</x:v>
       </x:c>
       <x:c r="K79" t="str">
-        <x:v>4-8 ohm speaker, low software master gain, startup mute and documented MAX98357 GAIN/SD profile are safely audible; no direct headphone, line-in or potentiometer across BTL output; separate DAC/headphone-amp decision</x:v>
+        <x:v>v0.16.0 startup mute, 0.08 gain, 0.25 ceiling and low-volume I2S profile pass 120 host tests; Done waits for audible 4-8 ohm speaker HIL without direct headphone, line-in or potentiometer across BTL</x:v>
       </x:c>
       <x:c r="L79" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-063-HOST-ACCEPTED-001 / MCP-US-075</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-075-START / v0.16.0</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4272,7 +4272,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R339451d923f54eea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2adc196b0f124b0b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4554,7 +4554,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5636b533507242ae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42a2e23646e4412f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4898,10 +4898,10 @@
         <x:v>Hardware/PO</x:v>
       </x:c>
       <x:c r="F17" s="24" t="str">
-        <x:v>Disconnect direct TRS load; use 4-8 ohm speaker; never ground, feed line input or place a potentiometer across BTL output; add software gain, startup mute and GAIN/SD profile in US-075</x:v>
+        <x:v>v0.16.0 software gain and startup mute are green; disconnect direct TRS load; use 4-8 ohm speaker; never ground, feed line input or place a potentiometer across BTL output</x:v>
       </x:c>
       <x:c r="G17" s="24" t="str">
-        <x:v>Impediment - MCP-US-075</x:v>
+        <x:v>In Review - speaker HIL open</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="38" customHeight="1">
@@ -5414,7 +5414,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5c0f065d602341d2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8668ea3d32cb43b7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5610,7 +5610,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R30f8779224214e2e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cab79d4b4444c56"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6104,7 +6104,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61a0573b7da6458f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8039a29941a744ad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: close US-075 with prototype audio exception
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R551b8b3104c842ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="Rdc6faae59e684d22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Rd9f6d05738144dcd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="Rf4524d525a7747d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="Rbc45aeadb92a4775"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R4b7a086187d64343"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rba2e158f025a4348"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R1add1eddce294695"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Rcdd2e6360e1545b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R365eada3671c465b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R3227d4e4ff7d4b32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rd36d7f6ccf1147d7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1095,7 +1095,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="102" t="str">
-        <x:v>Sprint 3 | scope v0.26.0 | runtime v0.16.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
+        <x:v>Sprint 3 | scope v0.27.0 | runtime v0.16.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
       </x:c>
       <x:c r="B2" s="103"/>
       <x:c r="C2" s="103"/>
@@ -1136,11 +1136,11 @@
         <x:v>Totale stories</x:v>
       </x:c>
       <x:c r="B5" s="113" t="n">
-        <x:v>75</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C5" s="85"/>
       <x:c r="D5" s="110" t="str">
-        <x:v>1. Verkry 4-8 ohm speaker; geen direkte koptelefoon-HIL</x:v>
+        <x:v>1. US-075 PO-uitzondering aanvaar; geen produksie-veiligheidsclaim</x:v>
       </x:c>
       <x:c r="E5" s="110"/>
       <x:c r="F5" s="110"/>
@@ -1152,11 +1152,11 @@
         <x:v>Done</x:v>
       </x:c>
       <x:c r="B6" s="114" t="n">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C6" s="85"/>
       <x:c r="D6" s="111" t="str">
-        <x:v>2. Deploy v0.16.0; voer lae-volume i2s_test.py uit</x:v>
+        <x:v>2. Direkte TRS-koptelefoon bly prototipe-risiko; US-076 parkeer cleanup</x:v>
       </x:c>
       <x:c r="E6" s="111"/>
       <x:c r="F6" s="111"/>
@@ -1168,12 +1168,11 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="B7" s="114" t="n">
-        <x:f>COUNTIF('Backlog'!$F$5:$F$200,"In Progress")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C7" s="85"/>
       <x:c r="D7" s="111" t="str">
-        <x:v>3. PO aanvaar sagte G-C-D en serial PASS vir US-075</x:v>
+        <x:v>3. US-055: Logic USB-MIDI -&gt; D1-kern -&gt; I2S is volgende MVP-integrasie</x:v>
       </x:c>
       <x:c r="E7" s="111"/>
       <x:c r="F7" s="111"/>
@@ -1189,7 +1188,7 @@
       </x:c>
       <x:c r="C8" s="85"/>
       <x:c r="D8" s="112" t="str">
-        <x:v>4. US-055: Logic External MIDI na veilige hoorbare D1</x:v>
+        <x:v>4. US-057 volg na US-055 vir end-to-end MVP burn-in/acceptance</x:v>
       </x:c>
       <x:c r="E8" s="112"/>
       <x:c r="F8" s="112"/>
@@ -1248,7 +1247,7 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="119" t="str">
-        <x:v>120 tests GREEN | US-075 IN REVIEW | veilige 4-8 ohm speaker-HIL nodig</x:v>
+        <x:v>120 tests GREEN | US-075 DONE WITH PO EXCEPTION | US-055 NEXT</x:v>
       </x:c>
       <x:c r="B13" s="120"/>
       <x:c r="C13" s="120"/>
@@ -1343,8 +1342,19 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Bron: docs/user_stories_v0.1.0.md v0.26.0 | 75 stories | 17-story veiligheidsaangepaste MVP Acceptance Set</x:v>
-      </x:c>
+        <x:v>Bron: docs/user_stories_v0.1.0.md v0.27.0 | 76 stories | 17-story veiligheidsaangepaste MVP Acceptance Set + US-076 post-MVP cleanup</x:v>
+      </x:c>
+      <x:c r="B2"/>
+      <x:c r="C2"/>
+      <x:c r="D2"/>
+      <x:c r="E2"/>
+      <x:c r="F2"/>
+      <x:c r="G2"/>
+      <x:c r="H2"/>
+      <x:c r="I2"/>
+      <x:c r="J2"/>
+      <x:c r="K2"/>
+      <x:c r="L2"/>
     </x:row>
     <x:row r="4" ht="28" customHeight="1">
       <x:c r="A4" s="14" t="str">
@@ -4213,25 +4223,63 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="F79" t="str">
-        <x:v>In Review</x:v>
+        <x:v>Done</x:v>
       </x:c>
       <x:c r="G79" t="str">
         <x:v>Sprint 3</x:v>
       </x:c>
       <x:c r="H79" t="str">
-        <x:v>MVP-Enabler</x:v>
+        <x:v>MVP-Enabler (Done; PO exception)</x:v>
       </x:c>
       <x:c r="I79" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="J79" t="str">
-        <x:v>MCP-US-016, MCP-US-063</x:v>
+        <x:v>US-016</x:v>
       </x:c>
       <x:c r="K79" t="str">
-        <x:v>v0.16.0 startup mute, 0.08 gain, 0.25 ceiling and low-volume I2S profile pass 120 host tests; Done waits for audible 4-8 ohm speaker HIL without direct headphone, line-in or potentiometer across BTL</x:v>
+        <x:v>HIL: G-C-D hoorbaar via MAX98357A; PO aanvaar cheap TRS-headphone prototype risk; no production safety claim</x:v>
       </x:c>
       <x:c r="L79" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-075-START / v0.16.0</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-075-PO-EXCEPTION-ACCEPTED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" t="str">
+        <x:v>MCP-US-076</x:v>
+      </x:c>
+      <x:c r="B80" t="str">
+        <x:v>MCP-EPIC-007</x:v>
+      </x:c>
+      <x:c r="C80" t="str">
+        <x:v>Certified Speaker, Headphone And Pedal Output Cleanup</x:v>
+      </x:c>
+      <x:c r="D80" t="str">
+        <x:v>Hardware/DSP</x:v>
+      </x:c>
+      <x:c r="E80" t="str">
+        <x:v>Should</x:v>
+      </x:c>
+      <x:c r="F80" t="str">
+        <x:v>Backlog</x:v>
+      </x:c>
+      <x:c r="G80" t="str">
+        <x:v>Post-MVP</x:v>
+      </x:c>
+      <x:c r="H80" t="str">
+        <x:v>Later</x:v>
+      </x:c>
+      <x:c r="I80" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="J80" t="str">
+        <x:v>US-047, US-075</x:v>
+      </x:c>
+      <x:c r="K80" t="str">
+        <x:v>Gescheiden speaker/headphone/line-out ontwerp, load profiles, volume hardware en KiCad guidance zijn gevalideerd</x:v>
+      </x:c>
+      <x:c r="L80" t="str">
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-075-PO-EXCEPTION-ACCEPTED / MCP-US-076</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4272,7 +4320,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2adc196b0f124b0b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d845a9ed4da476b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4472,7 +4520,7 @@
       </x:c>
       <x:c r="E11" s="65" t="n">
         <x:f>COUNTIFS('Backlog'!$B$5:$B$200,A11,'Backlog'!$F$5:$F$200,"Done")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F11" s="24" t="str">
         <x:v>Safe audio load and volume gate first; pedal power, protection, enclosure and KiCad hardware follow after MVP</x:v>
@@ -4554,7 +4602,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42a2e23646e4412f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6080077e0b2c4098"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4886,22 +4934,22 @@
         <x:v>R-013</x:v>
       </x:c>
       <x:c r="B17" s="24" t="str">
-        <x:v>MAX98357 bridge-tied output is grounded, used as line-out, or drives a full-volume headphone close to the user</x:v>
+        <x:v>Directe TRS/headphone of verkeerde load kan MAX98357A, koptelefoon of gehoor beschadigen</x:v>
       </x:c>
       <x:c r="C17" s="24" t="str">
-        <x:v>High</x:v>
+        <x:v>Hoog</x:v>
       </x:c>
       <x:c r="D17" s="24" t="str">
-        <x:v>Critical</x:v>
+        <x:v>Middel</x:v>
       </x:c>
       <x:c r="E17" s="24" t="str">
-        <x:v>Hardware/PO</x:v>
+        <x:v>US-075 begrenst amplitude/software-startup; PO accepteert prototype met goedkope TRS-koptelefoon. Productieclaim blijft verboden tot US-076.</x:v>
       </x:c>
       <x:c r="F17" s="24" t="str">
-        <x:v>v0.16.0 software gain and startup mute are green; disconnect direct TRS load; use 4-8 ohm speaker; never ground, feed line input or place a potentiometer across BTL output</x:v>
+        <x:v>Aanvaard voor prototype; US-076 cleanup</x:v>
       </x:c>
       <x:c r="G17" s="24" t="str">
-        <x:v>In Review - speaker HIL open</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-075-PO-EXCEPTION-ACCEPTED</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="38" customHeight="1">
@@ -5414,7 +5462,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8668ea3d32cb43b7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba474dab399142ba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5610,7 +5658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cab79d4b4444c56"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7052d15838a6460a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6097,6 +6145,20 @@
         <x:v>https://github.com/Malvineous/pyopl</x:v>
       </x:c>
     </x:row>
+    <x:row r="37">
+      <x:c r="A37" t="str">
+        <x:v>2026-07-16</x:v>
+      </x:c>
+      <x:c r="B37" t="str">
+        <x:v>PO exception / HIL evidence</x:v>
+      </x:c>
+      <x:c r="C37" t="str">
+        <x:v>US-075 hoorbare G-C-D via MAX98357A met goedkope TRS-koptelefoon; risico bewust geaccepteerd</x:v>
+      </x:c>
+      <x:c r="D37" t="str">
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-075-HIL-SOFTWARE-PASS</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>
@@ -6104,7 +6166,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8039a29941a744ad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c9e9a3e26fd4e02"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(us055): connect USB MIDI D1 runtime to I2S output
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rba2e158f025a4348"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R1add1eddce294695"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Rcdd2e6360e1545b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R365eada3671c465b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R3227d4e4ff7d4b32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rd36d7f6ccf1147d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R9d292bd1b0d34ff6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R1dc3137240c74cd3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Rb25454baa12a4200"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R7e67d74462ca4c64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R8752afc1984a49e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R3c4441397e634794"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1095,7 +1095,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="102" t="str">
-        <x:v>Sprint 3 | scope v0.27.0 | runtime v0.16.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
+        <x:v>Sprint 3 | scope v0.28.0 | runtime v0.17.0 | CHATOD-20260714-MCP-CP-MVP-001</x:v>
       </x:c>
       <x:c r="B2" s="103"/>
       <x:c r="C2" s="103"/>
@@ -1156,7 +1156,7 @@
       </x:c>
       <x:c r="C6" s="85"/>
       <x:c r="D6" s="111" t="str">
-        <x:v>2. Direkte TRS-koptelefoon bly prototipe-risiko; US-076 parkeer cleanup</x:v>
+        <x:v>2. US-055 v0.17.0 hostgroen: USB-MIDI -&gt; D1 -&gt; veilige I2S</x:v>
       </x:c>
       <x:c r="E6" s="111"/>
       <x:c r="F6" s="111"/>
@@ -1165,14 +1165,14 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="111" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>In Review</x:v>
       </x:c>
       <x:c r="B7" s="114" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C7" s="85"/>
       <x:c r="D7" s="111" t="str">
-        <x:v>3. US-055: Logic USB-MIDI -&gt; D1-kern -&gt; I2S is volgende MVP-integrasie</x:v>
+        <x:v>3. Product Owner HIL: Logic External MIDI na S2 Mini moet D1 hoorbaar speel</x:v>
       </x:c>
       <x:c r="E7" s="111"/>
       <x:c r="F7" s="111"/>
@@ -1188,7 +1188,7 @@
       </x:c>
       <x:c r="C8" s="85"/>
       <x:c r="D8" s="112" t="str">
-        <x:v>4. US-057 volg na US-055 vir end-to-end MVP burn-in/acceptance</x:v>
+        <x:v>4. US-057 volg ná US-055 vir end-to-end MVP burn-in/acceptance</x:v>
       </x:c>
       <x:c r="E8" s="112"/>
       <x:c r="F8" s="112"/>
@@ -1247,7 +1247,7 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="119" t="str">
-        <x:v>120 tests GREEN | US-075 DONE WITH PO EXCEPTION | US-055 NEXT</x:v>
+        <x:v>125 tests GREEN | US-055 IN REVIEW | Logic HIL needed</x:v>
       </x:c>
       <x:c r="B13" s="120"/>
       <x:c r="C13" s="120"/>
@@ -1342,7 +1342,7 @@
     </x:row>
     <x:row r="2" ht="28" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Bron: docs/user_stories_v0.1.0.md v0.27.0 | 76 stories | 17-story veiligheidsaangepaste MVP Acceptance Set + US-076 post-MVP cleanup</x:v>
+        <x:v>Bron: docs/user_stories_v0.1.0.md v0.28.0 | 76 stories | US-055 In Review for Logic/HIL acceptance</x:v>
       </x:c>
       <x:c r="B2"/>
       <x:c r="C2"/>
@@ -3463,25 +3463,25 @@
         <x:v>Must</x:v>
       </x:c>
       <x:c r="F59" s="24" t="str">
-        <x:v>Backlog</x:v>
+        <x:v>In Review</x:v>
       </x:c>
       <x:c r="G59" s="24" t="str">
-        <x:v>Release train</x:v>
+        <x:v>Sprint 3</x:v>
       </x:c>
       <x:c r="H59" s="24" t="str">
-        <x:v>MVP-Must</x:v>
+        <x:v>MVP-Must (In Review)</x:v>
       </x:c>
       <x:c r="I59" s="65" t="n">
         <x:v>5</x:v>
       </x:c>
       <x:c r="J59" s="24" t="str">
-        <x:v>MCP-US-003, MCP-US-007, MCP-US-009, MCP-US-014, MCP-US-016, MCP-US-063, MCP-US-075</x:v>
+        <x:v>US-003, US-007, US-009, US-014, US-016, US-063, US-075</x:v>
       </x:c>
       <x:c r="K59" s="24" t="str">
-        <x:v>Logic selects the board as External MIDI destination and the user hears D1 through the approved safe output profile; the board then passes the 8-hour USB MIDI, audio and heap burn-in</x:v>
+        <x:v>v0.17.0 verbind USB-MIDI, D1 en veilige I2S; 125 hosttoetse slaag; wag op Logic/HIL hoorbaarheid</x:v>
       </x:c>
       <x:c r="L59" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-055</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-055-START / v0.17.0</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="38" customHeight="1">
@@ -4320,7 +4320,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3d845a9ed4da476b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4083a7b99b9745eb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4602,7 +4602,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6080077e0b2c4098"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51a3cad393ab4532"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5462,7 +5462,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba474dab399142ba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0a9fc3549ba4242"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5658,7 +5658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7052d15838a6460a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc4ed2ba3f8445c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6159,6 +6159,20 @@
         <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-075-HIL-SOFTWARE-PASS</x:v>
       </x:c>
     </x:row>
+    <x:row r="38">
+      <x:c r="A38" t="str">
+        <x:v>2026-07-16</x:v>
+      </x:c>
+      <x:c r="B38" t="str">
+        <x:v>US-055 host evidence</x:v>
+      </x:c>
+      <x:c r="C38" t="str">
+        <x:v>v0.17.0 adds D1UsbMidiI2sRuntime and CircuitPythonI2sAudioOutput; 125 pytest tests pass</x:v>
+      </x:c>
+      <x:c r="D38" t="str">
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-055-START</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>
@@ -6166,7 +6180,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c9e9a3e26fd4e02"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R593448a5ac64499e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix(us055): latch d1 i2s tone for Logic MIDI
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R9d292bd1b0d34ff6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R1dc3137240c74cd3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Rb25454baa12a4200"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R7e67d74462ca4c64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R8752afc1984a49e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R3c4441397e634794"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R9ae5bba51ed84711"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="Re3f1d5bdd4304b41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Rf4dbab0441ac4e79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R419d1a0708ab49f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R09db2ff8927f4a63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R3b86a5b9b7b34a03"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1156,7 +1156,7 @@
       </x:c>
       <x:c r="C6" s="85"/>
       <x:c r="D6" s="111" t="str">
-        <x:v>2. US-055 v0.17.0 hostgroen: USB-MIDI -&gt; D1 -&gt; veilige I2S</x:v>
+        <x:v>2. US-055 v0.17.5 hostgroen: USB-MIDI -&gt; D1 -&gt; latched I2S tone</x:v>
       </x:c>
       <x:c r="E6" s="111"/>
       <x:c r="F6" s="111"/>
@@ -1247,7 +1247,7 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="119" t="str">
-        <x:v>125 tests GREEN | US-055 IN REVIEW | Logic HIL needed</x:v>
+        <x:v>131 tests GREEN | US-055 IN REVIEW | v0.17.5 Logic HIL retest needed</x:v>
       </x:c>
       <x:c r="B13" s="120"/>
       <x:c r="C13" s="120"/>
@@ -3469,7 +3469,7 @@
         <x:v>Sprint 3</x:v>
       </x:c>
       <x:c r="H59" s="24" t="str">
-        <x:v>MVP-Must (In Review)</x:v>
+        <x:v>MVP-Must (HIL Retest Ready)</x:v>
       </x:c>
       <x:c r="I59" s="65" t="n">
         <x:v>5</x:v>
@@ -3478,10 +3478,10 @@
         <x:v>US-003, US-007, US-009, US-014, US-016, US-063, US-075</x:v>
       </x:c>
       <x:c r="K59" s="24" t="str">
-        <x:v>v0.17.0 verbind USB-MIDI, D1 en veilige I2S; 125 hosttoetse slaag; wag op Logic/HIL hoorbaarheid</x:v>
+        <x:v>v0.17.5 deploy op CIRCUITPY; 131 hosttoetse groen. HIL-rettoets: Logic/S2 Mini moet D1 hoorbaar speel; verwag D1_REALTIME_MIDI_NOTE en D1_AUDIO_EVENT=audible_note;mode=latched_tone.</x:v>
       </x:c>
       <x:c r="L59" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / MCP-US-055-START / v0.17.0</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / US-055-HIL-PASS-RECEIVED / v0.17.5</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="38" customHeight="1">
@@ -4320,7 +4320,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4083a7b99b9745eb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ba25b59b453431e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4602,7 +4602,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51a3cad393ab4532"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd805b39e6d21414c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5462,7 +5462,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0a9fc3549ba4242"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c5139a01c854787"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5658,7 +5658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc4ed2ba3f8445c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2d6bd237d4847ae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6180,7 +6180,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R593448a5ac64499e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0a5ebf671534622"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix(us055): fast boot d1 runtime for realtime MIDI
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R9ae5bba51ed84711"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="Re3f1d5bdd4304b41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Rf4dbab0441ac4e79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R419d1a0708ab49f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R09db2ff8927f4a63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R3b86a5b9b7b34a03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R41027af65d594d0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="Rff51f40a8cf840e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Ree33ebd26e324c6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R6be5b68eed9842e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R8338c234915b43bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rc9494a10f948405f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1156,7 +1156,7 @@
       </x:c>
       <x:c r="C6" s="85"/>
       <x:c r="D6" s="111" t="str">
-        <x:v>2. US-055 v0.17.5 hostgroen: USB-MIDI -&gt; D1 -&gt; latched I2S tone</x:v>
+        <x:v>2. US-055 v0.17.6 fast boot: USB-MIDI -&gt; D1 -&gt; latched I2S tone</x:v>
       </x:c>
       <x:c r="E6" s="111"/>
       <x:c r="F6" s="111"/>
@@ -1247,7 +1247,7 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="119" t="str">
-        <x:v>131 tests GREEN | US-055 IN REVIEW | v0.17.5 Logic HIL retest needed</x:v>
+        <x:v>132 tests GREEN | US-055 IN REVIEW | v0.17.6 realtime Logic HIL retest needed</x:v>
       </x:c>
       <x:c r="B13" s="120"/>
       <x:c r="C13" s="120"/>
@@ -3478,10 +3478,10 @@
         <x:v>US-003, US-007, US-009, US-014, US-016, US-063, US-075</x:v>
       </x:c>
       <x:c r="K59" s="24" t="str">
-        <x:v>v0.17.5 deploy op CIRCUITPY; 131 hosttoetse groen. HIL-rettoets: Logic/S2 Mini moet D1 hoorbaar speel; verwag D1_REALTIME_MIDI_NOTE en D1_AUDIO_EVENT=audible_note;mode=latched_tone.</x:v>
+        <x:v>v0.17.6 fast-boot deploy op CIRCUITPY; 132 hosttoetse groen. HIL-rettoets: speel pas ná D1_RUNTIME_READY; Logic/S2 Mini moet D1 realtime hoorbaar speel; verwag note_latency_ms.</x:v>
       </x:c>
       <x:c r="L59" s="24" t="str">
-        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / US-055-HIL-PASS-RECEIVED / v0.17.5</x:v>
+        <x:v>CHATOD-20260714-MCP-CP-MVP-001 / US-055-REALTIME-ANALYSE-001 / v0.17.6</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="38" customHeight="1">
@@ -4320,7 +4320,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ba25b59b453431e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c9927a3c63a413b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4602,7 +4602,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd805b39e6d21414c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R402b1302db1e4eee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5462,7 +5462,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c5139a01c854787"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26bf836d96834a93"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5658,7 +5658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2d6bd237d4847ae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00dc47859ebc44a1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6180,7 +6180,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0a5ebf671534622"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4be915534714aee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix(us055): reduce D1 latency logging for Logic
</commit_message>
<xml_diff>
--- a/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
+++ b/outputs/CHATOD-20260714-MCP-CP-MVP-001/circuitpython_midi_chip_platform_mvp_kanban_v0.1.0.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R41027af65d594d0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="Rff51f40a8cf840e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="Ree33ebd26e324c6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R6be5b68eed9842e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="R8338c234915b43bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rc9494a10f948405f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rb3a0ffb87ad84f8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="2" r:id="R8b6a2a2830604661"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="3" r:id="R0650809a46ad41d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="4" r:id="R2d90a9bb62ef4628"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team RACI" sheetId="5" r:id="Re28e9e2ee0e24612"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rbb29bb5e30254894"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4320,7 +4320,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c9927a3c63a413b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde6d5c5337664b30"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4602,7 +4602,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R402b1302db1e4eee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbb9774c360d473b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5462,7 +5462,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26bf836d96834a93"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b9c78680d954d09"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5658,7 +5658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00dc47859ebc44a1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c7b587bcc724745"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6180,7 +6180,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4be915534714aee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R140a8ba0ee024cf3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>